<commit_message>
Actualizacion automatica dashboard lun 21/09/2026  9:18:37,50
</commit_message>
<xml_diff>
--- a/Reporte_Efectividad_Automatizacion.xlsx
+++ b/Reporte_Efectividad_Automatizacion.xlsx
@@ -47,7 +47,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -55,24 +55,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -478,152 +466,152 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Total Retiros Enero</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Enero</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Proyectado Enero</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Total Retiros Febrero</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Febrero</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Proyectado Febrero</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Total Retiros Marzo</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Marzo</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Proyectado Marzo</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Total Retiros Abril</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Abril</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Proyectado Abril</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Total Retiros Mayo</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Mayo</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Proyectado Mayo</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Total Retiros Junio</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Junio</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Proyectado Junio</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Total Retiros Julio</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Julio</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Proyectado Julio</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Total Retiros Agosto</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Agosto</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Proyectado Agosto</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Total Retiros Septiembre</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Septiembre</t>
         </is>
       </c>
-      <c r="AB1" s="2" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>% Automatización Proyectado Septiembre</t>
         </is>
       </c>
-      <c r="AC1" s="2" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Variación Tasa Auto (Septiembre vs Agosto)</t>
         </is>
       </c>
-      <c r="AD1" s="2" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Crecimiento Volumen MoM % (Septiembre vs Agosto)</t>
         </is>
@@ -708,19 +696,19 @@
         <v>71.65194435983349</v>
       </c>
       <c r="Z2" t="n">
-        <v>1280</v>
+        <v>2969</v>
       </c>
       <c r="AA2" t="n">
-        <v>36.25</v>
+        <v>35.63489390367127</v>
       </c>
       <c r="AB2" t="n">
-        <v>69.765625</v>
+        <v>69.51835634893904</v>
       </c>
       <c r="AC2" t="n">
-        <v>10.55195958980607</v>
+        <v>9.93685349347734</v>
       </c>
       <c r="AD2" t="n">
-        <v>-87.00375672657123</v>
+        <v>-69.85480759467966</v>
       </c>
     </row>
     <row r="3">
@@ -802,19 +790,19 @@
         <v>79.51807228915662</v>
       </c>
       <c r="Z3" t="n">
-        <v>98</v>
+        <v>231</v>
       </c>
       <c r="AA3" t="n">
-        <v>50</v>
+        <v>38.09523809523809</v>
       </c>
       <c r="AB3" t="n">
-        <v>91.83673469387756</v>
+        <v>80.08658008658008</v>
       </c>
       <c r="AC3" t="n">
-        <v>24.18244406196213</v>
+        <v>12.27768215720023</v>
       </c>
       <c r="AD3" t="n">
-        <v>-83.13253012048193</v>
+        <v>-60.24096385542169</v>
       </c>
     </row>
     <row r="4">
@@ -896,19 +884,19 @@
         <v>62.42171189979123</v>
       </c>
       <c r="Z4" t="n">
-        <v>18</v>
+        <v>103</v>
       </c>
       <c r="AA4" t="n">
-        <v>72.22222222222221</v>
+        <v>69.90291262135922</v>
       </c>
       <c r="AB4" t="n">
-        <v>88.88888888888889</v>
+        <v>75.72815533980582</v>
       </c>
       <c r="AC4" t="n">
-        <v>53.64184643934121</v>
+        <v>51.32253683847821</v>
       </c>
       <c r="AD4" t="n">
-        <v>-96.24217118997912</v>
+        <v>-78.49686847599166</v>
       </c>
     </row>
     <row r="5">
@@ -990,19 +978,19 @@
         <v>62.37424547283702</v>
       </c>
       <c r="Z5" t="n">
-        <v>286</v>
+        <v>561</v>
       </c>
       <c r="AA5" t="n">
-        <v>54.54545454545454</v>
+        <v>55.43672014260249</v>
       </c>
       <c r="AB5" t="n">
-        <v>59.09090909090909</v>
+        <v>59.18003565062389</v>
       </c>
       <c r="AC5" t="n">
-        <v>-1.188951893177247</v>
+        <v>-0.2976862960292976</v>
       </c>
       <c r="AD5" t="n">
-        <v>-85.61368209255534</v>
+        <v>-71.78068410462777</v>
       </c>
     </row>
     <row r="6">
@@ -1084,19 +1072,19 @@
         <v>82.54543623823189</v>
       </c>
       <c r="Z6" t="n">
-        <v>3125</v>
+        <v>6703</v>
       </c>
       <c r="AA6" t="n">
-        <v>58.11199999999999</v>
+        <v>66.2091600775772</v>
       </c>
       <c r="AB6" t="n">
-        <v>64.096</v>
+        <v>71.05773534238401</v>
       </c>
       <c r="AC6" t="n">
-        <v>-20.95460625283189</v>
+        <v>-12.85744617525469</v>
       </c>
       <c r="AD6" t="n">
-        <v>-84.2672305291245</v>
+        <v>-66.25383879575089</v>
       </c>
     </row>
     <row r="7">
@@ -1178,19 +1166,19 @@
         <v>64.37949170915806</v>
       </c>
       <c r="Z7" t="n">
-        <v>3808</v>
+        <v>8906</v>
       </c>
       <c r="AA7" t="n">
-        <v>54.51680672268907</v>
+        <v>52.64989894453178</v>
       </c>
       <c r="AB7" t="n">
-        <v>65.30987394957984</v>
+        <v>65.19200538962497</v>
       </c>
       <c r="AC7" t="n">
-        <v>10.01927590805865</v>
+        <v>8.152368129901362</v>
       </c>
       <c r="AD7" t="n">
-        <v>-84.71112538643754</v>
+        <v>-64.24298390010841</v>
       </c>
     </row>
     <row r="8">
@@ -1272,19 +1260,19 @@
         <v>63.24499030381383</v>
       </c>
       <c r="Z8" t="n">
-        <v>1660</v>
+        <v>3738</v>
       </c>
       <c r="AA8" t="n">
-        <v>50.96385542168674</v>
+        <v>50.42803638309257</v>
       </c>
       <c r="AB8" t="n">
-        <v>60.12048192771084</v>
+        <v>59.06902086677368</v>
       </c>
       <c r="AC8" t="n">
-        <v>1.55209071580439</v>
+        <v>1.016271677210213</v>
       </c>
       <c r="AD8" t="n">
-        <v>-78.53910795087266</v>
+        <v>-51.67420814479639</v>
       </c>
     </row>
     <row r="9">
@@ -1366,19 +1354,19 @@
         <v>78.380257212374</v>
       </c>
       <c r="Z9" t="n">
-        <v>309</v>
+        <v>864</v>
       </c>
       <c r="AA9" t="n">
-        <v>42.39482200647249</v>
+        <v>51.04166666666666</v>
       </c>
       <c r="AB9" t="n">
-        <v>57.28155339805825</v>
+        <v>59.02777777777778</v>
       </c>
       <c r="AC9" t="n">
-        <v>-30.49360343669747</v>
+        <v>-21.8467587765033</v>
       </c>
       <c r="AD9" t="n">
-        <v>-89.25964546402503</v>
+        <v>-69.9687174139729</v>
       </c>
     </row>
     <row r="10">
@@ -1460,19 +1448,19 @@
         <v>54.65631929046562</v>
       </c>
       <c r="Z10" t="n">
-        <v>433</v>
+        <v>1127</v>
       </c>
       <c r="AA10" t="n">
-        <v>51.73210161662818</v>
+        <v>49.15705412599822</v>
       </c>
       <c r="AB10" t="n">
-        <v>57.27482678983834</v>
+        <v>56.61047027506655</v>
       </c>
       <c r="AC10" t="n">
-        <v>18.25094862328006</v>
+        <v>15.6759011326501</v>
       </c>
       <c r="AD10" t="n">
-        <v>-83.99852180339985</v>
+        <v>-58.35181079083518</v>
       </c>
     </row>
     <row r="11">
@@ -1554,19 +1542,19 @@
         <v>81.92520288611654</v>
       </c>
       <c r="Z11" t="n">
-        <v>9221</v>
+        <v>25964</v>
       </c>
       <c r="AA11" t="n">
-        <v>76.90055308534866</v>
+        <v>76.21706978893853</v>
       </c>
       <c r="AB11" t="n">
-        <v>80.34920290640927</v>
+        <v>79.19812047450316</v>
       </c>
       <c r="AC11" t="n">
-        <v>-1.509832433435008</v>
+        <v>-2.193315729845139</v>
       </c>
       <c r="AD11" t="n">
-        <v>-87.03075992629995</v>
+        <v>-63.48190551203252</v>
       </c>
     </row>
     <row r="12">
@@ -1648,19 +1636,19 @@
         <v>79.3433378990412</v>
       </c>
       <c r="Z12" t="n">
-        <v>24739</v>
+        <v>66728</v>
       </c>
       <c r="AA12" t="n">
-        <v>65.6453373216379</v>
+        <v>62.42057307277305</v>
       </c>
       <c r="AB12" t="n">
-        <v>79.80920813290754</v>
+        <v>77.83988730368061</v>
       </c>
       <c r="AC12" t="n">
-        <v>3.370914950335866</v>
+        <v>0.1461507014710151</v>
       </c>
       <c r="AD12" t="n">
-        <v>-87.63309704961958</v>
+        <v>-66.64300496895652</v>
       </c>
     </row>
     <row r="13">
@@ -1742,19 +1730,19 @@
         <v>67.14883504675311</v>
       </c>
       <c r="Z13" t="n">
-        <v>5816</v>
+        <v>10918</v>
       </c>
       <c r="AA13" t="n">
-        <v>46.56121045392022</v>
+        <v>46.54698662758747</v>
       </c>
       <c r="AB13" t="n">
-        <v>66.23108665749656</v>
+        <v>65.90950723575747</v>
       </c>
       <c r="AC13" t="n">
-        <v>3.698163494164056</v>
+        <v>3.683939667831311</v>
       </c>
       <c r="AD13" t="n">
-        <v>-84.97701090044944</v>
+        <v>-71.79831585472955</v>
       </c>
     </row>
     <row r="14">
@@ -1836,19 +1824,19 @@
         <v>72.04349796103308</v>
       </c>
       <c r="Z14" t="n">
-        <v>432</v>
+        <v>731</v>
       </c>
       <c r="AA14" t="n">
-        <v>53.00925925925925</v>
+        <v>56.0875512995896</v>
       </c>
       <c r="AB14" t="n">
-        <v>73.14814814814815</v>
+        <v>72.64021887824897</v>
       </c>
       <c r="AC14" t="n">
-        <v>4.277949789390654</v>
+        <v>7.356241829721</v>
       </c>
       <c r="AD14" t="n">
-        <v>-90.21295876755777</v>
+        <v>-83.43905754417762</v>
       </c>
     </row>
     <row r="15">
@@ -1930,19 +1918,19 @@
         <v>78.43225419664267</v>
       </c>
       <c r="Z15" t="n">
-        <v>1522</v>
+        <v>3373</v>
       </c>
       <c r="AA15" t="n">
-        <v>67.47700394218134</v>
+        <v>68.98903053661429</v>
       </c>
       <c r="AB15" t="n">
-        <v>73.25886990801577</v>
+        <v>74.8295286095464</v>
       </c>
       <c r="AC15" t="n">
-        <v>-2.254710686116013</v>
+        <v>-0.7426840916830599</v>
       </c>
       <c r="AD15" t="n">
-        <v>-88.5941247002398</v>
+        <v>-74.72272182254197</v>
       </c>
     </row>
   </sheetData>
@@ -1985,45 +1973,45 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos Proyectados</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion Proyectado</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2343,77 +2331,77 @@
     </row>
     <row r="20"/>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Tipo Aprobacion</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Hrs)</t>
         </is>
@@ -3810,47 +3798,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Métricas por Nivel de Riesgo - Septiembre 2026</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Nivel De Riesgo</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Valor Promedio Automatico</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Valor Promedio Manual</t>
         </is>
@@ -3863,19 +3851,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>890</v>
+        <v>2690</v>
       </c>
       <c r="C4" t="n">
-        <v>84</v>
+        <v>339</v>
       </c>
       <c r="D4" t="n">
-        <v>9.438202247191011</v>
+        <v>12.60223048327138</v>
       </c>
       <c r="E4" t="n">
-        <v>882.4149999999998</v>
+        <v>1597.919646017699</v>
       </c>
       <c r="F4" t="n">
-        <v>3131.372717121588</v>
+        <v>1918.06940450872</v>
       </c>
     </row>
     <row r="5">
@@ -3885,19 +3873,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>37249</v>
+        <v>92740</v>
       </c>
       <c r="C5" t="n">
-        <v>30802</v>
+        <v>76197</v>
       </c>
       <c r="D5" t="n">
-        <v>82.69215280947139</v>
+        <v>82.16195816260513</v>
       </c>
       <c r="E5" t="n">
-        <v>3707.349971722616</v>
+        <v>3535.304440253553</v>
       </c>
       <c r="F5" t="n">
-        <v>11534.20088242593</v>
+        <v>8884.176789518226</v>
       </c>
     </row>
     <row r="6">
@@ -3907,19 +3895,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12226</v>
+        <v>30169</v>
       </c>
       <c r="C6" t="n">
-        <v>1349</v>
+        <v>3737</v>
       </c>
       <c r="D6" t="n">
-        <v>11.03386226075577</v>
+        <v>12.38688720209487</v>
       </c>
       <c r="E6" t="n">
-        <v>10517.2290437361</v>
+        <v>10332.67597805727</v>
       </c>
       <c r="F6" t="n">
-        <v>6244.661888388342</v>
+        <v>4782.103336107748</v>
       </c>
     </row>
     <row r="7">
@@ -3929,64 +3917,64 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2382</v>
+        <v>7317</v>
       </c>
       <c r="C7" t="n">
-        <v>835</v>
+        <v>2523</v>
       </c>
       <c r="D7" t="n">
-        <v>35.05457598656591</v>
+        <v>34.48134481344813</v>
       </c>
       <c r="E7" t="n">
-        <v>1869.074892215569</v>
+        <v>1479.006062227507</v>
       </c>
       <c r="F7" t="n">
-        <v>4984.897601809954</v>
+        <v>5528.920880267</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Métricas por Nivel de Riesgo - Agosto 2026</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="1" t="n"/>
+      <c r="C10" s="1" t="n"/>
+      <c r="D10" s="1" t="n"/>
+      <c r="E10" s="1" t="n"/>
+      <c r="F10" s="1" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Nivel De Riesgo</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Valor Promedio Automatico</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Valor Promedio Manual</t>
         </is>
@@ -4082,47 +4070,47 @@
     </row>
     <row r="16"/>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Métricas por Nivel de Riesgo - Julio 2026</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n"/>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n"/>
+      <c r="A18" s="1" t="n"/>
+      <c r="B18" s="1" t="n"/>
+      <c r="C18" s="1" t="n"/>
+      <c r="D18" s="1" t="n"/>
+      <c r="E18" s="1" t="n"/>
+      <c r="F18" s="1" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Nivel De Riesgo</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Valor Promedio Automatico</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Valor Promedio Manual</t>
         </is>
@@ -4218,47 +4206,47 @@
     </row>
     <row r="24"/>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Métricas por Nivel de Riesgo - Junio 2026</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n"/>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
+      <c r="A26" s="1" t="n"/>
+      <c r="B26" s="1" t="n"/>
+      <c r="C26" s="1" t="n"/>
+      <c r="D26" s="1" t="n"/>
+      <c r="E26" s="1" t="n"/>
+      <c r="F26" s="1" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Nivel De Riesgo</t>
         </is>
       </c>
-      <c r="B27" s="1" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>Valor Promedio Automatico</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Valor Promedio Manual</t>
         </is>
@@ -4354,47 +4342,47 @@
     </row>
     <row r="32"/>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Métricas por Nivel de Riesgo - Mayo 2026</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n"/>
-      <c r="B34" s="3" t="n"/>
-      <c r="C34" s="3" t="n"/>
-      <c r="D34" s="3" t="n"/>
-      <c r="E34" s="3" t="n"/>
-      <c r="F34" s="3" t="n"/>
+      <c r="A34" s="1" t="n"/>
+      <c r="B34" s="1" t="n"/>
+      <c r="C34" s="1" t="n"/>
+      <c r="D34" s="1" t="n"/>
+      <c r="E34" s="1" t="n"/>
+      <c r="F34" s="1" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Nivel De Riesgo</t>
         </is>
       </c>
-      <c r="B35" s="1" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C35" s="1" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D35" s="1" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E35" s="1" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Valor Promedio Automatico</t>
         </is>
       </c>
-      <c r="F35" s="1" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Valor Promedio Manual</t>
         </is>
@@ -4490,47 +4478,47 @@
     </row>
     <row r="40"/>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Métricas por Nivel de Riesgo - Abril 2026</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="n"/>
-      <c r="B42" s="3" t="n"/>
-      <c r="C42" s="3" t="n"/>
-      <c r="D42" s="3" t="n"/>
-      <c r="E42" s="3" t="n"/>
-      <c r="F42" s="3" t="n"/>
+      <c r="A42" s="1" t="n"/>
+      <c r="B42" s="1" t="n"/>
+      <c r="C42" s="1" t="n"/>
+      <c r="D42" s="1" t="n"/>
+      <c r="E42" s="1" t="n"/>
+      <c r="F42" s="1" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Nivel De Riesgo</t>
         </is>
       </c>
-      <c r="B43" s="1" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C43" s="1" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D43" s="1" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E43" s="1" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>Valor Promedio Automatico</t>
         </is>
       </c>
-      <c r="F43" s="1" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>Valor Promedio Manual</t>
         </is>
@@ -4626,47 +4614,47 @@
     </row>
     <row r="48"/>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>Métricas por Nivel de Riesgo - Marzo 2026</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="n"/>
-      <c r="B50" s="3" t="n"/>
-      <c r="C50" s="3" t="n"/>
-      <c r="D50" s="3" t="n"/>
-      <c r="E50" s="3" t="n"/>
-      <c r="F50" s="3" t="n"/>
+      <c r="A50" s="1" t="n"/>
+      <c r="B50" s="1" t="n"/>
+      <c r="C50" s="1" t="n"/>
+      <c r="D50" s="1" t="n"/>
+      <c r="E50" s="1" t="n"/>
+      <c r="F50" s="1" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>Nivel De Riesgo</t>
         </is>
       </c>
-      <c r="B51" s="1" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C51" s="1" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D51" s="1" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E51" s="1" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>Valor Promedio Automatico</t>
         </is>
       </c>
-      <c r="F51" s="1" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>Valor Promedio Manual</t>
         </is>
@@ -4762,47 +4750,47 @@
     </row>
     <row r="56"/>
     <row r="57">
-      <c r="A57" s="4" t="inlineStr">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>Métricas por Nivel de Riesgo - Febrero 2026</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="n"/>
-      <c r="B58" s="3" t="n"/>
-      <c r="C58" s="3" t="n"/>
-      <c r="D58" s="3" t="n"/>
-      <c r="E58" s="3" t="n"/>
-      <c r="F58" s="3" t="n"/>
+      <c r="A58" s="1" t="n"/>
+      <c r="B58" s="1" t="n"/>
+      <c r="C58" s="1" t="n"/>
+      <c r="D58" s="1" t="n"/>
+      <c r="E58" s="1" t="n"/>
+      <c r="F58" s="1" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="inlineStr">
+      <c r="A59" t="inlineStr">
         <is>
           <t>Nivel De Riesgo</t>
         </is>
       </c>
-      <c r="B59" s="1" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C59" s="1" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D59" s="1" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E59" s="1" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>Valor Promedio Automatico</t>
         </is>
       </c>
-      <c r="F59" s="1" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>Valor Promedio Manual</t>
         </is>
@@ -4898,47 +4886,47 @@
     </row>
     <row r="64"/>
     <row r="65">
-      <c r="A65" s="4" t="inlineStr">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>Métricas por Nivel de Riesgo - Enero 2026</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="n"/>
-      <c r="B66" s="3" t="n"/>
-      <c r="C66" s="3" t="n"/>
-      <c r="D66" s="3" t="n"/>
-      <c r="E66" s="3" t="n"/>
-      <c r="F66" s="3" t="n"/>
+      <c r="A66" s="1" t="n"/>
+      <c r="B66" s="1" t="n"/>
+      <c r="C66" s="1" t="n"/>
+      <c r="D66" s="1" t="n"/>
+      <c r="E66" s="1" t="n"/>
+      <c r="F66" s="1" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="inlineStr">
+      <c r="A67" t="inlineStr">
         <is>
           <t>Nivel De Riesgo</t>
         </is>
       </c>
-      <c r="B67" s="1" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C67" s="1" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D67" s="1" t="inlineStr">
+      <c r="D67" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E67" s="1" t="inlineStr">
+      <c r="E67" t="inlineStr">
         <is>
           <t>Valor Promedio Automatico</t>
         </is>
       </c>
-      <c r="F67" s="1" t="inlineStr">
+      <c r="F67" t="inlineStr">
         <is>
           <t>Valor Promedio Manual</t>
         </is>
@@ -5072,45 +5060,45 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos Proyectados</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion Proyectado</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5119,19 +5107,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1280</v>
+        <v>2969</v>
       </c>
       <c r="C4" t="n">
-        <v>464</v>
+        <v>1058</v>
       </c>
       <c r="D4" t="n">
-        <v>36.25</v>
+        <v>35.63489390367127</v>
       </c>
       <c r="E4" t="n">
-        <v>893</v>
+        <v>2064</v>
       </c>
       <c r="F4" t="n">
-        <v>69.765625</v>
+        <v>69.51835634893904</v>
       </c>
     </row>
     <row r="5">
@@ -5141,19 +5129,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>98</v>
+        <v>231</v>
       </c>
       <c r="C5" t="n">
-        <v>49</v>
+        <v>88</v>
       </c>
       <c r="D5" t="n">
-        <v>50</v>
+        <v>38.09523809523809</v>
       </c>
       <c r="E5" t="n">
-        <v>90</v>
+        <v>185</v>
       </c>
       <c r="F5" t="n">
-        <v>91.83673469387756</v>
+        <v>80.08658008658008</v>
       </c>
     </row>
     <row r="6">
@@ -5163,19 +5151,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18</v>
+        <v>103</v>
       </c>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>72</v>
       </c>
       <c r="D6" t="n">
-        <v>72.22222222222221</v>
+        <v>69.90291262135922</v>
       </c>
       <c r="E6" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="F6" t="n">
-        <v>88.88888888888889</v>
+        <v>75.72815533980582</v>
       </c>
     </row>
     <row r="7">
@@ -5185,19 +5173,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>286</v>
+        <v>561</v>
       </c>
       <c r="C7" t="n">
-        <v>156</v>
+        <v>311</v>
       </c>
       <c r="D7" t="n">
-        <v>54.54545454545454</v>
+        <v>55.43672014260249</v>
       </c>
       <c r="E7" t="n">
-        <v>169</v>
+        <v>332</v>
       </c>
       <c r="F7" t="n">
-        <v>59.09090909090909</v>
+        <v>59.18003565062389</v>
       </c>
     </row>
     <row r="8">
@@ -5207,19 +5195,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3125</v>
+        <v>6703</v>
       </c>
       <c r="C8" t="n">
-        <v>1816</v>
+        <v>4438</v>
       </c>
       <c r="D8" t="n">
-        <v>58.11199999999999</v>
+        <v>66.2091600775772</v>
       </c>
       <c r="E8" t="n">
-        <v>2003</v>
+        <v>4763</v>
       </c>
       <c r="F8" t="n">
-        <v>64.096</v>
+        <v>71.05773534238401</v>
       </c>
     </row>
     <row r="9">
@@ -5229,19 +5217,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3808</v>
+        <v>8906</v>
       </c>
       <c r="C9" t="n">
-        <v>2076</v>
+        <v>4689</v>
       </c>
       <c r="D9" t="n">
-        <v>54.51680672268907</v>
+        <v>52.64989894453178</v>
       </c>
       <c r="E9" t="n">
-        <v>2487</v>
+        <v>5806</v>
       </c>
       <c r="F9" t="n">
-        <v>65.30987394957984</v>
+        <v>65.19200538962497</v>
       </c>
     </row>
     <row r="10">
@@ -5251,19 +5239,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1660</v>
+        <v>3738</v>
       </c>
       <c r="C10" t="n">
-        <v>846</v>
+        <v>1885</v>
       </c>
       <c r="D10" t="n">
-        <v>50.96385542168674</v>
+        <v>50.42803638309257</v>
       </c>
       <c r="E10" t="n">
-        <v>998</v>
+        <v>2208</v>
       </c>
       <c r="F10" t="n">
-        <v>60.12048192771084</v>
+        <v>59.06902086677368</v>
       </c>
     </row>
     <row r="11">
@@ -5273,19 +5261,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>309</v>
+        <v>864</v>
       </c>
       <c r="C11" t="n">
-        <v>131</v>
+        <v>441</v>
       </c>
       <c r="D11" t="n">
-        <v>42.39482200647249</v>
+        <v>51.04166666666666</v>
       </c>
       <c r="E11" t="n">
-        <v>177</v>
+        <v>510</v>
       </c>
       <c r="F11" t="n">
-        <v>57.28155339805825</v>
+        <v>59.02777777777778</v>
       </c>
     </row>
     <row r="12">
@@ -5295,19 +5283,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>433</v>
+        <v>1127</v>
       </c>
       <c r="C12" t="n">
-        <v>224</v>
+        <v>554</v>
       </c>
       <c r="D12" t="n">
-        <v>51.73210161662818</v>
+        <v>49.15705412599822</v>
       </c>
       <c r="E12" t="n">
-        <v>248</v>
+        <v>638</v>
       </c>
       <c r="F12" t="n">
-        <v>57.27482678983834</v>
+        <v>56.61047027506655</v>
       </c>
     </row>
     <row r="13">
@@ -5317,19 +5305,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>9221</v>
+        <v>25964</v>
       </c>
       <c r="C13" t="n">
-        <v>7091</v>
+        <v>19789</v>
       </c>
       <c r="D13" t="n">
-        <v>76.90055308534866</v>
+        <v>76.21706978893853</v>
       </c>
       <c r="E13" t="n">
-        <v>7409</v>
+        <v>20563</v>
       </c>
       <c r="F13" t="n">
-        <v>80.34920290640927</v>
+        <v>79.19812047450316</v>
       </c>
     </row>
     <row r="14">
@@ -5339,19 +5327,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>24739</v>
+        <v>66728</v>
       </c>
       <c r="C14" t="n">
-        <v>16240</v>
+        <v>41652</v>
       </c>
       <c r="D14" t="n">
-        <v>65.6453373216379</v>
+        <v>62.42057307277305</v>
       </c>
       <c r="E14" t="n">
-        <v>19744</v>
+        <v>51941</v>
       </c>
       <c r="F14" t="n">
-        <v>79.80920813290754</v>
+        <v>77.83988730368061</v>
       </c>
     </row>
     <row r="15">
@@ -5361,19 +5349,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5816</v>
+        <v>10918</v>
       </c>
       <c r="C15" t="n">
-        <v>2708</v>
+        <v>5082</v>
       </c>
       <c r="D15" t="n">
-        <v>46.56121045392022</v>
+        <v>46.54698662758747</v>
       </c>
       <c r="E15" t="n">
-        <v>3852</v>
+        <v>7196</v>
       </c>
       <c r="F15" t="n">
-        <v>66.23108665749656</v>
+        <v>65.90950723575747</v>
       </c>
     </row>
     <row r="16">
@@ -5383,19 +5371,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>432</v>
+        <v>731</v>
       </c>
       <c r="C16" t="n">
-        <v>229</v>
+        <v>410</v>
       </c>
       <c r="D16" t="n">
-        <v>53.00925925925925</v>
+        <v>56.0875512995896</v>
       </c>
       <c r="E16" t="n">
-        <v>316</v>
+        <v>531</v>
       </c>
       <c r="F16" t="n">
-        <v>73.14814814814815</v>
+        <v>72.64021887824897</v>
       </c>
     </row>
     <row r="17">
@@ -5405,19 +5393,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1522</v>
+        <v>3373</v>
       </c>
       <c r="C17" t="n">
-        <v>1027</v>
+        <v>2327</v>
       </c>
       <c r="D17" t="n">
-        <v>67.47700394218134</v>
+        <v>68.98903053661429</v>
       </c>
       <c r="E17" t="n">
-        <v>1115</v>
+        <v>2524</v>
       </c>
       <c r="F17" t="n">
-        <v>73.25886990801577</v>
+        <v>74.8295286095464</v>
       </c>
     </row>
     <row r="18"/>
@@ -5430,77 +5418,77 @@
     </row>
     <row r="20"/>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Tipo Aprobacion</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Hrs)</t>
         </is>
@@ -5518,43 +5506,43 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>464</v>
+        <v>1058</v>
       </c>
       <c r="D22" t="n">
-        <v>2.283081896551724</v>
+        <v>5.055718336483932</v>
       </c>
       <c r="E22" t="n">
-        <v>2.566666666666667</v>
+        <v>2.033333333333333</v>
       </c>
       <c r="F22" t="n">
-        <v>0.03805136494252874</v>
+        <v>0.0842619722747322</v>
       </c>
       <c r="G22" t="n">
-        <v>0.04277777777777778</v>
+        <v>0.03388888888888889</v>
       </c>
       <c r="H22" t="n">
-        <v>213.1201265822785</v>
+        <v>195.410458240946</v>
       </c>
       <c r="I22" t="n">
-        <v>87.28333333333333</v>
+        <v>73.35833333333332</v>
       </c>
       <c r="J22" t="n">
-        <v>3.552002109704642</v>
+        <v>3.256840970682434</v>
       </c>
       <c r="K22" t="n">
-        <v>1.454722222222222</v>
+        <v>1.222638888888889</v>
       </c>
       <c r="L22" t="n">
-        <v>210.5104219409283</v>
+        <v>189.780155210643</v>
       </c>
       <c r="M22" t="n">
-        <v>85.13333333333334</v>
+        <v>67.46666666666667</v>
       </c>
       <c r="N22" t="n">
-        <v>3.508507032348805</v>
+        <v>3.163002586844051</v>
       </c>
       <c r="O22" t="n">
-        <v>1.418888888888889</v>
+        <v>1.124444444444444</v>
       </c>
     </row>
     <row r="23">
@@ -5569,43 +5557,43 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>816</v>
+        <v>1911</v>
       </c>
       <c r="D23" t="n">
-        <v>238.7686887254902</v>
+        <v>249.7237571951858</v>
       </c>
       <c r="E23" t="n">
-        <v>70.19999999999999</v>
+        <v>69.33333333333333</v>
       </c>
       <c r="F23" t="n">
-        <v>3.979478145424837</v>
+        <v>4.162062619919763</v>
       </c>
       <c r="G23" t="n">
-        <v>1.17</v>
+        <v>1.155555555555555</v>
       </c>
       <c r="H23" t="n">
-        <v>275.6725563909774</v>
+        <v>275.095775770457</v>
       </c>
       <c r="I23" t="n">
-        <v>106.0166666666667</v>
+        <v>97.65833333333333</v>
       </c>
       <c r="J23" t="n">
-        <v>4.59454260651629</v>
+        <v>4.584929596174282</v>
       </c>
       <c r="K23" t="n">
-        <v>1.766944444444444</v>
+        <v>1.627638888888889</v>
       </c>
       <c r="L23" t="n">
-        <v>32.26791979949875</v>
+        <v>22.97846262840949</v>
       </c>
       <c r="M23" t="n">
-        <v>7.441666666666666</v>
+        <v>8.683333333333334</v>
       </c>
       <c r="N23" t="n">
-        <v>0.5377986633249792</v>
+        <v>0.3829743771401583</v>
       </c>
       <c r="O23" t="n">
-        <v>0.1240277777777778</v>
+        <v>0.1447222222222222</v>
       </c>
     </row>
     <row r="24">
@@ -5620,43 +5608,43 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>49</v>
+        <v>88</v>
       </c>
       <c r="D24" t="n">
-        <v>2.169047619047619</v>
+        <v>4.358522727272727</v>
       </c>
       <c r="E24" t="n">
-        <v>2.533333333333333</v>
+        <v>2.283333333333333</v>
       </c>
       <c r="F24" t="n">
-        <v>0.03615079365079365</v>
+        <v>0.07264204545454546</v>
       </c>
       <c r="G24" t="n">
-        <v>0.04222222222222222</v>
+        <v>0.03805555555555555</v>
       </c>
       <c r="H24" t="n">
-        <v>267.8308823529412</v>
+        <v>233.2459770114943</v>
       </c>
       <c r="I24" t="n">
-        <v>16.55</v>
+        <v>13.425</v>
       </c>
       <c r="J24" t="n">
-        <v>4.463848039215685</v>
+        <v>3.887432950191571</v>
       </c>
       <c r="K24" t="n">
-        <v>0.2758333333333334</v>
+        <v>0.22375</v>
       </c>
       <c r="L24" t="n">
-        <v>265.1759803921569</v>
+        <v>227.6</v>
       </c>
       <c r="M24" t="n">
-        <v>14.025</v>
+        <v>10.575</v>
       </c>
       <c r="N24" t="n">
-        <v>4.419599673202614</v>
+        <v>3.793333333333333</v>
       </c>
       <c r="O24" t="n">
-        <v>0.23375</v>
+        <v>0.17625</v>
       </c>
     </row>
     <row r="25">
@@ -5671,43 +5659,43 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>49</v>
+        <v>143</v>
       </c>
       <c r="D25" t="n">
-        <v>396.5632653061224</v>
+        <v>325.7984848484849</v>
       </c>
       <c r="E25" t="n">
-        <v>58.2</v>
+        <v>19.63333333333333</v>
       </c>
       <c r="F25" t="n">
-        <v>6.609387755102041</v>
+        <v>5.429974747474748</v>
       </c>
       <c r="G25" t="n">
-        <v>0.9700000000000001</v>
+        <v>0.3272222222222222</v>
       </c>
       <c r="H25" t="n">
-        <v>389.8354166666667</v>
+        <v>329.7687793427231</v>
       </c>
       <c r="I25" t="n">
-        <v>56.73333333333333</v>
+        <v>27.78333333333333</v>
       </c>
       <c r="J25" t="n">
-        <v>6.497256944444444</v>
+        <v>5.496146322378717</v>
       </c>
       <c r="K25" t="n">
-        <v>0.9455555555555555</v>
+        <v>0.4630555555555556</v>
       </c>
       <c r="L25" t="n">
-        <v>10.92847222222222</v>
+        <v>10.43697183098591</v>
       </c>
       <c r="M25" t="n">
-        <v>1.691666666666667</v>
+        <v>2.058333333333334</v>
       </c>
       <c r="N25" t="n">
-        <v>0.1821412037037037</v>
+        <v>0.1739495305164319</v>
       </c>
       <c r="O25" t="n">
-        <v>0.02819444444444445</v>
+        <v>0.03430555555555555</v>
       </c>
     </row>
     <row r="26">
@@ -5722,43 +5710,43 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>13</v>
+        <v>72</v>
       </c>
       <c r="D26" t="n">
-        <v>0.776923076923077</v>
+        <v>5.28587962962963</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>1.558333333333333</v>
       </c>
       <c r="F26" t="n">
-        <v>0.01294871794871795</v>
+        <v>0.08809799382716049</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>0.02597222222222222</v>
       </c>
       <c r="H26" t="n">
-        <v>1514.916666666667</v>
+        <v>2062.413945578232</v>
       </c>
       <c r="I26" t="n">
-        <v>1539.35</v>
+        <v>1904.233333333333</v>
       </c>
       <c r="J26" t="n">
-        <v>25.24861111111111</v>
+        <v>34.37356575963719</v>
       </c>
       <c r="K26" t="n">
-        <v>25.65583333333333</v>
+        <v>31.73722222222222</v>
       </c>
       <c r="L26" t="n">
-        <v>1512.391666666667</v>
+        <v>2054.681632653061</v>
       </c>
       <c r="M26" t="n">
-        <v>1536.9</v>
+        <v>1851.366666666667</v>
       </c>
       <c r="N26" t="n">
-        <v>25.20652777777778</v>
+        <v>34.24469387755102</v>
       </c>
       <c r="O26" t="n">
-        <v>25.615</v>
+        <v>30.85611111111111</v>
       </c>
     </row>
     <row r="27">
@@ -5773,43 +5761,43 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="D27" t="n">
-        <v>531.3566666666667</v>
+        <v>361.5575268817204</v>
       </c>
       <c r="E27" t="n">
-        <v>294.6</v>
+        <v>205.6166666666667</v>
       </c>
       <c r="F27" t="n">
-        <v>8.855944444444443</v>
+        <v>6.025958781362008</v>
       </c>
       <c r="G27" t="n">
-        <v>4.91</v>
+        <v>3.426944444444445</v>
       </c>
       <c r="H27" t="n">
-        <v>2136.71</v>
+        <v>2259.420967741936</v>
       </c>
       <c r="I27" t="n">
-        <v>1899.9</v>
+        <v>2348.833333333333</v>
       </c>
       <c r="J27" t="n">
-        <v>35.61183333333334</v>
+        <v>37.65701612903226</v>
       </c>
       <c r="K27" t="n">
-        <v>31.665</v>
+        <v>39.14722222222223</v>
       </c>
       <c r="L27" t="n">
-        <v>1605.353333333333</v>
+        <v>1897.863440860215</v>
       </c>
       <c r="M27" t="n">
-        <v>1605.3</v>
+        <v>1729.366666666667</v>
       </c>
       <c r="N27" t="n">
-        <v>26.75588888888889</v>
+        <v>31.63105734767025</v>
       </c>
       <c r="O27" t="n">
-        <v>26.755</v>
+        <v>28.82277777777778</v>
       </c>
     </row>
     <row r="28">
@@ -5824,43 +5812,43 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>156</v>
+        <v>311</v>
       </c>
       <c r="D28" t="n">
-        <v>261.8352564102564</v>
+        <v>231.3711146838156</v>
       </c>
       <c r="E28" t="n">
-        <v>2.766666666666667</v>
+        <v>2.633333333333333</v>
       </c>
       <c r="F28" t="n">
-        <v>4.36392094017094</v>
+        <v>3.856185244730261</v>
       </c>
       <c r="G28" t="n">
-        <v>0.04611111111111111</v>
+        <v>0.04388888888888889</v>
       </c>
       <c r="H28" t="n">
-        <v>770.6377777777778</v>
+        <v>813.4525170068029</v>
       </c>
       <c r="I28" t="n">
-        <v>826.7416666666667</v>
+        <v>855.1833333333333</v>
       </c>
       <c r="J28" t="n">
-        <v>12.84396296296296</v>
+        <v>13.55754195011338</v>
       </c>
       <c r="K28" t="n">
-        <v>13.77902777777778</v>
+        <v>14.25305555555556</v>
       </c>
       <c r="L28" t="n">
-        <v>440.3436111111112</v>
+        <v>525.2495918367347</v>
       </c>
       <c r="M28" t="n">
-        <v>198.9666666666667</v>
+        <v>479.0166666666667</v>
       </c>
       <c r="N28" t="n">
-        <v>7.339060185185185</v>
+        <v>8.754159863945578</v>
       </c>
       <c r="O28" t="n">
-        <v>3.316111111111111</v>
+        <v>7.983611111111111</v>
       </c>
     </row>
     <row r="29">
@@ -5875,43 +5863,43 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>130</v>
+        <v>250</v>
       </c>
       <c r="D29" t="n">
-        <v>411.6869230769231</v>
+        <v>457.9451999999999</v>
       </c>
       <c r="E29" t="n">
-        <v>159.025</v>
+        <v>137.5416666666667</v>
       </c>
       <c r="F29" t="n">
-        <v>6.861448717948718</v>
+        <v>7.63242</v>
       </c>
       <c r="G29" t="n">
-        <v>2.650416666666667</v>
+        <v>2.292361111111111</v>
       </c>
       <c r="H29" t="n">
-        <v>825.6088461538461</v>
+        <v>915.1874163319947</v>
       </c>
       <c r="I29" t="n">
-        <v>919.1083333333333</v>
+        <v>930.5833333333334</v>
       </c>
       <c r="J29" t="n">
-        <v>13.76014743589744</v>
+        <v>15.25312360553324</v>
       </c>
       <c r="K29" t="n">
-        <v>15.31847222222222</v>
+        <v>15.50972222222222</v>
       </c>
       <c r="L29" t="n">
-        <v>413.9219230769231</v>
+        <v>456.0690763052209</v>
       </c>
       <c r="M29" t="n">
-        <v>163.7416666666667</v>
+        <v>163.2</v>
       </c>
       <c r="N29" t="n">
-        <v>6.898698717948718</v>
+        <v>7.601151271753681</v>
       </c>
       <c r="O29" t="n">
-        <v>2.729027777777778</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="30">
@@ -5926,43 +5914,43 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1816</v>
+        <v>4438</v>
       </c>
       <c r="D30" t="n">
-        <v>2.299045521292217</v>
+        <v>6.287738470782635</v>
       </c>
       <c r="E30" t="n">
-        <v>2.583333333333333</v>
+        <v>2.25</v>
       </c>
       <c r="F30" t="n">
-        <v>0.03831742535487029</v>
+        <v>0.1047956411797106</v>
       </c>
       <c r="G30" t="n">
-        <v>0.04305555555555556</v>
+        <v>0.0375</v>
       </c>
       <c r="H30" t="n">
-        <v>242.1395969498911</v>
+        <v>275.35937919914</v>
       </c>
       <c r="I30" t="n">
-        <v>90.84166666666667</v>
+        <v>100.7333333333333</v>
       </c>
       <c r="J30" t="n">
-        <v>4.035659949164851</v>
+        <v>4.589322986652334</v>
       </c>
       <c r="K30" t="n">
-        <v>1.514027777777778</v>
+        <v>1.678888888888889</v>
       </c>
       <c r="L30" t="n">
-        <v>239.5165468409586</v>
+        <v>267.9853130878796</v>
       </c>
       <c r="M30" t="n">
-        <v>88.15833333333333</v>
+        <v>97</v>
       </c>
       <c r="N30" t="n">
-        <v>3.99194244734931</v>
+        <v>4.466421884797993</v>
       </c>
       <c r="O30" t="n">
-        <v>1.469305555555556</v>
+        <v>1.616666666666667</v>
       </c>
     </row>
     <row r="31">
@@ -5977,43 +5965,43 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1309</v>
+        <v>2265</v>
       </c>
       <c r="D31" t="n">
-        <v>2556.705449452509</v>
+        <v>2399.42233995585</v>
       </c>
       <c r="E31" t="n">
-        <v>2044.233333333333</v>
+        <v>2078.766666666667</v>
       </c>
       <c r="F31" t="n">
-        <v>42.61175749087514</v>
+        <v>39.9903723325975</v>
       </c>
       <c r="G31" t="n">
-        <v>34.07055555555556</v>
+        <v>34.64611111111112</v>
       </c>
       <c r="H31" t="n">
-        <v>2894.496544876887</v>
+        <v>2719.90314232902</v>
       </c>
       <c r="I31" t="n">
-        <v>2372.7</v>
+        <v>2395.25</v>
       </c>
       <c r="J31" t="n">
-        <v>48.24160908128145</v>
+        <v>45.33171903881701</v>
       </c>
       <c r="K31" t="n">
-        <v>39.54499999999999</v>
+        <v>39.92083333333333</v>
       </c>
       <c r="L31" t="n">
-        <v>331.1936060365369</v>
+        <v>315.5275955021564</v>
       </c>
       <c r="M31" t="n">
-        <v>352.5833333333333</v>
+        <v>350.25</v>
       </c>
       <c r="N31" t="n">
-        <v>5.519893433942283</v>
+        <v>5.258793258369275</v>
       </c>
       <c r="O31" t="n">
-        <v>5.876388888888888</v>
+        <v>5.8375</v>
       </c>
     </row>
     <row r="32">
@@ -6028,43 +6016,43 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2076</v>
+        <v>4689</v>
       </c>
       <c r="D32" t="n">
-        <v>293.0092565831728</v>
+        <v>394.2848475154617</v>
       </c>
       <c r="E32" t="n">
-        <v>2.733333333333333</v>
+        <v>2.75</v>
       </c>
       <c r="F32" t="n">
-        <v>4.883487609719546</v>
+        <v>6.571414125257695</v>
       </c>
       <c r="G32" t="n">
-        <v>0.04555555555555556</v>
+        <v>0.04583333333333333</v>
       </c>
       <c r="H32" t="n">
-        <v>603.0128722970215</v>
+        <v>680.8264452152259</v>
       </c>
       <c r="I32" t="n">
-        <v>430.2416666666667</v>
+        <v>460.4833333333333</v>
       </c>
       <c r="J32" t="n">
-        <v>10.0502145382837</v>
+        <v>11.34710742025377</v>
       </c>
       <c r="K32" t="n">
-        <v>7.170694444444445</v>
+        <v>7.674722222222222</v>
       </c>
       <c r="L32" t="n">
-        <v>232.5903814769482</v>
+        <v>193.7567725008894</v>
       </c>
       <c r="M32" t="n">
-        <v>58.64166666666667</v>
+        <v>49.60833333333333</v>
       </c>
       <c r="N32" t="n">
-        <v>3.876506357949137</v>
+        <v>3.229279541681489</v>
       </c>
       <c r="O32" t="n">
-        <v>0.9773611111111111</v>
+        <v>0.8268055555555556</v>
       </c>
     </row>
     <row r="33">
@@ -6079,43 +6067,43 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1732</v>
+        <v>4217</v>
       </c>
       <c r="D33" t="n">
-        <v>450.8132217090069</v>
+        <v>524.9136550470319</v>
       </c>
       <c r="E33" t="n">
-        <v>153.0583333333333</v>
+        <v>162.3833333333333</v>
       </c>
       <c r="F33" t="n">
-        <v>7.513553695150116</v>
+        <v>8.748560917450531</v>
       </c>
       <c r="G33" t="n">
-        <v>2.550972222222222</v>
+        <v>2.706388888888889</v>
       </c>
       <c r="H33" t="n">
-        <v>665.5287597857437</v>
+        <v>744.4262180668948</v>
       </c>
       <c r="I33" t="n">
-        <v>545.275</v>
+        <v>563.1833333333333</v>
       </c>
       <c r="J33" t="n">
-        <v>11.09214599642906</v>
+        <v>12.40710363444825</v>
       </c>
       <c r="K33" t="n">
-        <v>9.087916666666665</v>
+        <v>9.386388888888888</v>
       </c>
       <c r="L33" t="n">
-        <v>200.658941079522</v>
+        <v>190.1863269247652</v>
       </c>
       <c r="M33" t="n">
-        <v>44.8</v>
+        <v>48.61666666666667</v>
       </c>
       <c r="N33" t="n">
-        <v>3.344315684658701</v>
+        <v>3.169772115412753</v>
       </c>
       <c r="O33" t="n">
-        <v>0.7466666666666666</v>
+        <v>0.8102777777777778</v>
       </c>
     </row>
     <row r="34">
@@ -6130,43 +6118,43 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>846</v>
+        <v>1885</v>
       </c>
       <c r="D34" t="n">
-        <v>1385.587765957447</v>
+        <v>1223.31658709107</v>
       </c>
       <c r="E34" t="n">
-        <v>1148.316666666667</v>
+        <v>911.1166666666667</v>
       </c>
       <c r="F34" t="n">
-        <v>23.09312943262411</v>
+        <v>20.38860978485116</v>
       </c>
       <c r="G34" t="n">
-        <v>19.13861111111111</v>
+        <v>15.18527777777778</v>
       </c>
       <c r="H34" t="n">
-        <v>1603.701923076923</v>
+        <v>1565.748784440843</v>
       </c>
       <c r="I34" t="n">
-        <v>1530.525</v>
+        <v>1217.275</v>
       </c>
       <c r="J34" t="n">
-        <v>26.72836538461538</v>
+        <v>26.09581307401405</v>
       </c>
       <c r="K34" t="n">
-        <v>25.50875</v>
+        <v>20.28791666666667</v>
       </c>
       <c r="L34" t="n">
-        <v>452.9673076923077</v>
+        <v>378.1214613722312</v>
       </c>
       <c r="M34" t="n">
-        <v>562.1</v>
+        <v>437.1833333333333</v>
       </c>
       <c r="N34" t="n">
-        <v>7.549455128205129</v>
+        <v>6.302024356203853</v>
       </c>
       <c r="O34" t="n">
-        <v>9.368333333333334</v>
+        <v>7.286388888888889</v>
       </c>
     </row>
     <row r="35">
@@ -6181,43 +6169,43 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>814</v>
+        <v>1853</v>
       </c>
       <c r="D35" t="n">
-        <v>1728.951842751843</v>
+        <v>1505.343658931462</v>
       </c>
       <c r="E35" t="n">
-        <v>1830.591666666667</v>
+        <v>1048.533333333333</v>
       </c>
       <c r="F35" t="n">
-        <v>28.81586404586405</v>
+        <v>25.08906098219104</v>
       </c>
       <c r="G35" t="n">
-        <v>30.50986111111111</v>
+        <v>17.47555555555556</v>
       </c>
       <c r="H35" t="n">
-        <v>1939.052753623188</v>
+        <v>1828.769950124688</v>
       </c>
       <c r="I35" t="n">
-        <v>1737</v>
+        <v>1448.966666666667</v>
       </c>
       <c r="J35" t="n">
-        <v>32.31754589371981</v>
+        <v>30.47949916874481</v>
       </c>
       <c r="K35" t="n">
-        <v>28.95</v>
+        <v>24.14944444444444</v>
       </c>
       <c r="L35" t="n">
-        <v>474.3645893719806</v>
+        <v>381.515599889166</v>
       </c>
       <c r="M35" t="n">
-        <v>562</v>
+        <v>437.1666666666667</v>
       </c>
       <c r="N35" t="n">
-        <v>7.906076489533012</v>
+        <v>6.3585933314861</v>
       </c>
       <c r="O35" t="n">
-        <v>9.366666666666667</v>
+        <v>7.286111111111111</v>
       </c>
     </row>
     <row r="36">
@@ -6232,43 +6220,43 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>131</v>
+        <v>441</v>
       </c>
       <c r="D36" t="n">
-        <v>1.233206106870229</v>
+        <v>6.653061224489795</v>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="F36" t="n">
-        <v>0.02055343511450381</v>
+        <v>0.1108843537414966</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="H36" t="n">
-        <v>690.9660256410257</v>
+        <v>1127.888141025641</v>
       </c>
       <c r="I36" t="n">
-        <v>396.15</v>
+        <v>1187.741666666667</v>
       </c>
       <c r="J36" t="n">
-        <v>11.51610042735043</v>
+        <v>18.79813568376069</v>
       </c>
       <c r="K36" t="n">
-        <v>6.6025</v>
+        <v>19.79569444444444</v>
       </c>
       <c r="L36" t="n">
-        <v>688.3766025641027</v>
+        <v>1117.468461538462</v>
       </c>
       <c r="M36" t="n">
-        <v>393.4833333333333</v>
+        <v>1183.9</v>
       </c>
       <c r="N36" t="n">
-        <v>11.47294337606838</v>
+        <v>18.62447435897436</v>
       </c>
       <c r="O36" t="n">
-        <v>6.558055555555556</v>
+        <v>19.73166666666667</v>
       </c>
     </row>
     <row r="37">
@@ -6283,43 +6271,43 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>178</v>
+        <v>423</v>
       </c>
       <c r="D37" t="n">
-        <v>5612.686235955057</v>
+        <v>3711.479078014184</v>
       </c>
       <c r="E37" t="n">
-        <v>6836.775</v>
+        <v>3594.85</v>
       </c>
       <c r="F37" t="n">
-        <v>93.54477059925094</v>
+        <v>61.85798463356974</v>
       </c>
       <c r="G37" t="n">
-        <v>113.94625</v>
+        <v>59.91416666666667</v>
       </c>
       <c r="H37" t="n">
-        <v>6325.357723577235</v>
+        <v>4214.574083546462</v>
       </c>
       <c r="I37" t="n">
-        <v>7186.825000000001</v>
+        <v>4370.65</v>
       </c>
       <c r="J37" t="n">
-        <v>105.4226287262873</v>
+        <v>70.24290139244103</v>
       </c>
       <c r="K37" t="n">
-        <v>119.7804166666667</v>
+        <v>72.84416666666667</v>
       </c>
       <c r="L37" t="n">
-        <v>293.5424796747968</v>
+        <v>235.9774083546462</v>
       </c>
       <c r="M37" t="n">
-        <v>303.6083333333333</v>
+        <v>238.5666666666667</v>
       </c>
       <c r="N37" t="n">
-        <v>4.892374661246611</v>
+        <v>3.932956805910769</v>
       </c>
       <c r="O37" t="n">
-        <v>5.06013888888889</v>
+        <v>3.976111111111111</v>
       </c>
     </row>
     <row r="38">
@@ -6334,43 +6322,43 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>224</v>
+        <v>554</v>
       </c>
       <c r="D38" t="n">
-        <v>1.953050595238095</v>
+        <v>3.376865222623346</v>
       </c>
       <c r="E38" t="n">
-        <v>2.433333333333333</v>
+        <v>1.808333333333333</v>
       </c>
       <c r="F38" t="n">
-        <v>0.03255084325396825</v>
+        <v>0.05628108704372242</v>
       </c>
       <c r="G38" t="n">
-        <v>0.04055555555555555</v>
+        <v>0.03013888888888889</v>
       </c>
       <c r="H38" t="n">
-        <v>388.2659763313609</v>
+        <v>494.613768115942</v>
       </c>
       <c r="I38" t="n">
-        <v>411.2833333333334</v>
+        <v>425.3916666666667</v>
       </c>
       <c r="J38" t="n">
-        <v>6.471099605522682</v>
+        <v>8.243562801932367</v>
       </c>
       <c r="K38" t="n">
-        <v>6.854722222222223</v>
+        <v>7.089861111111111</v>
       </c>
       <c r="L38" t="n">
-        <v>385.8447731755424</v>
+        <v>490.2009661835749</v>
       </c>
       <c r="M38" t="n">
-        <v>409.05</v>
+        <v>423.075</v>
       </c>
       <c r="N38" t="n">
-        <v>6.430746219592375</v>
+        <v>8.170016103059581</v>
       </c>
       <c r="O38" t="n">
-        <v>6.8175</v>
+        <v>7.05125</v>
       </c>
     </row>
     <row r="39">
@@ -6385,43 +6373,43 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>209</v>
+        <v>573</v>
       </c>
       <c r="D39" t="n">
-        <v>241.2178628389155</v>
+        <v>209.3271087841769</v>
       </c>
       <c r="E39" t="n">
-        <v>68.34999999999999</v>
+        <v>70.71666666666667</v>
       </c>
       <c r="F39" t="n">
-        <v>4.020297713981924</v>
+        <v>3.488785146402948</v>
       </c>
       <c r="G39" t="n">
-        <v>1.139166666666667</v>
+        <v>1.178611111111111</v>
       </c>
       <c r="H39" t="n">
-        <v>626.7366834170854</v>
+        <v>700.2947954271962</v>
       </c>
       <c r="I39" t="n">
-        <v>535.4833333333333</v>
+        <v>666.45</v>
       </c>
       <c r="J39" t="n">
-        <v>10.44561139028476</v>
+        <v>11.6715799237866</v>
       </c>
       <c r="K39" t="n">
-        <v>8.924722222222222</v>
+        <v>11.1075</v>
       </c>
       <c r="L39" t="n">
-        <v>379.7951423785595</v>
+        <v>488.8802948255114</v>
       </c>
       <c r="M39" t="n">
-        <v>297.2166666666666</v>
+        <v>311.5333333333333</v>
       </c>
       <c r="N39" t="n">
-        <v>6.329919039642657</v>
+        <v>8.148004913758523</v>
       </c>
       <c r="O39" t="n">
-        <v>4.953611111111111</v>
+        <v>5.192222222222222</v>
       </c>
     </row>
     <row r="40">
@@ -6436,40 +6424,40 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>7091</v>
+        <v>19789</v>
       </c>
       <c r="D40" t="n">
-        <v>25.77965026089409</v>
+        <v>42.78900820321054</v>
       </c>
       <c r="E40" t="n">
-        <v>2.566666666666667</v>
+        <v>2</v>
       </c>
       <c r="F40" t="n">
-        <v>0.4296608376815682</v>
+        <v>0.7131501367201756</v>
       </c>
       <c r="G40" t="n">
-        <v>0.04277777777777778</v>
+        <v>0.03333333333333333</v>
       </c>
       <c r="H40" t="n">
-        <v>40.47532175032175</v>
+        <v>63.28917757249166</v>
       </c>
       <c r="I40" t="n">
-        <v>2.9</v>
+        <v>2.65</v>
       </c>
       <c r="J40" t="n">
-        <v>0.6745886958386959</v>
+        <v>1.054819626208195</v>
       </c>
       <c r="K40" t="n">
-        <v>0.04833333333333333</v>
+        <v>0.04416666666666667</v>
       </c>
       <c r="L40" t="n">
-        <v>8.916959166959169</v>
+        <v>10.4029606107262</v>
       </c>
       <c r="M40" t="n">
         <v>0.2333333333333333</v>
       </c>
       <c r="N40" t="n">
-        <v>0.1486159861159861</v>
+        <v>0.1733826768454367</v>
       </c>
       <c r="O40" t="n">
         <v>0.003888888888888889</v>
@@ -6487,43 +6475,43 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2130</v>
+        <v>6175</v>
       </c>
       <c r="D41" t="n">
-        <v>541.180297339593</v>
+        <v>837.8131848852902</v>
       </c>
       <c r="E41" t="n">
-        <v>355.0583333333333</v>
+        <v>758.0833333333334</v>
       </c>
       <c r="F41" t="n">
-        <v>9.019671622326552</v>
+        <v>13.9635530814215</v>
       </c>
       <c r="G41" t="n">
-        <v>5.917638888888889</v>
+        <v>12.63472222222222</v>
       </c>
       <c r="H41" t="n">
-        <v>599.6213436194149</v>
+        <v>892.2253652280584</v>
       </c>
       <c r="I41" t="n">
-        <v>441.55</v>
+        <v>813.6416666666667</v>
       </c>
       <c r="J41" t="n">
-        <v>9.993689060323584</v>
+        <v>14.87042275380097</v>
       </c>
       <c r="K41" t="n">
-        <v>7.359166666666667</v>
+        <v>13.56069444444444</v>
       </c>
       <c r="L41" t="n">
-        <v>56.12655094824815</v>
+        <v>47.41918423106947</v>
       </c>
       <c r="M41" t="n">
-        <v>49.58333333333334</v>
+        <v>41.975</v>
       </c>
       <c r="N41" t="n">
-        <v>0.9354425158041357</v>
+        <v>0.7903197371844912</v>
       </c>
       <c r="O41" t="n">
-        <v>0.826388888888889</v>
+        <v>0.6995833333333333</v>
       </c>
     </row>
     <row r="42">
@@ -6538,43 +6526,43 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>16240</v>
+        <v>41652</v>
       </c>
       <c r="D42" t="n">
-        <v>2.520657840722496</v>
+        <v>4.700954736067096</v>
       </c>
       <c r="E42" t="n">
-        <v>2.616666666666667</v>
+        <v>2.3</v>
       </c>
       <c r="F42" t="n">
-        <v>0.04201096401204159</v>
+        <v>0.07834924560111828</v>
       </c>
       <c r="G42" t="n">
-        <v>0.04361111111111111</v>
+        <v>0.03833333333333333</v>
       </c>
       <c r="H42" t="n">
-        <v>304.2713635570186</v>
+        <v>328.1241875116349</v>
       </c>
       <c r="I42" t="n">
-        <v>155.4666666666667</v>
+        <v>157.0833333333333</v>
       </c>
       <c r="J42" t="n">
-        <v>5.071189392616975</v>
+        <v>5.46873645852725</v>
       </c>
       <c r="K42" t="n">
-        <v>2.591111111111111</v>
+        <v>2.618055555555556</v>
       </c>
       <c r="L42" t="n">
-        <v>301.6504039799506</v>
+        <v>322.9746421328003</v>
       </c>
       <c r="M42" t="n">
-        <v>152.7833333333333</v>
+        <v>153.1666666666667</v>
       </c>
       <c r="N42" t="n">
-        <v>5.027506732999177</v>
+        <v>5.382910702213339</v>
       </c>
       <c r="O42" t="n">
-        <v>2.546388888888889</v>
+        <v>2.552777777777778</v>
       </c>
     </row>
     <row r="43">
@@ -6589,43 +6577,43 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>8499</v>
+        <v>25076</v>
       </c>
       <c r="D43" t="n">
-        <v>183.9063615327293</v>
+        <v>186.422750172808</v>
       </c>
       <c r="E43" t="n">
-        <v>94.81666666666666</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="F43" t="n">
-        <v>3.065106025545489</v>
+        <v>3.107045836213467</v>
       </c>
       <c r="G43" t="n">
-        <v>1.580277777777778</v>
+        <v>1.626666666666666</v>
       </c>
       <c r="H43" t="n">
-        <v>401.2816377599448</v>
+        <v>442.9232868705701</v>
       </c>
       <c r="I43" t="n">
-        <v>234.75</v>
+        <v>248.95</v>
       </c>
       <c r="J43" t="n">
-        <v>6.688027295999079</v>
+        <v>7.382054781176169</v>
       </c>
       <c r="K43" t="n">
-        <v>3.9125</v>
+        <v>4.149166666666667</v>
       </c>
       <c r="L43" t="n">
-        <v>224.0738998187937</v>
+        <v>261.4122342078394</v>
       </c>
       <c r="M43" t="n">
-        <v>106.8833333333333</v>
+        <v>104.1666666666667</v>
       </c>
       <c r="N43" t="n">
-        <v>3.734564996979895</v>
+        <v>4.356870570130658</v>
       </c>
       <c r="O43" t="n">
-        <v>1.781388888888889</v>
+        <v>1.736111111111111</v>
       </c>
     </row>
     <row r="44">
@@ -6640,43 +6628,43 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2708</v>
+        <v>5082</v>
       </c>
       <c r="D44" t="n">
-        <v>2.301550960118169</v>
+        <v>5.300721500721502</v>
       </c>
       <c r="E44" t="n">
-        <v>2.55</v>
+        <v>2.366666666666667</v>
       </c>
       <c r="F44" t="n">
-        <v>0.03835918266863614</v>
+        <v>0.08834535834535835</v>
       </c>
       <c r="G44" t="n">
-        <v>0.0425</v>
+        <v>0.03944444444444444</v>
       </c>
       <c r="H44" t="n">
-        <v>623.2935766111823</v>
+        <v>749.6880664652568</v>
       </c>
       <c r="I44" t="n">
-        <v>638.5166666666667</v>
+        <v>730.5833333333334</v>
       </c>
       <c r="J44" t="n">
-        <v>10.38822627685304</v>
+        <v>12.49480110775428</v>
       </c>
       <c r="K44" t="n">
-        <v>10.64194444444444</v>
+        <v>12.17638888888889</v>
       </c>
       <c r="L44" t="n">
-        <v>620.6899061032865</v>
+        <v>743.6155666589202</v>
       </c>
       <c r="M44" t="n">
-        <v>636.1333333333333</v>
+        <v>718.9</v>
       </c>
       <c r="N44" t="n">
-        <v>10.34483176838811</v>
+        <v>12.39359277764867</v>
       </c>
       <c r="O44" t="n">
-        <v>10.60222222222222</v>
+        <v>11.98166666666667</v>
       </c>
     </row>
     <row r="45">
@@ -6691,43 +6679,43 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>3108</v>
+        <v>5836</v>
       </c>
       <c r="D45" t="n">
-        <v>266.4696374946375</v>
+        <v>253.6480865889879</v>
       </c>
       <c r="E45" t="n">
-        <v>62.18333333333334</v>
+        <v>60.75833333333333</v>
       </c>
       <c r="F45" t="n">
-        <v>4.441160624910625</v>
+        <v>4.227468109816464</v>
       </c>
       <c r="G45" t="n">
-        <v>1.036388888888889</v>
+        <v>1.012638888888889</v>
       </c>
       <c r="H45" t="n">
-        <v>768.6591913806509</v>
+        <v>892.3451599476751</v>
       </c>
       <c r="I45" t="n">
-        <v>756.6166666666667</v>
+        <v>864.3666666666667</v>
       </c>
       <c r="J45" t="n">
-        <v>12.81098652301085</v>
+        <v>14.87241933246125</v>
       </c>
       <c r="K45" t="n">
-        <v>12.61027777777778</v>
+        <v>14.40611111111111</v>
       </c>
       <c r="L45" t="n">
-        <v>503.5153004554038</v>
+        <v>639.42041859912</v>
       </c>
       <c r="M45" t="n">
-        <v>459.1333333333333</v>
+        <v>486.4583333333334</v>
       </c>
       <c r="N45" t="n">
-        <v>8.391921674256729</v>
+        <v>10.657006976652</v>
       </c>
       <c r="O45" t="n">
-        <v>7.652222222222222</v>
+        <v>8.107638888888889</v>
       </c>
     </row>
     <row r="46">
@@ -6742,43 +6730,43 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>229</v>
+        <v>410</v>
       </c>
       <c r="D46" t="n">
-        <v>1.828311499272198</v>
+        <v>1.844634146341463</v>
       </c>
       <c r="E46" t="n">
-        <v>2.433333333333333</v>
+        <v>1.783333333333333</v>
       </c>
       <c r="F46" t="n">
-        <v>0.0304718583212033</v>
+        <v>0.03074390243902439</v>
       </c>
       <c r="G46" t="n">
-        <v>0.04055555555555555</v>
+        <v>0.02972222222222222</v>
       </c>
       <c r="H46" t="n">
-        <v>2286.81326754386</v>
+        <v>1978.26329588015</v>
       </c>
       <c r="I46" t="n">
-        <v>2410.116666666667</v>
+        <v>2088.65</v>
       </c>
       <c r="J46" t="n">
-        <v>38.11355445906432</v>
+        <v>32.97105493133584</v>
       </c>
       <c r="K46" t="n">
-        <v>40.16861111111111</v>
+        <v>34.81083333333333</v>
       </c>
       <c r="L46" t="n">
-        <v>2284.205372807017</v>
+        <v>1976.041947565543</v>
       </c>
       <c r="M46" t="n">
-        <v>2407.791666666667</v>
+        <v>2087.2</v>
       </c>
       <c r="N46" t="n">
-        <v>38.07008954678363</v>
+        <v>32.93403245942572</v>
       </c>
       <c r="O46" t="n">
-        <v>40.12986111111111</v>
+        <v>34.78666666666666</v>
       </c>
     </row>
     <row r="47">
@@ -6793,43 +6781,43 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>203</v>
+        <v>321</v>
       </c>
       <c r="D47" t="n">
-        <v>378.3878489326765</v>
+        <v>349.8322429906542</v>
       </c>
       <c r="E47" t="n">
-        <v>327.9333333333333</v>
+        <v>226.4166666666667</v>
       </c>
       <c r="F47" t="n">
-        <v>6.306464148877943</v>
+        <v>5.83053738317757</v>
       </c>
       <c r="G47" t="n">
-        <v>5.465555555555556</v>
+        <v>3.773611111111111</v>
       </c>
       <c r="H47" t="n">
-        <v>2301.548395721925</v>
+        <v>2061.298761261261</v>
       </c>
       <c r="I47" t="n">
-        <v>2545.85</v>
+        <v>2319.916666666667</v>
       </c>
       <c r="J47" t="n">
-        <v>38.35913992869875</v>
+        <v>34.35497935435435</v>
       </c>
       <c r="K47" t="n">
-        <v>42.43083333333333</v>
+        <v>38.66527777777777</v>
       </c>
       <c r="L47" t="n">
-        <v>1911.210071301248</v>
+        <v>1703.817060810811</v>
       </c>
       <c r="M47" t="n">
-        <v>1856.466666666667</v>
+        <v>1772.75</v>
       </c>
       <c r="N47" t="n">
-        <v>31.85350118835413</v>
+        <v>28.39695101351351</v>
       </c>
       <c r="O47" t="n">
-        <v>30.94111111111111</v>
+        <v>29.54583333333333</v>
       </c>
     </row>
     <row r="48">
@@ -6844,43 +6832,43 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1027</v>
+        <v>2327</v>
       </c>
       <c r="D48" t="n">
-        <v>2.400227198961376</v>
+        <v>4.991877954447786</v>
       </c>
       <c r="E48" t="n">
-        <v>2.6</v>
+        <v>2.266666666666667</v>
       </c>
       <c r="F48" t="n">
-        <v>0.04000378664935628</v>
+        <v>0.0831979659074631</v>
       </c>
       <c r="G48" t="n">
-        <v>0.04333333333333333</v>
+        <v>0.03777777777777778</v>
       </c>
       <c r="H48" t="n">
-        <v>387.2921736036997</v>
+        <v>458.702861952862</v>
       </c>
       <c r="I48" t="n">
-        <v>302.75</v>
+        <v>431.8</v>
       </c>
       <c r="J48" t="n">
-        <v>6.454869560061662</v>
+        <v>7.645047699214366</v>
       </c>
       <c r="K48" t="n">
-        <v>5.045833333333333</v>
+        <v>7.196666666666667</v>
       </c>
       <c r="L48" t="n">
-        <v>384.6745464247599</v>
+        <v>453.1417187750521</v>
       </c>
       <c r="M48" t="n">
-        <v>299.9333333333333</v>
+        <v>423.05</v>
       </c>
       <c r="N48" t="n">
-        <v>6.411242440412664</v>
+        <v>7.552361979584202</v>
       </c>
       <c r="O48" t="n">
-        <v>4.998888888888889</v>
+        <v>7.050833333333333</v>
       </c>
     </row>
     <row r="49">
@@ -6895,43 +6883,43 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>495</v>
+        <v>1046</v>
       </c>
       <c r="D49" t="n">
-        <v>230.5010101010101</v>
+        <v>321.2919056724028</v>
       </c>
       <c r="E49" t="n">
-        <v>71.36666666666666</v>
+        <v>93.60833333333333</v>
       </c>
       <c r="F49" t="n">
-        <v>3.841683501683502</v>
+        <v>5.354865094540047</v>
       </c>
       <c r="G49" t="n">
-        <v>1.189444444444444</v>
+        <v>1.560138888888889</v>
       </c>
       <c r="H49" t="n">
-        <v>621.4152173913044</v>
+        <v>745.5879129865882</v>
       </c>
       <c r="I49" t="n">
-        <v>529.5833333333334</v>
+        <v>594.9</v>
       </c>
       <c r="J49" t="n">
-        <v>10.35692028985507</v>
+        <v>12.42646521644314</v>
       </c>
       <c r="K49" t="n">
-        <v>8.826388888888889</v>
+        <v>9.914999999999999</v>
       </c>
       <c r="L49" t="n">
-        <v>391.1469289164942</v>
+        <v>424.0026005888126</v>
       </c>
       <c r="M49" t="n">
-        <v>253.0166666666667</v>
+        <v>276.6833333333333</v>
       </c>
       <c r="N49" t="n">
-        <v>6.519115481941569</v>
+        <v>7.066710009813542</v>
       </c>
       <c r="O49" t="n">
-        <v>4.216944444444445</v>
+        <v>4.611388888888889</v>
       </c>
     </row>
   </sheetData>
@@ -6974,45 +6962,45 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos Proyectados</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion Proyectado</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7332,77 +7320,77 @@
     </row>
     <row r="20"/>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Tipo Aprobacion</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Hrs)</t>
         </is>
@@ -8852,45 +8840,45 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos Proyectados</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion Proyectado</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9210,77 +9198,77 @@
     </row>
     <row r="20"/>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Tipo Aprobacion</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Hrs)</t>
         </is>
@@ -10730,45 +10718,45 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos Proyectados</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion Proyectado</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -11088,77 +11076,77 @@
     </row>
     <row r="20"/>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Tipo Aprobacion</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Hrs)</t>
         </is>
@@ -12608,45 +12596,45 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos Proyectados</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion Proyectado</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -12966,77 +12954,77 @@
     </row>
     <row r="20"/>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Tipo Aprobacion</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Hrs)</t>
         </is>
@@ -14462,45 +14450,45 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos Proyectados</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion Proyectado</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -14820,77 +14808,77 @@
     </row>
     <row r="20"/>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Tipo Aprobacion</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Hrs)</t>
         </is>
@@ -16304,45 +16292,45 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos Proyectados</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion Proyectado</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -16662,77 +16650,77 @@
     </row>
     <row r="20"/>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Tipo Aprobacion</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Hrs)</t>
         </is>
@@ -18134,45 +18122,45 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Retiros Automaticos Proyectados</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>% Automatizacion Proyectado</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18492,77 +18480,77 @@
     </row>
     <row r="20"/>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Tipo Aprobacion</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Total Retiros</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Min)</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Aprobado (Hrs)</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="1" t="inlineStr">
         <is>
           <t>Promedio Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K21" s="1" t="inlineStr">
         <is>
           <t>Mediana Creado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Min)</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N21" s="1" t="inlineStr">
         <is>
           <t>Promedio Aprobado a Pagado (Hrs)</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O21" s="1" t="inlineStr">
         <is>
           <t>Mediana Aprobado a Pagado (Hrs)</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica dashboard lun 21/09/2026 14:12:52,91
</commit_message>
<xml_diff>
--- a/Reporte_Efectividad_Automatizacion.xlsx
+++ b/Reporte_Efectividad_Automatizacion.xlsx
@@ -696,19 +696,19 @@
         <v>71.65194435983349</v>
       </c>
       <c r="Z2" t="n">
-        <v>2969</v>
+        <v>4144</v>
       </c>
       <c r="AA2" t="n">
-        <v>35.63489390367127</v>
+        <v>36.46235521235521</v>
       </c>
       <c r="AB2" t="n">
-        <v>69.51835634893904</v>
+        <v>69.73938223938224</v>
       </c>
       <c r="AC2" t="n">
-        <v>9.93685349347734</v>
+        <v>10.76431480216128</v>
       </c>
       <c r="AD2" t="n">
-        <v>-69.85480759467966</v>
+        <v>-57.92466240227434</v>
       </c>
     </row>
     <row r="3">
@@ -790,19 +790,19 @@
         <v>79.51807228915662</v>
       </c>
       <c r="Z3" t="n">
-        <v>231</v>
+        <v>309</v>
       </c>
       <c r="AA3" t="n">
-        <v>38.09523809523809</v>
+        <v>38.51132686084142</v>
       </c>
       <c r="AB3" t="n">
-        <v>80.08658008658008</v>
+        <v>80.90614886731392</v>
       </c>
       <c r="AC3" t="n">
-        <v>12.27768215720023</v>
+        <v>12.69377092280356</v>
       </c>
       <c r="AD3" t="n">
-        <v>-60.24096385542169</v>
+        <v>-46.815834767642</v>
       </c>
     </row>
     <row r="4">
@@ -884,19 +884,19 @@
         <v>62.42171189979123</v>
       </c>
       <c r="Z4" t="n">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="AA4" t="n">
-        <v>69.90291262135922</v>
+        <v>71.29629629629629</v>
       </c>
       <c r="AB4" t="n">
-        <v>75.72815533980582</v>
+        <v>76.85185185185185</v>
       </c>
       <c r="AC4" t="n">
-        <v>51.32253683847821</v>
+        <v>52.71592051341528</v>
       </c>
       <c r="AD4" t="n">
-        <v>-78.49686847599166</v>
+        <v>-77.45302713987473</v>
       </c>
     </row>
     <row r="5">
@@ -978,19 +978,19 @@
         <v>62.37424547283702</v>
       </c>
       <c r="Z5" t="n">
-        <v>561</v>
+        <v>725</v>
       </c>
       <c r="AA5" t="n">
-        <v>55.43672014260249</v>
+        <v>56.00000000000001</v>
       </c>
       <c r="AB5" t="n">
-        <v>59.18003565062389</v>
+        <v>59.72413793103448</v>
       </c>
       <c r="AC5" t="n">
-        <v>-0.2976862960292976</v>
+        <v>0.2655935613682203</v>
       </c>
       <c r="AD5" t="n">
-        <v>-71.78068410462777</v>
+        <v>-63.53118712273642</v>
       </c>
     </row>
     <row r="6">
@@ -1072,19 +1072,19 @@
         <v>82.54543623823189</v>
       </c>
       <c r="Z6" t="n">
-        <v>6703</v>
+        <v>8342</v>
       </c>
       <c r="AA6" t="n">
-        <v>66.2091600775772</v>
+        <v>72.5845121074083</v>
       </c>
       <c r="AB6" t="n">
-        <v>71.05773534238401</v>
+        <v>76.66027331575161</v>
       </c>
       <c r="AC6" t="n">
-        <v>-12.85744617525469</v>
+        <v>-6.482094145423588</v>
       </c>
       <c r="AD6" t="n">
-        <v>-66.25383879575089</v>
+        <v>-58.00231586366611</v>
       </c>
     </row>
     <row r="7">
@@ -1166,19 +1166,19 @@
         <v>64.37949170915806</v>
       </c>
       <c r="Z7" t="n">
-        <v>8906</v>
+        <v>11471</v>
       </c>
       <c r="AA7" t="n">
-        <v>52.64989894453178</v>
+        <v>53.31706041321593</v>
       </c>
       <c r="AB7" t="n">
-        <v>65.19200538962497</v>
+        <v>65.53046813704123</v>
       </c>
       <c r="AC7" t="n">
-        <v>8.152368129901362</v>
+        <v>8.819529598585511</v>
       </c>
       <c r="AD7" t="n">
-        <v>-64.24298390010841</v>
+        <v>-53.94467418797928</v>
       </c>
     </row>
     <row r="8">
@@ -1260,19 +1260,19 @@
         <v>63.24499030381383</v>
       </c>
       <c r="Z8" t="n">
-        <v>3738</v>
+        <v>4629</v>
       </c>
       <c r="AA8" t="n">
-        <v>50.42803638309257</v>
+        <v>49.85958090300281</v>
       </c>
       <c r="AB8" t="n">
-        <v>59.06902086677368</v>
+        <v>58.6951825448261</v>
       </c>
       <c r="AC8" t="n">
-        <v>1.016271677210213</v>
+        <v>0.4478161971204528</v>
       </c>
       <c r="AD8" t="n">
-        <v>-51.67420814479639</v>
+        <v>-40.15513897866839</v>
       </c>
     </row>
     <row r="9">
@@ -1354,19 +1354,19 @@
         <v>78.380257212374</v>
       </c>
       <c r="Z9" t="n">
-        <v>864</v>
+        <v>929</v>
       </c>
       <c r="AA9" t="n">
-        <v>51.04166666666666</v>
+        <v>52.52960172228202</v>
       </c>
       <c r="AB9" t="n">
-        <v>59.02777777777778</v>
+        <v>59.95694294940797</v>
       </c>
       <c r="AC9" t="n">
-        <v>-21.8467587765033</v>
+        <v>-20.35882372088794</v>
       </c>
       <c r="AD9" t="n">
-        <v>-69.9687174139729</v>
+        <v>-67.70941953423704</v>
       </c>
     </row>
     <row r="10">
@@ -1448,19 +1448,19 @@
         <v>54.65631929046562</v>
       </c>
       <c r="Z10" t="n">
-        <v>1127</v>
+        <v>1524</v>
       </c>
       <c r="AA10" t="n">
-        <v>49.15705412599822</v>
+        <v>47.76902887139108</v>
       </c>
       <c r="AB10" t="n">
-        <v>56.61047027506655</v>
+        <v>54.92125984251969</v>
       </c>
       <c r="AC10" t="n">
-        <v>15.6759011326501</v>
+        <v>14.28787587804296</v>
       </c>
       <c r="AD10" t="n">
-        <v>-58.35181079083518</v>
+        <v>-43.68070953436807</v>
       </c>
     </row>
     <row r="11">
@@ -1542,19 +1542,19 @@
         <v>81.92520288611654</v>
       </c>
       <c r="Z11" t="n">
-        <v>25964</v>
+        <v>34668</v>
       </c>
       <c r="AA11" t="n">
-        <v>76.21706978893853</v>
+        <v>80.2296065535941</v>
       </c>
       <c r="AB11" t="n">
-        <v>79.19812047450316</v>
+        <v>82.62086073612554</v>
       </c>
       <c r="AC11" t="n">
-        <v>-2.193315729845139</v>
+        <v>1.819221034810425</v>
       </c>
       <c r="AD11" t="n">
-        <v>-63.48190551203252</v>
+        <v>-51.23982053193434</v>
       </c>
     </row>
     <row r="12">
@@ -1636,19 +1636,19 @@
         <v>79.3433378990412</v>
       </c>
       <c r="Z12" t="n">
-        <v>66728</v>
+        <v>93138</v>
       </c>
       <c r="AA12" t="n">
-        <v>62.42057307277305</v>
+        <v>62.36337477721231</v>
       </c>
       <c r="AB12" t="n">
-        <v>77.83988730368061</v>
+        <v>77.71800983486868</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.1461507014710151</v>
+        <v>0.08895240591027687</v>
       </c>
       <c r="AD12" t="n">
-        <v>-66.64300496895652</v>
+        <v>-53.44077743673829</v>
       </c>
     </row>
     <row r="13">
@@ -1730,19 +1730,19 @@
         <v>67.14883504675311</v>
       </c>
       <c r="Z13" t="n">
-        <v>10918</v>
+        <v>14316</v>
       </c>
       <c r="AA13" t="n">
-        <v>46.54698662758747</v>
+        <v>46.17211511595418</v>
       </c>
       <c r="AB13" t="n">
-        <v>65.90950723575747</v>
+        <v>65.66778429728974</v>
       </c>
       <c r="AC13" t="n">
-        <v>3.683939667831311</v>
+        <v>3.309068156198016</v>
       </c>
       <c r="AD13" t="n">
-        <v>-71.79831585472955</v>
+        <v>-63.02112930722736</v>
       </c>
     </row>
     <row r="14">
@@ -1824,19 +1824,19 @@
         <v>72.04349796103308</v>
       </c>
       <c r="Z14" t="n">
-        <v>731</v>
+        <v>800</v>
       </c>
       <c r="AA14" t="n">
-        <v>56.0875512995896</v>
+        <v>56.75</v>
       </c>
       <c r="AB14" t="n">
-        <v>72.64021887824897</v>
+        <v>74</v>
       </c>
       <c r="AC14" t="n">
-        <v>7.356241829721</v>
+        <v>8.018690530131401</v>
       </c>
       <c r="AD14" t="n">
-        <v>-83.43905754417762</v>
+        <v>-81.87584956955143</v>
       </c>
     </row>
     <row r="15">
@@ -1918,19 +1918,19 @@
         <v>78.43225419664267</v>
       </c>
       <c r="Z15" t="n">
-        <v>3373</v>
+        <v>4376</v>
       </c>
       <c r="AA15" t="n">
-        <v>68.98903053661429</v>
+        <v>70.58957952468006</v>
       </c>
       <c r="AB15" t="n">
-        <v>74.8295286095464</v>
+        <v>76.21115173674589</v>
       </c>
       <c r="AC15" t="n">
-        <v>-0.7426840916830599</v>
+        <v>0.8578648963827078</v>
       </c>
       <c r="AD15" t="n">
-        <v>-74.72272182254197</v>
+        <v>-67.20623501199042</v>
       </c>
     </row>
   </sheetData>
@@ -3851,19 +3851,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2690</v>
+        <v>4024</v>
       </c>
       <c r="C4" t="n">
-        <v>339</v>
+        <v>490</v>
       </c>
       <c r="D4" t="n">
-        <v>12.60223048327138</v>
+        <v>12.17693836978131</v>
       </c>
       <c r="E4" t="n">
-        <v>1597.919646017699</v>
+        <v>1470.57206122449</v>
       </c>
       <c r="F4" t="n">
-        <v>1918.06940450872</v>
+        <v>1584.896924165252</v>
       </c>
     </row>
     <row r="5">
@@ -3873,19 +3873,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>92740</v>
+        <v>126762</v>
       </c>
       <c r="C5" t="n">
-        <v>76197</v>
+        <v>104586</v>
       </c>
       <c r="D5" t="n">
-        <v>82.16195816260513</v>
+        <v>82.50579826761964</v>
       </c>
       <c r="E5" t="n">
-        <v>3535.304440253553</v>
+        <v>3525.8840265809</v>
       </c>
       <c r="F5" t="n">
-        <v>8884.176789518226</v>
+        <v>7913.708640827922</v>
       </c>
     </row>
     <row r="6">
@@ -3895,19 +3895,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30169</v>
+        <v>39499</v>
       </c>
       <c r="C6" t="n">
-        <v>3737</v>
+        <v>5463</v>
       </c>
       <c r="D6" t="n">
-        <v>12.38688720209487</v>
+        <v>13.830729891896</v>
       </c>
       <c r="E6" t="n">
-        <v>10332.67597805727</v>
+        <v>9392.321089145158</v>
       </c>
       <c r="F6" t="n">
-        <v>4782.103336107748</v>
+        <v>4252.136308908215</v>
       </c>
     </row>
     <row r="7">
@@ -3917,19 +3917,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7317</v>
+        <v>9194</v>
       </c>
       <c r="C7" t="n">
-        <v>2523</v>
+        <v>3320</v>
       </c>
       <c r="D7" t="n">
-        <v>34.48134481344813</v>
+        <v>36.11050685229498</v>
       </c>
       <c r="E7" t="n">
-        <v>1479.006062227507</v>
+        <v>1585.639206325301</v>
       </c>
       <c r="F7" t="n">
-        <v>5528.920880267</v>
+        <v>4614.78207524685</v>
       </c>
     </row>
     <row r="8"/>
@@ -5107,19 +5107,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2969</v>
+        <v>4144</v>
       </c>
       <c r="C4" t="n">
-        <v>1058</v>
+        <v>1511</v>
       </c>
       <c r="D4" t="n">
-        <v>35.63489390367127</v>
+        <v>36.46235521235521</v>
       </c>
       <c r="E4" t="n">
-        <v>2064</v>
+        <v>2890</v>
       </c>
       <c r="F4" t="n">
-        <v>69.51835634893904</v>
+        <v>69.73938223938224</v>
       </c>
     </row>
     <row r="5">
@@ -5129,19 +5129,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>231</v>
+        <v>309</v>
       </c>
       <c r="C5" t="n">
-        <v>88</v>
+        <v>119</v>
       </c>
       <c r="D5" t="n">
-        <v>38.09523809523809</v>
+        <v>38.51132686084142</v>
       </c>
       <c r="E5" t="n">
-        <v>185</v>
+        <v>250</v>
       </c>
       <c r="F5" t="n">
-        <v>80.08658008658008</v>
+        <v>80.90614886731392</v>
       </c>
     </row>
     <row r="6">
@@ -5151,19 +5151,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C6" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D6" t="n">
-        <v>69.90291262135922</v>
+        <v>71.29629629629629</v>
       </c>
       <c r="E6" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F6" t="n">
-        <v>75.72815533980582</v>
+        <v>76.85185185185185</v>
       </c>
     </row>
     <row r="7">
@@ -5173,19 +5173,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>561</v>
+        <v>725</v>
       </c>
       <c r="C7" t="n">
-        <v>311</v>
+        <v>406</v>
       </c>
       <c r="D7" t="n">
-        <v>55.43672014260249</v>
+        <v>56.00000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>332</v>
+        <v>433</v>
       </c>
       <c r="F7" t="n">
-        <v>59.18003565062389</v>
+        <v>59.72413793103448</v>
       </c>
     </row>
     <row r="8">
@@ -5195,19 +5195,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6703</v>
+        <v>8342</v>
       </c>
       <c r="C8" t="n">
-        <v>4438</v>
+        <v>6055</v>
       </c>
       <c r="D8" t="n">
-        <v>66.2091600775772</v>
+        <v>72.5845121074083</v>
       </c>
       <c r="E8" t="n">
-        <v>4763</v>
+        <v>6395</v>
       </c>
       <c r="F8" t="n">
-        <v>71.05773534238401</v>
+        <v>76.66027331575161</v>
       </c>
     </row>
     <row r="9">
@@ -5217,19 +5217,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8906</v>
+        <v>11471</v>
       </c>
       <c r="C9" t="n">
-        <v>4689</v>
+        <v>6116</v>
       </c>
       <c r="D9" t="n">
-        <v>52.64989894453178</v>
+        <v>53.31706041321593</v>
       </c>
       <c r="E9" t="n">
-        <v>5806</v>
+        <v>7517</v>
       </c>
       <c r="F9" t="n">
-        <v>65.19200538962497</v>
+        <v>65.53046813704123</v>
       </c>
     </row>
     <row r="10">
@@ -5239,19 +5239,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3738</v>
+        <v>4629</v>
       </c>
       <c r="C10" t="n">
-        <v>1885</v>
+        <v>2308</v>
       </c>
       <c r="D10" t="n">
-        <v>50.42803638309257</v>
+        <v>49.85958090300281</v>
       </c>
       <c r="E10" t="n">
-        <v>2208</v>
+        <v>2717</v>
       </c>
       <c r="F10" t="n">
-        <v>59.06902086677368</v>
+        <v>58.6951825448261</v>
       </c>
     </row>
     <row r="11">
@@ -5261,19 +5261,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>864</v>
+        <v>929</v>
       </c>
       <c r="C11" t="n">
-        <v>441</v>
+        <v>488</v>
       </c>
       <c r="D11" t="n">
-        <v>51.04166666666666</v>
+        <v>52.52960172228202</v>
       </c>
       <c r="E11" t="n">
-        <v>510</v>
+        <v>557</v>
       </c>
       <c r="F11" t="n">
-        <v>59.02777777777778</v>
+        <v>59.95694294940797</v>
       </c>
     </row>
     <row r="12">
@@ -5283,19 +5283,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1127</v>
+        <v>1524</v>
       </c>
       <c r="C12" t="n">
-        <v>554</v>
+        <v>728</v>
       </c>
       <c r="D12" t="n">
-        <v>49.15705412599822</v>
+        <v>47.76902887139108</v>
       </c>
       <c r="E12" t="n">
-        <v>638</v>
+        <v>837</v>
       </c>
       <c r="F12" t="n">
-        <v>56.61047027506655</v>
+        <v>54.92125984251969</v>
       </c>
     </row>
     <row r="13">
@@ -5305,19 +5305,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>25964</v>
+        <v>34668</v>
       </c>
       <c r="C13" t="n">
-        <v>19789</v>
+        <v>27814</v>
       </c>
       <c r="D13" t="n">
-        <v>76.21706978893853</v>
+        <v>80.2296065535941</v>
       </c>
       <c r="E13" t="n">
-        <v>20563</v>
+        <v>28643</v>
       </c>
       <c r="F13" t="n">
-        <v>79.19812047450316</v>
+        <v>82.62086073612554</v>
       </c>
     </row>
     <row r="14">
@@ -5327,19 +5327,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>66728</v>
+        <v>93138</v>
       </c>
       <c r="C14" t="n">
-        <v>41652</v>
+        <v>58084</v>
       </c>
       <c r="D14" t="n">
-        <v>62.42057307277305</v>
+        <v>62.36337477721231</v>
       </c>
       <c r="E14" t="n">
-        <v>51941</v>
+        <v>72385</v>
       </c>
       <c r="F14" t="n">
-        <v>77.83988730368061</v>
+        <v>77.71800983486868</v>
       </c>
     </row>
     <row r="15">
@@ -5349,19 +5349,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10918</v>
+        <v>14316</v>
       </c>
       <c r="C15" t="n">
-        <v>5082</v>
+        <v>6610</v>
       </c>
       <c r="D15" t="n">
-        <v>46.54698662758747</v>
+        <v>46.17211511595418</v>
       </c>
       <c r="E15" t="n">
-        <v>7196</v>
+        <v>9401</v>
       </c>
       <c r="F15" t="n">
-        <v>65.90950723575747</v>
+        <v>65.66778429728974</v>
       </c>
     </row>
     <row r="16">
@@ -5371,19 +5371,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>731</v>
+        <v>800</v>
       </c>
       <c r="C16" t="n">
-        <v>410</v>
+        <v>454</v>
       </c>
       <c r="D16" t="n">
-        <v>56.0875512995896</v>
+        <v>56.75</v>
       </c>
       <c r="E16" t="n">
-        <v>531</v>
+        <v>592</v>
       </c>
       <c r="F16" t="n">
-        <v>72.64021887824897</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17">
@@ -5393,19 +5393,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3373</v>
+        <v>4376</v>
       </c>
       <c r="C17" t="n">
-        <v>2327</v>
+        <v>3089</v>
       </c>
       <c r="D17" t="n">
-        <v>68.98903053661429</v>
+        <v>70.58957952468006</v>
       </c>
       <c r="E17" t="n">
-        <v>2524</v>
+        <v>3335</v>
       </c>
       <c r="F17" t="n">
-        <v>74.8295286095464</v>
+        <v>76.21115173674589</v>
       </c>
     </row>
     <row r="18"/>
@@ -5506,43 +5506,43 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1058</v>
+        <v>1511</v>
       </c>
       <c r="D22" t="n">
-        <v>5.055718336483932</v>
+        <v>3.950838296933598</v>
       </c>
       <c r="E22" t="n">
-        <v>2.033333333333333</v>
+        <v>1.8</v>
       </c>
       <c r="F22" t="n">
-        <v>0.0842619722747322</v>
+        <v>0.06584730494889329</v>
       </c>
       <c r="G22" t="n">
-        <v>0.03388888888888889</v>
+        <v>0.03</v>
       </c>
       <c r="H22" t="n">
-        <v>195.410458240946</v>
+        <v>211.7491827438371</v>
       </c>
       <c r="I22" t="n">
-        <v>73.35833333333332</v>
+        <v>79.26666666666667</v>
       </c>
       <c r="J22" t="n">
-        <v>3.256840970682434</v>
+        <v>3.529153045730618</v>
       </c>
       <c r="K22" t="n">
-        <v>1.222638888888889</v>
+        <v>1.321111111111111</v>
       </c>
       <c r="L22" t="n">
-        <v>189.780155210643</v>
+        <v>207.1934887459807</v>
       </c>
       <c r="M22" t="n">
-        <v>67.46666666666667</v>
+        <v>73.97499999999999</v>
       </c>
       <c r="N22" t="n">
-        <v>3.163002586844051</v>
+        <v>3.453224812433012</v>
       </c>
       <c r="O22" t="n">
-        <v>1.124444444444444</v>
+        <v>1.232916666666667</v>
       </c>
     </row>
     <row r="23">
@@ -5557,43 +5557,43 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1911</v>
+        <v>2633</v>
       </c>
       <c r="D23" t="n">
-        <v>249.7237571951858</v>
+        <v>270.6461704013166</v>
       </c>
       <c r="E23" t="n">
-        <v>69.33333333333333</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>4.162062619919763</v>
+        <v>4.51076950668861</v>
       </c>
       <c r="G23" t="n">
-        <v>1.155555555555555</v>
+        <v>1.385</v>
       </c>
       <c r="H23" t="n">
-        <v>275.095775770457</v>
+        <v>293.4541073032987</v>
       </c>
       <c r="I23" t="n">
-        <v>97.65833333333333</v>
+        <v>110.5166666666667</v>
       </c>
       <c r="J23" t="n">
-        <v>4.584929596174282</v>
+        <v>4.890901788388311</v>
       </c>
       <c r="K23" t="n">
-        <v>1.627638888888889</v>
+        <v>1.841944444444444</v>
       </c>
       <c r="L23" t="n">
-        <v>22.97846262840949</v>
+        <v>20.29873572070338</v>
       </c>
       <c r="M23" t="n">
-        <v>8.683333333333334</v>
+        <v>7.35</v>
       </c>
       <c r="N23" t="n">
-        <v>0.3829743771401583</v>
+        <v>0.3383122620117229</v>
       </c>
       <c r="O23" t="n">
-        <v>0.1447222222222222</v>
+        <v>0.1225</v>
       </c>
     </row>
     <row r="24">
@@ -5608,43 +5608,43 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>88</v>
+        <v>119</v>
       </c>
       <c r="D24" t="n">
-        <v>4.358522727272727</v>
+        <v>3.526050420168068</v>
       </c>
       <c r="E24" t="n">
-        <v>2.283333333333333</v>
+        <v>1.85</v>
       </c>
       <c r="F24" t="n">
-        <v>0.07264204545454546</v>
+        <v>0.05876750700280112</v>
       </c>
       <c r="G24" t="n">
-        <v>0.03805555555555555</v>
+        <v>0.03083333333333333</v>
       </c>
       <c r="H24" t="n">
-        <v>233.2459770114943</v>
+        <v>206.0036796536797</v>
       </c>
       <c r="I24" t="n">
-        <v>13.425</v>
+        <v>12.98333333333333</v>
       </c>
       <c r="J24" t="n">
-        <v>3.887432950191571</v>
+        <v>3.433394660894661</v>
       </c>
       <c r="K24" t="n">
-        <v>0.22375</v>
+        <v>0.2163888888888889</v>
       </c>
       <c r="L24" t="n">
-        <v>227.6</v>
+        <v>201.3603896103896</v>
       </c>
       <c r="M24" t="n">
-        <v>10.575</v>
+        <v>10.31666666666667</v>
       </c>
       <c r="N24" t="n">
-        <v>3.793333333333333</v>
+        <v>3.356006493506493</v>
       </c>
       <c r="O24" t="n">
-        <v>0.17625</v>
+        <v>0.1719444444444444</v>
       </c>
     </row>
     <row r="25">
@@ -5659,43 +5659,43 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>143</v>
+        <v>190</v>
       </c>
       <c r="D25" t="n">
-        <v>325.7984848484849</v>
+        <v>307.6045614035088</v>
       </c>
       <c r="E25" t="n">
-        <v>19.63333333333333</v>
+        <v>19.58333333333334</v>
       </c>
       <c r="F25" t="n">
-        <v>5.429974747474748</v>
+        <v>5.12674269005848</v>
       </c>
       <c r="G25" t="n">
-        <v>0.3272222222222222</v>
+        <v>0.3263888888888889</v>
       </c>
       <c r="H25" t="n">
-        <v>329.7687793427231</v>
+        <v>312.7460992907802</v>
       </c>
       <c r="I25" t="n">
-        <v>27.78333333333333</v>
+        <v>25.1</v>
       </c>
       <c r="J25" t="n">
-        <v>5.496146322378717</v>
+        <v>5.212434988179669</v>
       </c>
       <c r="K25" t="n">
-        <v>0.4630555555555556</v>
+        <v>0.4183333333333333</v>
       </c>
       <c r="L25" t="n">
-        <v>10.43697183098591</v>
+        <v>8.521631205673758</v>
       </c>
       <c r="M25" t="n">
-        <v>2.058333333333334</v>
+        <v>1.991666666666667</v>
       </c>
       <c r="N25" t="n">
-        <v>0.1739495305164319</v>
+        <v>0.1420271867612293</v>
       </c>
       <c r="O25" t="n">
-        <v>0.03430555555555555</v>
+        <v>0.03319444444444444</v>
       </c>
     </row>
     <row r="26">
@@ -5710,19 +5710,19 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D26" t="n">
-        <v>5.28587962962963</v>
+        <v>4.942640692640692</v>
       </c>
       <c r="E26" t="n">
-        <v>1.558333333333333</v>
+        <v>1.466666666666667</v>
       </c>
       <c r="F26" t="n">
-        <v>0.08809799382716049</v>
+        <v>0.08237734487734487</v>
       </c>
       <c r="G26" t="n">
-        <v>0.02597222222222222</v>
+        <v>0.02444444444444444</v>
       </c>
       <c r="H26" t="n">
         <v>2062.413945578232</v>
@@ -5812,43 +5812,43 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>311</v>
+        <v>406</v>
       </c>
       <c r="D28" t="n">
-        <v>231.3711146838156</v>
+        <v>177.6495073891626</v>
       </c>
       <c r="E28" t="n">
-        <v>2.633333333333333</v>
+        <v>1.991666666666667</v>
       </c>
       <c r="F28" t="n">
-        <v>3.856185244730261</v>
+        <v>2.960825123152709</v>
       </c>
       <c r="G28" t="n">
-        <v>0.04388888888888889</v>
+        <v>0.03319444444444444</v>
       </c>
       <c r="H28" t="n">
-        <v>813.4525170068029</v>
+        <v>868.3449848024316</v>
       </c>
       <c r="I28" t="n">
-        <v>855.1833333333333</v>
+        <v>839.1333333333333</v>
       </c>
       <c r="J28" t="n">
-        <v>13.55754195011338</v>
+        <v>14.47241641337386</v>
       </c>
       <c r="K28" t="n">
-        <v>14.25305555555556</v>
+        <v>13.98555555555556</v>
       </c>
       <c r="L28" t="n">
-        <v>525.2495918367347</v>
+        <v>653.2248226950355</v>
       </c>
       <c r="M28" t="n">
-        <v>479.0166666666667</v>
+        <v>533.0166666666667</v>
       </c>
       <c r="N28" t="n">
-        <v>8.754159863945578</v>
+        <v>10.88708037825059</v>
       </c>
       <c r="O28" t="n">
-        <v>7.983611111111111</v>
+        <v>8.883611111111112</v>
       </c>
     </row>
     <row r="29">
@@ -5863,43 +5863,43 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>250</v>
+        <v>319</v>
       </c>
       <c r="D29" t="n">
-        <v>457.9451999999999</v>
+        <v>396.9627481713688</v>
       </c>
       <c r="E29" t="n">
-        <v>137.5416666666667</v>
+        <v>101.3166666666667</v>
       </c>
       <c r="F29" t="n">
-        <v>7.63242</v>
+        <v>6.616045802856148</v>
       </c>
       <c r="G29" t="n">
-        <v>2.292361111111111</v>
+        <v>1.688611111111111</v>
       </c>
       <c r="H29" t="n">
-        <v>915.1874163319947</v>
+        <v>912.8494708994708</v>
       </c>
       <c r="I29" t="n">
-        <v>930.5833333333334</v>
+        <v>903.3166666666667</v>
       </c>
       <c r="J29" t="n">
-        <v>15.25312360553324</v>
+        <v>15.21415784832451</v>
       </c>
       <c r="K29" t="n">
-        <v>15.50972222222222</v>
+        <v>15.05527777777778</v>
       </c>
       <c r="L29" t="n">
-        <v>456.0690763052209</v>
+        <v>515.9643915343916</v>
       </c>
       <c r="M29" t="n">
-        <v>163.2</v>
+        <v>187.9833333333333</v>
       </c>
       <c r="N29" t="n">
-        <v>7.601151271753681</v>
+        <v>8.599406525573194</v>
       </c>
       <c r="O29" t="n">
-        <v>2.72</v>
+        <v>3.133055555555555</v>
       </c>
     </row>
     <row r="30">
@@ -5914,43 +5914,43 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>4438</v>
+        <v>6055</v>
       </c>
       <c r="D30" t="n">
-        <v>6.287738470782635</v>
+        <v>5.020239471511148</v>
       </c>
       <c r="E30" t="n">
-        <v>2.25</v>
+        <v>1.883333333333333</v>
       </c>
       <c r="F30" t="n">
-        <v>0.1047956411797106</v>
+        <v>0.08367065785851913</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0375</v>
+        <v>0.03138888888888889</v>
       </c>
       <c r="H30" t="n">
-        <v>275.35937919914</v>
+        <v>298.2195666404818</v>
       </c>
       <c r="I30" t="n">
-        <v>100.7333333333333</v>
+        <v>116.9583333333333</v>
       </c>
       <c r="J30" t="n">
-        <v>4.589322986652334</v>
+        <v>4.970326110674697</v>
       </c>
       <c r="K30" t="n">
-        <v>1.678888888888889</v>
+        <v>1.949305555555555</v>
       </c>
       <c r="L30" t="n">
-        <v>267.9853130878796</v>
+        <v>292.3526184865148</v>
       </c>
       <c r="M30" t="n">
-        <v>97</v>
+        <v>111.975</v>
       </c>
       <c r="N30" t="n">
-        <v>4.466421884797993</v>
+        <v>4.872543641441913</v>
       </c>
       <c r="O30" t="n">
-        <v>1.616666666666667</v>
+        <v>1.86625</v>
       </c>
     </row>
     <row r="31">
@@ -5965,19 +5965,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2265</v>
+        <v>2287</v>
       </c>
       <c r="D31" t="n">
-        <v>2399.42233995585</v>
+        <v>2388.069661856872</v>
       </c>
       <c r="E31" t="n">
-        <v>2078.766666666667</v>
+        <v>2065.633333333333</v>
       </c>
       <c r="F31" t="n">
-        <v>39.9903723325975</v>
+        <v>39.80116103094787</v>
       </c>
       <c r="G31" t="n">
-        <v>34.64611111111112</v>
+        <v>34.42722222222222</v>
       </c>
       <c r="H31" t="n">
         <v>2719.90314232902</v>
@@ -5992,7 +5992,7 @@
         <v>39.92083333333333</v>
       </c>
       <c r="L31" t="n">
-        <v>315.5275955021564</v>
+        <v>315.5275955021565</v>
       </c>
       <c r="M31" t="n">
         <v>350.25</v>
@@ -6016,43 +6016,43 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>4689</v>
+        <v>6116</v>
       </c>
       <c r="D32" t="n">
-        <v>394.2848475154617</v>
+        <v>441.9897427512535</v>
       </c>
       <c r="E32" t="n">
-        <v>2.75</v>
+        <v>2.566666666666667</v>
       </c>
       <c r="F32" t="n">
-        <v>6.571414125257695</v>
+        <v>7.366495712520893</v>
       </c>
       <c r="G32" t="n">
-        <v>0.04583333333333333</v>
+        <v>0.04277777777777778</v>
       </c>
       <c r="H32" t="n">
-        <v>680.8264452152259</v>
+        <v>741.9601811965811</v>
       </c>
       <c r="I32" t="n">
-        <v>460.4833333333333</v>
+        <v>430.9166666666667</v>
       </c>
       <c r="J32" t="n">
-        <v>11.34710742025377</v>
+        <v>12.36600301994302</v>
       </c>
       <c r="K32" t="n">
-        <v>7.674722222222222</v>
+        <v>7.181944444444444</v>
       </c>
       <c r="L32" t="n">
-        <v>193.7567725008894</v>
+        <v>193.3965264957265</v>
       </c>
       <c r="M32" t="n">
-        <v>49.60833333333333</v>
+        <v>51.53333333333333</v>
       </c>
       <c r="N32" t="n">
-        <v>3.229279541681489</v>
+        <v>3.223275441595442</v>
       </c>
       <c r="O32" t="n">
-        <v>0.8268055555555556</v>
+        <v>0.8588888888888888</v>
       </c>
     </row>
     <row r="33">
@@ -6067,43 +6067,43 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4217</v>
+        <v>5355</v>
       </c>
       <c r="D33" t="n">
-        <v>524.9136550470319</v>
+        <v>568.2112138188609</v>
       </c>
       <c r="E33" t="n">
-        <v>162.3833333333333</v>
+        <v>163.2</v>
       </c>
       <c r="F33" t="n">
-        <v>8.748560917450531</v>
+        <v>9.470186896981016</v>
       </c>
       <c r="G33" t="n">
-        <v>2.706388888888889</v>
+        <v>2.72</v>
       </c>
       <c r="H33" t="n">
-        <v>744.4262180668948</v>
+        <v>795.264374173798</v>
       </c>
       <c r="I33" t="n">
-        <v>563.1833333333333</v>
+        <v>566.1833333333333</v>
       </c>
       <c r="J33" t="n">
-        <v>12.40710363444825</v>
+        <v>13.25440623622997</v>
       </c>
       <c r="K33" t="n">
-        <v>9.386388888888888</v>
+        <v>9.436388888888889</v>
       </c>
       <c r="L33" t="n">
-        <v>190.1863269247652</v>
+        <v>190.1371982188826</v>
       </c>
       <c r="M33" t="n">
-        <v>48.61666666666667</v>
+        <v>51.03333333333333</v>
       </c>
       <c r="N33" t="n">
-        <v>3.169772115412753</v>
+        <v>3.168953303648044</v>
       </c>
       <c r="O33" t="n">
-        <v>0.8102777777777778</v>
+        <v>0.8505555555555555</v>
       </c>
     </row>
     <row r="34">
@@ -6118,43 +6118,43 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1885</v>
+        <v>2308</v>
       </c>
       <c r="D34" t="n">
-        <v>1223.31658709107</v>
+        <v>1263.163272674754</v>
       </c>
       <c r="E34" t="n">
-        <v>911.1166666666667</v>
+        <v>906.5999999999999</v>
       </c>
       <c r="F34" t="n">
-        <v>20.38860978485116</v>
+        <v>21.05272121124591</v>
       </c>
       <c r="G34" t="n">
-        <v>15.18527777777778</v>
+        <v>15.11</v>
       </c>
       <c r="H34" t="n">
-        <v>1565.748784440843</v>
+        <v>1498.737374128583</v>
       </c>
       <c r="I34" t="n">
-        <v>1217.275</v>
+        <v>1190.9</v>
       </c>
       <c r="J34" t="n">
-        <v>26.09581307401405</v>
+        <v>24.97895623547637</v>
       </c>
       <c r="K34" t="n">
-        <v>20.28791666666667</v>
+        <v>19.84833333333334</v>
       </c>
       <c r="L34" t="n">
-        <v>378.1214613722312</v>
+        <v>363.4699457784663</v>
       </c>
       <c r="M34" t="n">
-        <v>437.1833333333333</v>
+        <v>437.1333333333333</v>
       </c>
       <c r="N34" t="n">
-        <v>6.302024356203853</v>
+        <v>6.057832429641104</v>
       </c>
       <c r="O34" t="n">
-        <v>7.286388888888889</v>
+        <v>7.285555555555556</v>
       </c>
     </row>
     <row r="35">
@@ -6169,43 +6169,43 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1853</v>
+        <v>2321</v>
       </c>
       <c r="D35" t="n">
-        <v>1505.343658931462</v>
+        <v>1506.567133419503</v>
       </c>
       <c r="E35" t="n">
-        <v>1048.533333333333</v>
+        <v>1013.666666666667</v>
       </c>
       <c r="F35" t="n">
-        <v>25.08906098219104</v>
+        <v>25.10945222365838</v>
       </c>
       <c r="G35" t="n">
-        <v>17.47555555555556</v>
+        <v>16.89444444444444</v>
       </c>
       <c r="H35" t="n">
-        <v>1828.769950124688</v>
+        <v>1748.829237947123</v>
       </c>
       <c r="I35" t="n">
-        <v>1448.966666666667</v>
+        <v>1370.8</v>
       </c>
       <c r="J35" t="n">
-        <v>30.47949916874481</v>
+        <v>29.14715396578539</v>
       </c>
       <c r="K35" t="n">
-        <v>24.14944444444444</v>
+        <v>22.84666666666667</v>
       </c>
       <c r="L35" t="n">
-        <v>381.515599889166</v>
+        <v>363.0080093312597</v>
       </c>
       <c r="M35" t="n">
-        <v>437.1666666666667</v>
+        <v>399.925</v>
       </c>
       <c r="N35" t="n">
-        <v>6.3585933314861</v>
+        <v>6.050133488854329</v>
       </c>
       <c r="O35" t="n">
-        <v>7.286111111111111</v>
+        <v>6.665416666666666</v>
       </c>
     </row>
     <row r="36">
@@ -6220,43 +6220,43 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>441</v>
+        <v>488</v>
       </c>
       <c r="D36" t="n">
-        <v>6.653061224489795</v>
+        <v>6.110382513661201</v>
       </c>
       <c r="E36" t="n">
-        <v>1.8</v>
+        <v>1.716666666666667</v>
       </c>
       <c r="F36" t="n">
-        <v>0.1108843537414966</v>
+        <v>0.10183970856102</v>
       </c>
       <c r="G36" t="n">
-        <v>0.03</v>
+        <v>0.02861111111111111</v>
       </c>
       <c r="H36" t="n">
-        <v>1127.888141025641</v>
+        <v>1072.92518115942</v>
       </c>
       <c r="I36" t="n">
-        <v>1187.741666666667</v>
+        <v>1154.15</v>
       </c>
       <c r="J36" t="n">
-        <v>18.79813568376069</v>
+        <v>17.88208635265701</v>
       </c>
       <c r="K36" t="n">
-        <v>19.79569444444444</v>
+        <v>19.23583333333333</v>
       </c>
       <c r="L36" t="n">
-        <v>1117.468461538462</v>
+        <v>1062.995531400966</v>
       </c>
       <c r="M36" t="n">
-        <v>1183.9</v>
+        <v>1150.308333333333</v>
       </c>
       <c r="N36" t="n">
-        <v>18.62447435897436</v>
+        <v>17.7165921900161</v>
       </c>
       <c r="O36" t="n">
-        <v>19.73166666666667</v>
+        <v>19.17180555555556</v>
       </c>
     </row>
     <row r="37">
@@ -6271,43 +6271,43 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>423</v>
+        <v>441</v>
       </c>
       <c r="D37" t="n">
-        <v>3711.479078014184</v>
+        <v>3563.801965230537</v>
       </c>
       <c r="E37" t="n">
-        <v>3594.85</v>
+        <v>2929.883333333333</v>
       </c>
       <c r="F37" t="n">
-        <v>61.85798463356974</v>
+        <v>59.39669942050894</v>
       </c>
       <c r="G37" t="n">
-        <v>59.91416666666667</v>
+        <v>48.83138888888889</v>
       </c>
       <c r="H37" t="n">
-        <v>4214.574083546462</v>
+        <v>4119.318204488778</v>
       </c>
       <c r="I37" t="n">
-        <v>4370.65</v>
+        <v>4314.4</v>
       </c>
       <c r="J37" t="n">
-        <v>70.24290139244103</v>
+        <v>68.6553034081463</v>
       </c>
       <c r="K37" t="n">
-        <v>72.84416666666667</v>
+        <v>71.90666666666667</v>
       </c>
       <c r="L37" t="n">
-        <v>235.9774083546462</v>
+        <v>237.6677888611804</v>
       </c>
       <c r="M37" t="n">
-        <v>238.5666666666667</v>
+        <v>235.75</v>
       </c>
       <c r="N37" t="n">
-        <v>3.932956805910769</v>
+        <v>3.961129814353006</v>
       </c>
       <c r="O37" t="n">
-        <v>3.976111111111111</v>
+        <v>3.929166666666667</v>
       </c>
     </row>
     <row r="38">
@@ -6322,43 +6322,43 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>554</v>
+        <v>728</v>
       </c>
       <c r="D38" t="n">
-        <v>3.376865222623346</v>
+        <v>2.844665750915751</v>
       </c>
       <c r="E38" t="n">
-        <v>1.808333333333333</v>
+        <v>1.716666666666667</v>
       </c>
       <c r="F38" t="n">
-        <v>0.05628108704372242</v>
+        <v>0.04741109584859585</v>
       </c>
       <c r="G38" t="n">
-        <v>0.03013888888888889</v>
+        <v>0.02861111111111111</v>
       </c>
       <c r="H38" t="n">
-        <v>494.613768115942</v>
+        <v>487.3917133956386</v>
       </c>
       <c r="I38" t="n">
-        <v>425.3916666666667</v>
+        <v>421.75</v>
       </c>
       <c r="J38" t="n">
-        <v>8.243562801932367</v>
+        <v>8.123195223260643</v>
       </c>
       <c r="K38" t="n">
-        <v>7.089861111111111</v>
+        <v>7.029166666666667</v>
       </c>
       <c r="L38" t="n">
-        <v>490.2009661835749</v>
+        <v>483.6088785046729</v>
       </c>
       <c r="M38" t="n">
-        <v>423.075</v>
+        <v>419.3833333333333</v>
       </c>
       <c r="N38" t="n">
-        <v>8.170016103059581</v>
+        <v>8.060147975077882</v>
       </c>
       <c r="O38" t="n">
-        <v>7.05125</v>
+        <v>6.989722222222222</v>
       </c>
     </row>
     <row r="39">
@@ -6373,43 +6373,43 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>573</v>
+        <v>796</v>
       </c>
       <c r="D39" t="n">
-        <v>209.3271087841769</v>
+        <v>203.6789572864322</v>
       </c>
       <c r="E39" t="n">
-        <v>70.71666666666667</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="F39" t="n">
-        <v>3.488785146402948</v>
+        <v>3.394649288107203</v>
       </c>
       <c r="G39" t="n">
-        <v>1.178611111111111</v>
+        <v>1.256666666666667</v>
       </c>
       <c r="H39" t="n">
-        <v>700.2947954271962</v>
+        <v>674.4561985262245</v>
       </c>
       <c r="I39" t="n">
-        <v>666.45</v>
+        <v>639.6333333333333</v>
       </c>
       <c r="J39" t="n">
-        <v>11.6715799237866</v>
+        <v>11.24093664210374</v>
       </c>
       <c r="K39" t="n">
-        <v>11.1075</v>
+        <v>10.66055555555556</v>
       </c>
       <c r="L39" t="n">
-        <v>488.8802948255114</v>
+        <v>469.6657563935847</v>
       </c>
       <c r="M39" t="n">
-        <v>311.5333333333333</v>
+        <v>302.5833333333333</v>
       </c>
       <c r="N39" t="n">
-        <v>8.148004913758523</v>
+        <v>7.827762606559746</v>
       </c>
       <c r="O39" t="n">
-        <v>5.192222222222222</v>
+        <v>5.043055555555555</v>
       </c>
     </row>
     <row r="40">
@@ -6424,40 +6424,40 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>19789</v>
+        <v>27814</v>
       </c>
       <c r="D40" t="n">
-        <v>42.78900820321054</v>
+        <v>50.04443026293713</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>1.833333333333333</v>
       </c>
       <c r="F40" t="n">
-        <v>0.7131501367201756</v>
+        <v>0.8340738377156188</v>
       </c>
       <c r="G40" t="n">
-        <v>0.03333333333333333</v>
+        <v>0.03055555555555555</v>
       </c>
       <c r="H40" t="n">
-        <v>63.28917757249166</v>
+        <v>76.69005151320026</v>
       </c>
       <c r="I40" t="n">
-        <v>2.65</v>
+        <v>2.216666666666667</v>
       </c>
       <c r="J40" t="n">
-        <v>1.054819626208195</v>
+        <v>1.278167525220004</v>
       </c>
       <c r="K40" t="n">
-        <v>0.04416666666666667</v>
+        <v>0.03694444444444445</v>
       </c>
       <c r="L40" t="n">
-        <v>10.4029606107262</v>
+        <v>14.25813172661209</v>
       </c>
       <c r="M40" t="n">
         <v>0.2333333333333333</v>
       </c>
       <c r="N40" t="n">
-        <v>0.1733826768454367</v>
+        <v>0.2376355287768681</v>
       </c>
       <c r="O40" t="n">
         <v>0.003888888888888889</v>
@@ -6475,43 +6475,43 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>6175</v>
+        <v>6854</v>
       </c>
       <c r="D41" t="n">
-        <v>837.8131848852902</v>
+        <v>865.0610373504522</v>
       </c>
       <c r="E41" t="n">
-        <v>758.0833333333334</v>
+        <v>791.2083333333334</v>
       </c>
       <c r="F41" t="n">
-        <v>13.9635530814215</v>
+        <v>14.41768395584087</v>
       </c>
       <c r="G41" t="n">
-        <v>12.63472222222222</v>
+        <v>13.18680555555556</v>
       </c>
       <c r="H41" t="n">
-        <v>892.2253652280584</v>
+        <v>922.7099593495934</v>
       </c>
       <c r="I41" t="n">
-        <v>813.6416666666667</v>
+        <v>839.9166666666666</v>
       </c>
       <c r="J41" t="n">
-        <v>14.87042275380097</v>
+        <v>15.37849932249322</v>
       </c>
       <c r="K41" t="n">
-        <v>13.56069444444444</v>
+        <v>13.99861111111111</v>
       </c>
       <c r="L41" t="n">
-        <v>47.41918423106947</v>
+        <v>50.42740138512496</v>
       </c>
       <c r="M41" t="n">
-        <v>41.975</v>
+        <v>42.05</v>
       </c>
       <c r="N41" t="n">
-        <v>0.7903197371844912</v>
+        <v>0.8404566897520828</v>
       </c>
       <c r="O41" t="n">
-        <v>0.6995833333333333</v>
+        <v>0.7008333333333333</v>
       </c>
     </row>
     <row r="42">
@@ -6526,43 +6526,43 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>41652</v>
+        <v>58084</v>
       </c>
       <c r="D42" t="n">
-        <v>4.700954736067096</v>
+        <v>3.86301735417671</v>
       </c>
       <c r="E42" t="n">
-        <v>2.3</v>
+        <v>1.916666666666667</v>
       </c>
       <c r="F42" t="n">
-        <v>0.07834924560111828</v>
+        <v>0.06438362256961183</v>
       </c>
       <c r="G42" t="n">
-        <v>0.03833333333333333</v>
+        <v>0.03194444444444445</v>
       </c>
       <c r="H42" t="n">
-        <v>328.1241875116349</v>
+        <v>355.0888420809345</v>
       </c>
       <c r="I42" t="n">
-        <v>157.0833333333333</v>
+        <v>152.0166666666667</v>
       </c>
       <c r="J42" t="n">
-        <v>5.46873645852725</v>
+        <v>5.918147368015576</v>
       </c>
       <c r="K42" t="n">
-        <v>2.618055555555556</v>
+        <v>2.533611111111111</v>
       </c>
       <c r="L42" t="n">
-        <v>322.9746421328003</v>
+        <v>350.8898148926335</v>
       </c>
       <c r="M42" t="n">
-        <v>153.1666666666667</v>
+        <v>148.925</v>
       </c>
       <c r="N42" t="n">
-        <v>5.382910702213339</v>
+        <v>5.848163581543892</v>
       </c>
       <c r="O42" t="n">
-        <v>2.552777777777778</v>
+        <v>2.482083333333333</v>
       </c>
     </row>
     <row r="43">
@@ -6577,43 +6577,43 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>25076</v>
+        <v>35054</v>
       </c>
       <c r="D43" t="n">
-        <v>186.422750172808</v>
+        <v>179.2518994503718</v>
       </c>
       <c r="E43" t="n">
-        <v>97.59999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="F43" t="n">
-        <v>3.107045836213467</v>
+        <v>2.987531657506196</v>
       </c>
       <c r="G43" t="n">
-        <v>1.626666666666666</v>
+        <v>1.578333333333333</v>
       </c>
       <c r="H43" t="n">
-        <v>442.9232868705701</v>
+        <v>476.3966606230252</v>
       </c>
       <c r="I43" t="n">
-        <v>248.95</v>
+        <v>238.8416666666667</v>
       </c>
       <c r="J43" t="n">
-        <v>7.382054781176169</v>
+        <v>7.939944343717087</v>
       </c>
       <c r="K43" t="n">
-        <v>4.149166666666667</v>
+        <v>3.980694444444445</v>
       </c>
       <c r="L43" t="n">
-        <v>261.4122342078394</v>
+        <v>301.3248409568039</v>
       </c>
       <c r="M43" t="n">
-        <v>104.1666666666667</v>
+        <v>101.3416666666667</v>
       </c>
       <c r="N43" t="n">
-        <v>4.356870570130658</v>
+        <v>5.022080682613398</v>
       </c>
       <c r="O43" t="n">
-        <v>1.736111111111111</v>
+        <v>1.689027777777778</v>
       </c>
     </row>
     <row r="44">
@@ -6628,43 +6628,43 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>5082</v>
+        <v>6610</v>
       </c>
       <c r="D44" t="n">
-        <v>5.300721500721502</v>
+        <v>4.45160363086233</v>
       </c>
       <c r="E44" t="n">
-        <v>2.366666666666667</v>
+        <v>1.983333333333333</v>
       </c>
       <c r="F44" t="n">
-        <v>0.08834535834535835</v>
+        <v>0.0741933938477055</v>
       </c>
       <c r="G44" t="n">
-        <v>0.03944444444444444</v>
+        <v>0.03305555555555555</v>
       </c>
       <c r="H44" t="n">
-        <v>749.6880664652568</v>
+        <v>799.7591884161602</v>
       </c>
       <c r="I44" t="n">
-        <v>730.5833333333334</v>
+        <v>816.8833333333333</v>
       </c>
       <c r="J44" t="n">
-        <v>12.49480110775428</v>
+        <v>13.329319806936</v>
       </c>
       <c r="K44" t="n">
-        <v>12.17638888888889</v>
+        <v>13.61472222222222</v>
       </c>
       <c r="L44" t="n">
-        <v>743.6155666589202</v>
+        <v>794.6534203313074</v>
       </c>
       <c r="M44" t="n">
-        <v>718.9</v>
+        <v>794.8</v>
       </c>
       <c r="N44" t="n">
-        <v>12.39359277764867</v>
+        <v>13.24422367218845</v>
       </c>
       <c r="O44" t="n">
-        <v>11.98166666666667</v>
+        <v>13.24666666666667</v>
       </c>
     </row>
     <row r="45">
@@ -6679,43 +6679,43 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>5836</v>
+        <v>7706</v>
       </c>
       <c r="D45" t="n">
-        <v>253.6480865889879</v>
+        <v>241.4909096807683</v>
       </c>
       <c r="E45" t="n">
-        <v>60.75833333333333</v>
+        <v>52.75</v>
       </c>
       <c r="F45" t="n">
-        <v>4.227468109816464</v>
+        <v>4.024848494679471</v>
       </c>
       <c r="G45" t="n">
-        <v>1.012638888888889</v>
+        <v>0.8791666666666667</v>
       </c>
       <c r="H45" t="n">
-        <v>892.3451599476751</v>
+        <v>933.6757616729764</v>
       </c>
       <c r="I45" t="n">
-        <v>864.3666666666667</v>
+        <v>939.8666666666667</v>
       </c>
       <c r="J45" t="n">
-        <v>14.87241933246125</v>
+        <v>15.5612626945496</v>
       </c>
       <c r="K45" t="n">
-        <v>14.40611111111111</v>
+        <v>15.66444444444445</v>
       </c>
       <c r="L45" t="n">
-        <v>639.42041859912</v>
+        <v>693.1163714620516</v>
       </c>
       <c r="M45" t="n">
-        <v>486.4583333333334</v>
+        <v>511.9583333333333</v>
       </c>
       <c r="N45" t="n">
-        <v>10.657006976652</v>
+        <v>11.55193952436753</v>
       </c>
       <c r="O45" t="n">
-        <v>8.107638888888889</v>
+        <v>8.53263888888889</v>
       </c>
     </row>
     <row r="46">
@@ -6730,43 +6730,43 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>410</v>
+        <v>454</v>
       </c>
       <c r="D46" t="n">
-        <v>1.844634146341463</v>
+        <v>1.718795888399413</v>
       </c>
       <c r="E46" t="n">
-        <v>1.783333333333333</v>
+        <v>1.716666666666667</v>
       </c>
       <c r="F46" t="n">
-        <v>0.03074390243902439</v>
+        <v>0.02864659813999021</v>
       </c>
       <c r="G46" t="n">
-        <v>0.02972222222222222</v>
+        <v>0.02861111111111111</v>
       </c>
       <c r="H46" t="n">
-        <v>1978.26329588015</v>
+        <v>1936.881588447653</v>
       </c>
       <c r="I46" t="n">
-        <v>2088.65</v>
+        <v>2066.466666666667</v>
       </c>
       <c r="J46" t="n">
-        <v>32.97105493133584</v>
+        <v>32.28135980746089</v>
       </c>
       <c r="K46" t="n">
-        <v>34.81083333333333</v>
+        <v>34.44111111111111</v>
       </c>
       <c r="L46" t="n">
-        <v>1976.041947565543</v>
+        <v>1934.677858002407</v>
       </c>
       <c r="M46" t="n">
-        <v>2087.2</v>
+        <v>2064.566666666667</v>
       </c>
       <c r="N46" t="n">
-        <v>32.93403245942572</v>
+        <v>32.24463096670678</v>
       </c>
       <c r="O46" t="n">
-        <v>34.78666666666666</v>
+        <v>34.40944444444445</v>
       </c>
     </row>
     <row r="47">
@@ -6781,43 +6781,43 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>321</v>
+        <v>346</v>
       </c>
       <c r="D47" t="n">
-        <v>349.8322429906542</v>
+        <v>333.0520231213873</v>
       </c>
       <c r="E47" t="n">
-        <v>226.4166666666667</v>
+        <v>152.4583333333333</v>
       </c>
       <c r="F47" t="n">
-        <v>5.83053738317757</v>
+        <v>5.550867052023122</v>
       </c>
       <c r="G47" t="n">
-        <v>3.773611111111111</v>
+        <v>2.540972222222222</v>
       </c>
       <c r="H47" t="n">
-        <v>2061.298761261261</v>
+        <v>1983.986612903226</v>
       </c>
       <c r="I47" t="n">
-        <v>2319.916666666667</v>
+        <v>2267.308333333333</v>
       </c>
       <c r="J47" t="n">
-        <v>34.35497935435435</v>
+        <v>33.0664435483871</v>
       </c>
       <c r="K47" t="n">
-        <v>38.66527777777777</v>
+        <v>37.78847222222223</v>
       </c>
       <c r="L47" t="n">
-        <v>1703.817060810811</v>
+        <v>1636.380967741936</v>
       </c>
       <c r="M47" t="n">
-        <v>1772.75</v>
+        <v>1768.725</v>
       </c>
       <c r="N47" t="n">
-        <v>28.39695101351351</v>
+        <v>27.27301612903226</v>
       </c>
       <c r="O47" t="n">
-        <v>29.54583333333333</v>
+        <v>29.47875</v>
       </c>
     </row>
     <row r="48">
@@ -6832,43 +6832,43 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2327</v>
+        <v>3089</v>
       </c>
       <c r="D48" t="n">
-        <v>4.991877954447786</v>
+        <v>4.139003992662134</v>
       </c>
       <c r="E48" t="n">
-        <v>2.266666666666667</v>
+        <v>1.916666666666667</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0831979659074631</v>
+        <v>0.06898339987770225</v>
       </c>
       <c r="G48" t="n">
-        <v>0.03777777777777778</v>
+        <v>0.03194444444444445</v>
       </c>
       <c r="H48" t="n">
-        <v>458.702861952862</v>
+        <v>460.4456556082148</v>
       </c>
       <c r="I48" t="n">
-        <v>431.8</v>
+        <v>388.8166666666667</v>
       </c>
       <c r="J48" t="n">
-        <v>7.645047699214366</v>
+        <v>7.674094260136914</v>
       </c>
       <c r="K48" t="n">
-        <v>7.196666666666667</v>
+        <v>6.480277777777777</v>
       </c>
       <c r="L48" t="n">
-        <v>453.1417187750521</v>
+        <v>455.8080325677482</v>
       </c>
       <c r="M48" t="n">
-        <v>423.05</v>
+        <v>382.5833333333333</v>
       </c>
       <c r="N48" t="n">
-        <v>7.552361979584202</v>
+        <v>7.596800542795805</v>
       </c>
       <c r="O48" t="n">
-        <v>7.050833333333333</v>
+        <v>6.376388888888888</v>
       </c>
     </row>
     <row r="49">
@@ -6883,43 +6883,43 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1046</v>
+        <v>1287</v>
       </c>
       <c r="D49" t="n">
-        <v>321.2919056724028</v>
+        <v>299.5193732193732</v>
       </c>
       <c r="E49" t="n">
-        <v>93.60833333333333</v>
+        <v>96.76666666666667</v>
       </c>
       <c r="F49" t="n">
-        <v>5.354865094540047</v>
+        <v>4.99198955365622</v>
       </c>
       <c r="G49" t="n">
-        <v>1.560138888888889</v>
+        <v>1.612777777777778</v>
       </c>
       <c r="H49" t="n">
-        <v>745.5879129865882</v>
+        <v>729.1852118305355</v>
       </c>
       <c r="I49" t="n">
-        <v>594.9</v>
+        <v>591.75</v>
       </c>
       <c r="J49" t="n">
-        <v>12.42646521644314</v>
+        <v>12.15308686384226</v>
       </c>
       <c r="K49" t="n">
-        <v>9.914999999999999</v>
+        <v>9.862500000000001</v>
       </c>
       <c r="L49" t="n">
-        <v>424.0026005888126</v>
+        <v>429.4550093258727</v>
       </c>
       <c r="M49" t="n">
-        <v>276.6833333333333</v>
+        <v>265.9833333333333</v>
       </c>
       <c r="N49" t="n">
-        <v>7.066710009813542</v>
+        <v>7.157583488764544</v>
       </c>
       <c r="O49" t="n">
-        <v>4.611388888888889</v>
+        <v>4.433055555555556</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion automatica dashboard mié 23/09/2026 15:09:28,97
</commit_message>
<xml_diff>
--- a/Reporte_Efectividad_Automatizacion.xlsx
+++ b/Reporte_Efectividad_Automatizacion.xlsx
@@ -696,19 +696,19 @@
         <v>71.65194435983349</v>
       </c>
       <c r="Z2" t="n">
-        <v>4144</v>
+        <v>5075</v>
       </c>
       <c r="AA2" t="n">
-        <v>36.46235521235521</v>
+        <v>37.2807881773399</v>
       </c>
       <c r="AB2" t="n">
-        <v>69.73938223938224</v>
+        <v>69.63546798029556</v>
       </c>
       <c r="AC2" t="n">
-        <v>10.76431480216128</v>
+        <v>11.58274776714597</v>
       </c>
       <c r="AD2" t="n">
-        <v>-57.92466240227434</v>
+        <v>-48.47192608386639</v>
       </c>
     </row>
     <row r="3">
@@ -790,19 +790,19 @@
         <v>79.51807228915662</v>
       </c>
       <c r="Z3" t="n">
-        <v>309</v>
+        <v>360</v>
       </c>
       <c r="AA3" t="n">
-        <v>38.51132686084142</v>
+        <v>39.16666666666666</v>
       </c>
       <c r="AB3" t="n">
-        <v>80.90614886731392</v>
+        <v>80.27777777777779</v>
       </c>
       <c r="AC3" t="n">
-        <v>12.69377092280356</v>
+        <v>13.3491107286288</v>
       </c>
       <c r="AD3" t="n">
-        <v>-46.815834767642</v>
+        <v>-38.03786574870912</v>
       </c>
     </row>
     <row r="4">
@@ -884,19 +884,19 @@
         <v>62.42171189979123</v>
       </c>
       <c r="Z4" t="n">
-        <v>108</v>
+        <v>136</v>
       </c>
       <c r="AA4" t="n">
-        <v>71.29629629629629</v>
+        <v>70.58823529411765</v>
       </c>
       <c r="AB4" t="n">
-        <v>76.85185185185185</v>
+        <v>75</v>
       </c>
       <c r="AC4" t="n">
-        <v>52.71592051341528</v>
+        <v>52.00785951123665</v>
       </c>
       <c r="AD4" t="n">
-        <v>-77.45302713987473</v>
+        <v>-71.60751565762004</v>
       </c>
     </row>
     <row r="5">
@@ -978,19 +978,19 @@
         <v>62.37424547283702</v>
       </c>
       <c r="Z5" t="n">
-        <v>725</v>
+        <v>846</v>
       </c>
       <c r="AA5" t="n">
-        <v>56.00000000000001</v>
+        <v>56.97399527186762</v>
       </c>
       <c r="AB5" t="n">
-        <v>59.72413793103448</v>
+        <v>60.87470449172577</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.2655935613682203</v>
+        <v>1.239588833235828</v>
       </c>
       <c r="AD5" t="n">
-        <v>-63.53118712273642</v>
+        <v>-57.4446680080483</v>
       </c>
     </row>
     <row r="6">
@@ -1072,19 +1072,19 @@
         <v>82.54543623823189</v>
       </c>
       <c r="Z6" t="n">
-        <v>8342</v>
+        <v>10435</v>
       </c>
       <c r="AA6" t="n">
-        <v>72.5845121074083</v>
+        <v>68.00191662673694</v>
       </c>
       <c r="AB6" t="n">
-        <v>76.66027331575161</v>
+        <v>73.01389554384284</v>
       </c>
       <c r="AC6" t="n">
-        <v>-6.482094145423588</v>
+        <v>-11.06468962609495</v>
       </c>
       <c r="AD6" t="n">
-        <v>-58.00231586366611</v>
+        <v>-47.46513618285254</v>
       </c>
     </row>
     <row r="7">
@@ -1166,19 +1166,19 @@
         <v>64.37949170915806</v>
       </c>
       <c r="Z7" t="n">
-        <v>11471</v>
+        <v>13716</v>
       </c>
       <c r="AA7" t="n">
-        <v>53.31706041321593</v>
+        <v>52.92359288422281</v>
       </c>
       <c r="AB7" t="n">
-        <v>65.53046813704123</v>
+        <v>64.80752405949256</v>
       </c>
       <c r="AC7" t="n">
-        <v>8.819529598585511</v>
+        <v>8.426062069592383</v>
       </c>
       <c r="AD7" t="n">
-        <v>-53.94467418797928</v>
+        <v>-44.93114385514112</v>
       </c>
     </row>
     <row r="8">
@@ -1260,19 +1260,19 @@
         <v>63.24499030381383</v>
       </c>
       <c r="Z8" t="n">
-        <v>4629</v>
+        <v>5582</v>
       </c>
       <c r="AA8" t="n">
-        <v>49.85958090300281</v>
+        <v>50.71658903618774</v>
       </c>
       <c r="AB8" t="n">
-        <v>58.6951825448261</v>
+        <v>59.22608384091723</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.4478161971204528</v>
+        <v>1.304824330305387</v>
       </c>
       <c r="AD8" t="n">
-        <v>-40.15513897866839</v>
+        <v>-27.83451842275372</v>
       </c>
     </row>
     <row r="9">
@@ -1354,19 +1354,19 @@
         <v>78.380257212374</v>
       </c>
       <c r="Z9" t="n">
-        <v>929</v>
+        <v>1182</v>
       </c>
       <c r="AA9" t="n">
-        <v>52.52960172228202</v>
+        <v>49.66159052453469</v>
       </c>
       <c r="AB9" t="n">
-        <v>59.95694294940797</v>
+        <v>57.1912013536379</v>
       </c>
       <c r="AC9" t="n">
-        <v>-20.35882372088794</v>
+        <v>-23.22683491863528</v>
       </c>
       <c r="AD9" t="n">
-        <v>-67.70941953423704</v>
+        <v>-58.91553701772679</v>
       </c>
     </row>
     <row r="10">
@@ -1448,19 +1448,19 @@
         <v>54.65631929046562</v>
       </c>
       <c r="Z10" t="n">
-        <v>1524</v>
+        <v>1872</v>
       </c>
       <c r="AA10" t="n">
-        <v>47.76902887139108</v>
+        <v>47.86324786324786</v>
       </c>
       <c r="AB10" t="n">
-        <v>54.92125984251969</v>
+        <v>55.12820512820513</v>
       </c>
       <c r="AC10" t="n">
-        <v>14.28787587804296</v>
+        <v>14.38209486989975</v>
       </c>
       <c r="AD10" t="n">
-        <v>-43.68070953436807</v>
+        <v>-30.82039911308204</v>
       </c>
     </row>
     <row r="11">
@@ -1542,19 +1542,19 @@
         <v>81.92520288611654</v>
       </c>
       <c r="Z11" t="n">
-        <v>34668</v>
+        <v>40871</v>
       </c>
       <c r="AA11" t="n">
-        <v>80.2296065535941</v>
+        <v>76.31083164101686</v>
       </c>
       <c r="AB11" t="n">
-        <v>82.62086073612554</v>
+        <v>79.62369406180422</v>
       </c>
       <c r="AC11" t="n">
-        <v>1.819221034810425</v>
+        <v>-2.099553877766809</v>
       </c>
       <c r="AD11" t="n">
-        <v>-51.23982053193434</v>
+        <v>-42.51536589825455</v>
       </c>
     </row>
     <row r="12">
@@ -1636,19 +1636,19 @@
         <v>79.3433378990412</v>
       </c>
       <c r="Z12" t="n">
-        <v>93138</v>
+        <v>111489</v>
       </c>
       <c r="AA12" t="n">
-        <v>62.36337477721231</v>
+        <v>61.73703235296756</v>
       </c>
       <c r="AB12" t="n">
-        <v>77.71800983486868</v>
+        <v>77.07755922108907</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.08895240591027687</v>
+        <v>-0.5373900183344702</v>
       </c>
       <c r="AD12" t="n">
-        <v>-53.44077743673829</v>
+        <v>-44.26720388718369</v>
       </c>
     </row>
     <row r="13">
@@ -1730,19 +1730,19 @@
         <v>67.14883504675311</v>
       </c>
       <c r="Z13" t="n">
-        <v>14316</v>
+        <v>19091</v>
       </c>
       <c r="AA13" t="n">
-        <v>46.17211511595418</v>
+        <v>46.93310984233408</v>
       </c>
       <c r="AB13" t="n">
-        <v>65.66778429728974</v>
+        <v>65.90540045047405</v>
       </c>
       <c r="AC13" t="n">
-        <v>3.309068156198016</v>
+        <v>4.070062882577922</v>
       </c>
       <c r="AD13" t="n">
-        <v>-63.02112930722736</v>
+        <v>-50.68708994162319</v>
       </c>
     </row>
     <row r="14">
@@ -1824,19 +1824,19 @@
         <v>72.04349796103308</v>
       </c>
       <c r="Z14" t="n">
-        <v>800</v>
+        <v>865</v>
       </c>
       <c r="AA14" t="n">
-        <v>56.75</v>
+        <v>58.72832369942197</v>
       </c>
       <c r="AB14" t="n">
-        <v>74</v>
+        <v>75.02890173410405</v>
       </c>
       <c r="AC14" t="n">
-        <v>8.018690530131401</v>
+        <v>9.997014229553372</v>
       </c>
       <c r="AD14" t="n">
-        <v>-81.87584956955143</v>
+        <v>-80.40326234707747</v>
       </c>
     </row>
     <row r="15">
@@ -1918,19 +1918,19 @@
         <v>78.43225419664267</v>
       </c>
       <c r="Z15" t="n">
-        <v>4376</v>
+        <v>5586</v>
       </c>
       <c r="AA15" t="n">
-        <v>70.58957952468006</v>
+        <v>69.90691013247404</v>
       </c>
       <c r="AB15" t="n">
-        <v>76.21115173674589</v>
+        <v>75.5281059792338</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.8578648963827078</v>
+        <v>0.1751955041766848</v>
       </c>
       <c r="AD15" t="n">
-        <v>-67.20623501199042</v>
+        <v>-58.13848920863309</v>
       </c>
     </row>
   </sheetData>
@@ -3851,19 +3851,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4024</v>
+        <v>5127</v>
       </c>
       <c r="C4" t="n">
-        <v>490</v>
+        <v>570</v>
       </c>
       <c r="D4" t="n">
-        <v>12.17693836978131</v>
+        <v>11.11761263897016</v>
       </c>
       <c r="E4" t="n">
-        <v>1470.57206122449</v>
+        <v>1277.931052631579</v>
       </c>
       <c r="F4" t="n">
-        <v>1584.896924165252</v>
+        <v>1590.569684002633</v>
       </c>
     </row>
     <row r="5">
@@ -3873,19 +3873,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>126762</v>
+        <v>150993</v>
       </c>
       <c r="C5" t="n">
-        <v>104586</v>
+        <v>123777</v>
       </c>
       <c r="D5" t="n">
-        <v>82.50579826761964</v>
+        <v>81.97532335936103</v>
       </c>
       <c r="E5" t="n">
-        <v>3525.8840265809</v>
+        <v>3535.703465781122</v>
       </c>
       <c r="F5" t="n">
-        <v>7913.708640827922</v>
+        <v>8756.25698409024</v>
       </c>
     </row>
     <row r="6">
@@ -3895,19 +3895,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>39499</v>
+        <v>50000</v>
       </c>
       <c r="C6" t="n">
-        <v>5463</v>
+        <v>6459</v>
       </c>
       <c r="D6" t="n">
-        <v>13.830729891896</v>
+        <v>12.918</v>
       </c>
       <c r="E6" t="n">
-        <v>9392.321089145158</v>
+        <v>10221.23078495123</v>
       </c>
       <c r="F6" t="n">
-        <v>4252.136308908215</v>
+        <v>4451.432756941733</v>
       </c>
     </row>
     <row r="7">
@@ -3917,19 +3917,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9194</v>
+        <v>10986</v>
       </c>
       <c r="C7" t="n">
-        <v>3320</v>
+        <v>3866</v>
       </c>
       <c r="D7" t="n">
-        <v>36.11050685229498</v>
+        <v>35.19024212634262</v>
       </c>
       <c r="E7" t="n">
-        <v>1585.639206325301</v>
+        <v>1511.938969218831</v>
       </c>
       <c r="F7" t="n">
-        <v>4614.78207524685</v>
+        <v>4548.612266853932</v>
       </c>
     </row>
     <row r="8"/>
@@ -5107,19 +5107,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4144</v>
+        <v>5075</v>
       </c>
       <c r="C4" t="n">
-        <v>1511</v>
+        <v>1892</v>
       </c>
       <c r="D4" t="n">
-        <v>36.46235521235521</v>
+        <v>37.2807881773399</v>
       </c>
       <c r="E4" t="n">
-        <v>2890</v>
+        <v>3534</v>
       </c>
       <c r="F4" t="n">
-        <v>69.73938223938224</v>
+        <v>69.63546798029556</v>
       </c>
     </row>
     <row r="5">
@@ -5129,19 +5129,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>309</v>
+        <v>360</v>
       </c>
       <c r="C5" t="n">
-        <v>119</v>
+        <v>141</v>
       </c>
       <c r="D5" t="n">
-        <v>38.51132686084142</v>
+        <v>39.16666666666666</v>
       </c>
       <c r="E5" t="n">
-        <v>250</v>
+        <v>289</v>
       </c>
       <c r="F5" t="n">
-        <v>80.90614886731392</v>
+        <v>80.27777777777779</v>
       </c>
     </row>
     <row r="6">
@@ -5151,19 +5151,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>108</v>
+        <v>136</v>
       </c>
       <c r="C6" t="n">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="D6" t="n">
-        <v>71.29629629629629</v>
+        <v>70.58823529411765</v>
       </c>
       <c r="E6" t="n">
-        <v>83</v>
+        <v>102</v>
       </c>
       <c r="F6" t="n">
-        <v>76.85185185185185</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7">
@@ -5173,19 +5173,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>725</v>
+        <v>846</v>
       </c>
       <c r="C7" t="n">
-        <v>406</v>
+        <v>482</v>
       </c>
       <c r="D7" t="n">
-        <v>56.00000000000001</v>
+        <v>56.97399527186762</v>
       </c>
       <c r="E7" t="n">
-        <v>433</v>
+        <v>515</v>
       </c>
       <c r="F7" t="n">
-        <v>59.72413793103448</v>
+        <v>60.87470449172577</v>
       </c>
     </row>
     <row r="8">
@@ -5195,19 +5195,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8342</v>
+        <v>10435</v>
       </c>
       <c r="C8" t="n">
-        <v>6055</v>
+        <v>7096</v>
       </c>
       <c r="D8" t="n">
-        <v>72.5845121074083</v>
+        <v>68.00191662673694</v>
       </c>
       <c r="E8" t="n">
-        <v>6395</v>
+        <v>7619</v>
       </c>
       <c r="F8" t="n">
-        <v>76.66027331575161</v>
+        <v>73.01389554384284</v>
       </c>
     </row>
     <row r="9">
@@ -5217,19 +5217,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11471</v>
+        <v>13716</v>
       </c>
       <c r="C9" t="n">
-        <v>6116</v>
+        <v>7259</v>
       </c>
       <c r="D9" t="n">
-        <v>53.31706041321593</v>
+        <v>52.92359288422281</v>
       </c>
       <c r="E9" t="n">
-        <v>7517</v>
+        <v>8889</v>
       </c>
       <c r="F9" t="n">
-        <v>65.53046813704123</v>
+        <v>64.80752405949256</v>
       </c>
     </row>
     <row r="10">
@@ -5239,19 +5239,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4629</v>
+        <v>5582</v>
       </c>
       <c r="C10" t="n">
-        <v>2308</v>
+        <v>2831</v>
       </c>
       <c r="D10" t="n">
-        <v>49.85958090300281</v>
+        <v>50.71658903618774</v>
       </c>
       <c r="E10" t="n">
-        <v>2717</v>
+        <v>3306</v>
       </c>
       <c r="F10" t="n">
-        <v>58.6951825448261</v>
+        <v>59.22608384091723</v>
       </c>
     </row>
     <row r="11">
@@ -5261,19 +5261,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>929</v>
+        <v>1182</v>
       </c>
       <c r="C11" t="n">
-        <v>488</v>
+        <v>587</v>
       </c>
       <c r="D11" t="n">
-        <v>52.52960172228202</v>
+        <v>49.66159052453469</v>
       </c>
       <c r="E11" t="n">
-        <v>557</v>
+        <v>676</v>
       </c>
       <c r="F11" t="n">
-        <v>59.95694294940797</v>
+        <v>57.1912013536379</v>
       </c>
     </row>
     <row r="12">
@@ -5283,19 +5283,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1524</v>
+        <v>1872</v>
       </c>
       <c r="C12" t="n">
-        <v>728</v>
+        <v>896</v>
       </c>
       <c r="D12" t="n">
-        <v>47.76902887139108</v>
+        <v>47.86324786324786</v>
       </c>
       <c r="E12" t="n">
-        <v>837</v>
+        <v>1032</v>
       </c>
       <c r="F12" t="n">
-        <v>54.92125984251969</v>
+        <v>55.12820512820513</v>
       </c>
     </row>
     <row r="13">
@@ -5305,19 +5305,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>34668</v>
+        <v>40871</v>
       </c>
       <c r="C13" t="n">
-        <v>27814</v>
+        <v>31189</v>
       </c>
       <c r="D13" t="n">
-        <v>80.2296065535941</v>
+        <v>76.31083164101686</v>
       </c>
       <c r="E13" t="n">
-        <v>28643</v>
+        <v>32543</v>
       </c>
       <c r="F13" t="n">
-        <v>82.62086073612554</v>
+        <v>79.62369406180422</v>
       </c>
     </row>
     <row r="14">
@@ -5327,19 +5327,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>93138</v>
+        <v>111489</v>
       </c>
       <c r="C14" t="n">
-        <v>58084</v>
+        <v>68830</v>
       </c>
       <c r="D14" t="n">
-        <v>62.36337477721231</v>
+        <v>61.73703235296756</v>
       </c>
       <c r="E14" t="n">
-        <v>72385</v>
+        <v>85933</v>
       </c>
       <c r="F14" t="n">
-        <v>77.71800983486868</v>
+        <v>77.07755922108907</v>
       </c>
     </row>
     <row r="15">
@@ -5349,19 +5349,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>14316</v>
+        <v>19091</v>
       </c>
       <c r="C15" t="n">
-        <v>6610</v>
+        <v>8960</v>
       </c>
       <c r="D15" t="n">
-        <v>46.17211511595418</v>
+        <v>46.93310984233408</v>
       </c>
       <c r="E15" t="n">
-        <v>9401</v>
+        <v>12582</v>
       </c>
       <c r="F15" t="n">
-        <v>65.66778429728974</v>
+        <v>65.90540045047405</v>
       </c>
     </row>
     <row r="16">
@@ -5371,19 +5371,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>800</v>
+        <v>865</v>
       </c>
       <c r="C16" t="n">
-        <v>454</v>
+        <v>508</v>
       </c>
       <c r="D16" t="n">
-        <v>56.75</v>
+        <v>58.72832369942197</v>
       </c>
       <c r="E16" t="n">
-        <v>592</v>
+        <v>649</v>
       </c>
       <c r="F16" t="n">
-        <v>74</v>
+        <v>75.02890173410405</v>
       </c>
     </row>
     <row r="17">
@@ -5393,19 +5393,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>4376</v>
+        <v>5586</v>
       </c>
       <c r="C17" t="n">
-        <v>3089</v>
+        <v>3905</v>
       </c>
       <c r="D17" t="n">
-        <v>70.58957952468006</v>
+        <v>69.90691013247404</v>
       </c>
       <c r="E17" t="n">
-        <v>3335</v>
+        <v>4219</v>
       </c>
       <c r="F17" t="n">
-        <v>76.21115173674589</v>
+        <v>75.5281059792338</v>
       </c>
     </row>
     <row r="18"/>
@@ -5506,43 +5506,43 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1511</v>
+        <v>1892</v>
       </c>
       <c r="D22" t="n">
-        <v>3.950838296933598</v>
+        <v>3.400924947145878</v>
       </c>
       <c r="E22" t="n">
-        <v>1.8</v>
+        <v>1.716666666666667</v>
       </c>
       <c r="F22" t="n">
-        <v>0.06584730494889329</v>
+        <v>0.05668208245243129</v>
       </c>
       <c r="G22" t="n">
-        <v>0.03</v>
+        <v>0.02861111111111111</v>
       </c>
       <c r="H22" t="n">
-        <v>211.7491827438371</v>
+        <v>217.0047048379938</v>
       </c>
       <c r="I22" t="n">
-        <v>79.26666666666667</v>
+        <v>79.425</v>
       </c>
       <c r="J22" t="n">
-        <v>3.529153045730618</v>
+        <v>3.61674508063323</v>
       </c>
       <c r="K22" t="n">
-        <v>1.321111111111111</v>
+        <v>1.32375</v>
       </c>
       <c r="L22" t="n">
-        <v>207.1934887459807</v>
+        <v>212.956269418553</v>
       </c>
       <c r="M22" t="n">
-        <v>73.97499999999999</v>
+        <v>75.05833333333334</v>
       </c>
       <c r="N22" t="n">
-        <v>3.453224812433012</v>
+        <v>3.549271156975884</v>
       </c>
       <c r="O22" t="n">
-        <v>1.232916666666667</v>
+        <v>1.250972222222222</v>
       </c>
     </row>
     <row r="23">
@@ -5557,43 +5557,43 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2633</v>
+        <v>3183</v>
       </c>
       <c r="D23" t="n">
-        <v>270.6461704013166</v>
+        <v>277.3046287569379</v>
       </c>
       <c r="E23" t="n">
-        <v>83.09999999999999</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F23" t="n">
-        <v>4.51076950668861</v>
+        <v>4.621743812615632</v>
       </c>
       <c r="G23" t="n">
-        <v>1.385</v>
+        <v>1.306666666666667</v>
       </c>
       <c r="H23" t="n">
-        <v>293.4541073032987</v>
+        <v>298.9027839643653</v>
       </c>
       <c r="I23" t="n">
-        <v>110.5166666666667</v>
+        <v>102.8333333333333</v>
       </c>
       <c r="J23" t="n">
-        <v>4.890901788388311</v>
+        <v>4.981713066072754</v>
       </c>
       <c r="K23" t="n">
-        <v>1.841944444444444</v>
+        <v>1.713888888888889</v>
       </c>
       <c r="L23" t="n">
-        <v>20.29873572070338</v>
+        <v>19.15384452221868</v>
       </c>
       <c r="M23" t="n">
-        <v>7.35</v>
+        <v>7.116666666666666</v>
       </c>
       <c r="N23" t="n">
-        <v>0.3383122620117229</v>
+        <v>0.3192307420369782</v>
       </c>
       <c r="O23" t="n">
-        <v>0.1225</v>
+        <v>0.1186111111111111</v>
       </c>
     </row>
     <row r="24">
@@ -5608,43 +5608,43 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>119</v>
+        <v>141</v>
       </c>
       <c r="D24" t="n">
-        <v>3.526050420168068</v>
+        <v>3.169385342789599</v>
       </c>
       <c r="E24" t="n">
-        <v>1.85</v>
+        <v>1.75</v>
       </c>
       <c r="F24" t="n">
-        <v>0.05876750700280112</v>
+        <v>0.0528230890464933</v>
       </c>
       <c r="G24" t="n">
-        <v>0.03083333333333333</v>
+        <v>0.02916666666666667</v>
       </c>
       <c r="H24" t="n">
-        <v>206.0036796536797</v>
+        <v>230.5644927536232</v>
       </c>
       <c r="I24" t="n">
-        <v>12.98333333333333</v>
+        <v>16.55</v>
       </c>
       <c r="J24" t="n">
-        <v>3.433394660894661</v>
+        <v>3.84274154589372</v>
       </c>
       <c r="K24" t="n">
-        <v>0.2163888888888889</v>
+        <v>0.2758333333333334</v>
       </c>
       <c r="L24" t="n">
-        <v>201.3603896103896</v>
+        <v>226.409420289855</v>
       </c>
       <c r="M24" t="n">
-        <v>10.31666666666667</v>
+        <v>14.025</v>
       </c>
       <c r="N24" t="n">
-        <v>3.356006493506493</v>
+        <v>3.773490338164252</v>
       </c>
       <c r="O24" t="n">
-        <v>0.1719444444444444</v>
+        <v>0.23375</v>
       </c>
     </row>
     <row r="25">
@@ -5659,43 +5659,43 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>190</v>
+        <v>219</v>
       </c>
       <c r="D25" t="n">
-        <v>307.6045614035088</v>
+        <v>316.8875951293759</v>
       </c>
       <c r="E25" t="n">
-        <v>19.58333333333334</v>
+        <v>19.53333333333333</v>
       </c>
       <c r="F25" t="n">
-        <v>5.12674269005848</v>
+        <v>5.281459918822932</v>
       </c>
       <c r="G25" t="n">
-        <v>0.3263888888888889</v>
+        <v>0.3255555555555556</v>
       </c>
       <c r="H25" t="n">
-        <v>312.7460992907802</v>
+        <v>320.6519113149847</v>
       </c>
       <c r="I25" t="n">
-        <v>25.1</v>
+        <v>24.1</v>
       </c>
       <c r="J25" t="n">
-        <v>5.212434988179669</v>
+        <v>5.344198521916413</v>
       </c>
       <c r="K25" t="n">
-        <v>0.4183333333333333</v>
+        <v>0.4016666666666666</v>
       </c>
       <c r="L25" t="n">
-        <v>8.521631205673758</v>
+        <v>8.017431192660549</v>
       </c>
       <c r="M25" t="n">
-        <v>1.991666666666667</v>
+        <v>2.1</v>
       </c>
       <c r="N25" t="n">
-        <v>0.1420271867612293</v>
+        <v>0.1336238532110092</v>
       </c>
       <c r="O25" t="n">
-        <v>0.03319444444444444</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="26">
@@ -5710,43 +5710,43 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="D26" t="n">
-        <v>4.942640692640692</v>
+        <v>4.1453125</v>
       </c>
       <c r="E26" t="n">
-        <v>1.466666666666667</v>
+        <v>1.433333333333333</v>
       </c>
       <c r="F26" t="n">
-        <v>0.08237734487734487</v>
+        <v>0.06908854166666667</v>
       </c>
       <c r="G26" t="n">
-        <v>0.02444444444444444</v>
+        <v>0.02388888888888889</v>
       </c>
       <c r="H26" t="n">
-        <v>2062.413945578232</v>
+        <v>2040.781073446328</v>
       </c>
       <c r="I26" t="n">
-        <v>1904.233333333333</v>
+        <v>1853.183333333333</v>
       </c>
       <c r="J26" t="n">
-        <v>34.37356575963719</v>
+        <v>34.01301789077213</v>
       </c>
       <c r="K26" t="n">
-        <v>31.73722222222222</v>
+        <v>30.88638888888889</v>
       </c>
       <c r="L26" t="n">
-        <v>2054.681632653061</v>
+        <v>2034.088983050847</v>
       </c>
       <c r="M26" t="n">
-        <v>1851.366666666667</v>
+        <v>1788.2</v>
       </c>
       <c r="N26" t="n">
-        <v>34.24469387755102</v>
+        <v>33.90148305084746</v>
       </c>
       <c r="O26" t="n">
-        <v>30.85611111111111</v>
+        <v>29.80333333333333</v>
       </c>
     </row>
     <row r="27">
@@ -5761,43 +5761,43 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="D27" t="n">
-        <v>361.5575268817204</v>
+        <v>365.8383333333333</v>
       </c>
       <c r="E27" t="n">
-        <v>205.6166666666667</v>
+        <v>188.3166666666667</v>
       </c>
       <c r="F27" t="n">
-        <v>6.025958781362008</v>
+        <v>6.097305555555556</v>
       </c>
       <c r="G27" t="n">
-        <v>3.426944444444445</v>
+        <v>3.138611111111111</v>
       </c>
       <c r="H27" t="n">
-        <v>2259.420967741936</v>
+        <v>2223.545416666667</v>
       </c>
       <c r="I27" t="n">
-        <v>2348.833333333333</v>
+        <v>2276.766666666666</v>
       </c>
       <c r="J27" t="n">
-        <v>37.65701612903226</v>
+        <v>37.05909027777778</v>
       </c>
       <c r="K27" t="n">
-        <v>39.14722222222223</v>
+        <v>37.94611111111111</v>
       </c>
       <c r="L27" t="n">
-        <v>1897.863440860215</v>
+        <v>1857.707083333333</v>
       </c>
       <c r="M27" t="n">
-        <v>1729.366666666667</v>
+        <v>1728.566666666667</v>
       </c>
       <c r="N27" t="n">
-        <v>31.63105734767025</v>
+        <v>30.96178472222222</v>
       </c>
       <c r="O27" t="n">
-        <v>28.82277777777778</v>
+        <v>28.80944444444444</v>
       </c>
     </row>
     <row r="28">
@@ -5812,43 +5812,43 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>406</v>
+        <v>482</v>
       </c>
       <c r="D28" t="n">
-        <v>177.6495073891626</v>
+        <v>149.8610650069157</v>
       </c>
       <c r="E28" t="n">
-        <v>1.991666666666667</v>
+        <v>1.85</v>
       </c>
       <c r="F28" t="n">
-        <v>2.960825123152709</v>
+        <v>2.497684416781927</v>
       </c>
       <c r="G28" t="n">
-        <v>0.03319444444444444</v>
+        <v>0.03083333333333333</v>
       </c>
       <c r="H28" t="n">
-        <v>868.3449848024316</v>
+        <v>818.1746395250211</v>
       </c>
       <c r="I28" t="n">
-        <v>839.1333333333333</v>
+        <v>811.4666666666667</v>
       </c>
       <c r="J28" t="n">
-        <v>14.47241641337386</v>
+        <v>13.63624399208369</v>
       </c>
       <c r="K28" t="n">
-        <v>13.98555555555556</v>
+        <v>13.52444444444444</v>
       </c>
       <c r="L28" t="n">
-        <v>653.2248226950355</v>
+        <v>637.8246395250213</v>
       </c>
       <c r="M28" t="n">
-        <v>533.0166666666667</v>
+        <v>542</v>
       </c>
       <c r="N28" t="n">
-        <v>10.88708037825059</v>
+        <v>10.63041065875035</v>
       </c>
       <c r="O28" t="n">
-        <v>8.883611111111112</v>
+        <v>9.033333333333333</v>
       </c>
     </row>
     <row r="29">
@@ -5863,43 +5863,43 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="D29" t="n">
-        <v>396.9627481713688</v>
+        <v>366.1142857142858</v>
       </c>
       <c r="E29" t="n">
-        <v>101.3166666666667</v>
+        <v>96.79166666666666</v>
       </c>
       <c r="F29" t="n">
-        <v>6.616045802856148</v>
+        <v>6.101904761904762</v>
       </c>
       <c r="G29" t="n">
-        <v>1.688611111111111</v>
+        <v>1.613194444444444</v>
       </c>
       <c r="H29" t="n">
-        <v>912.8494708994708</v>
+        <v>867.7253703703702</v>
       </c>
       <c r="I29" t="n">
-        <v>903.3166666666667</v>
+        <v>869.625</v>
       </c>
       <c r="J29" t="n">
-        <v>15.21415784832451</v>
+        <v>14.46208950617284</v>
       </c>
       <c r="K29" t="n">
-        <v>15.05527777777778</v>
+        <v>14.49375</v>
       </c>
       <c r="L29" t="n">
-        <v>515.9643915343916</v>
+        <v>502.0218055555555</v>
       </c>
       <c r="M29" t="n">
-        <v>187.9833333333333</v>
+        <v>186.5583333333333</v>
       </c>
       <c r="N29" t="n">
-        <v>8.599406525573194</v>
+        <v>8.367030092592593</v>
       </c>
       <c r="O29" t="n">
-        <v>3.133055555555555</v>
+        <v>3.109305555555555</v>
       </c>
     </row>
     <row r="30">
@@ -5914,43 +5914,43 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>6055</v>
+        <v>7096</v>
       </c>
       <c r="D30" t="n">
-        <v>5.020239471511148</v>
+        <v>4.486912814731304</v>
       </c>
       <c r="E30" t="n">
-        <v>1.883333333333333</v>
+        <v>1.8</v>
       </c>
       <c r="F30" t="n">
-        <v>0.08367065785851913</v>
+        <v>0.07478188024552174</v>
       </c>
       <c r="G30" t="n">
-        <v>0.03138888888888889</v>
+        <v>0.03</v>
       </c>
       <c r="H30" t="n">
-        <v>298.2195666404818</v>
+        <v>291.8230136145519</v>
       </c>
       <c r="I30" t="n">
-        <v>116.9583333333333</v>
+        <v>114.4583333333333</v>
       </c>
       <c r="J30" t="n">
-        <v>4.970326110674697</v>
+        <v>4.863716893575866</v>
       </c>
       <c r="K30" t="n">
-        <v>1.949305555555555</v>
+        <v>1.907638888888889</v>
       </c>
       <c r="L30" t="n">
-        <v>292.3526184865148</v>
+        <v>286.5855540676264</v>
       </c>
       <c r="M30" t="n">
-        <v>111.975</v>
+        <v>110.575</v>
       </c>
       <c r="N30" t="n">
-        <v>4.872543641441913</v>
+        <v>4.776425901127107</v>
       </c>
       <c r="O30" t="n">
-        <v>1.86625</v>
+        <v>1.842916666666667</v>
       </c>
     </row>
     <row r="31">
@@ -5965,43 +5965,43 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2287</v>
+        <v>3339</v>
       </c>
       <c r="D31" t="n">
-        <v>2388.069661856872</v>
+        <v>2252.446880303484</v>
       </c>
       <c r="E31" t="n">
-        <v>2065.633333333333</v>
+        <v>1760.216666666667</v>
       </c>
       <c r="F31" t="n">
-        <v>39.80116103094787</v>
+        <v>37.5407813383914</v>
       </c>
       <c r="G31" t="n">
-        <v>34.42722222222222</v>
+        <v>29.33694444444444</v>
       </c>
       <c r="H31" t="n">
-        <v>2719.90314232902</v>
+        <v>2529.654866372053</v>
       </c>
       <c r="I31" t="n">
-        <v>2395.25</v>
+        <v>2053.591666666667</v>
       </c>
       <c r="J31" t="n">
-        <v>45.33171903881701</v>
+        <v>42.16091443953424</v>
       </c>
       <c r="K31" t="n">
-        <v>39.92083333333333</v>
+        <v>34.22652777777778</v>
       </c>
       <c r="L31" t="n">
-        <v>315.5275955021565</v>
+        <v>265.8380366161616</v>
       </c>
       <c r="M31" t="n">
-        <v>350.25</v>
+        <v>278.8666666666667</v>
       </c>
       <c r="N31" t="n">
-        <v>5.258793258369275</v>
+        <v>4.430633943602694</v>
       </c>
       <c r="O31" t="n">
-        <v>5.8375</v>
+        <v>4.647777777777778</v>
       </c>
     </row>
     <row r="32">
@@ -6016,43 +6016,43 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6116</v>
+        <v>7259</v>
       </c>
       <c r="D32" t="n">
-        <v>441.9897427512535</v>
+        <v>400.5894016623043</v>
       </c>
       <c r="E32" t="n">
-        <v>2.566666666666667</v>
+        <v>2.4</v>
       </c>
       <c r="F32" t="n">
-        <v>7.366495712520893</v>
+        <v>6.67649002770507</v>
       </c>
       <c r="G32" t="n">
-        <v>0.04277777777777778</v>
+        <v>0.04</v>
       </c>
       <c r="H32" t="n">
-        <v>741.9601811965811</v>
+        <v>695.0364603147154</v>
       </c>
       <c r="I32" t="n">
-        <v>430.9166666666667</v>
+        <v>412.1833333333333</v>
       </c>
       <c r="J32" t="n">
-        <v>12.36600301994302</v>
+        <v>11.58394100524526</v>
       </c>
       <c r="K32" t="n">
-        <v>7.181944444444444</v>
+        <v>6.869722222222222</v>
       </c>
       <c r="L32" t="n">
-        <v>193.3965264957265</v>
+        <v>197.5324226180183</v>
       </c>
       <c r="M32" t="n">
-        <v>51.53333333333333</v>
+        <v>53.05</v>
       </c>
       <c r="N32" t="n">
-        <v>3.223275441595442</v>
+        <v>3.292207043633639</v>
       </c>
       <c r="O32" t="n">
-        <v>0.8588888888888888</v>
+        <v>0.8841666666666667</v>
       </c>
     </row>
     <row r="33">
@@ -6067,43 +6067,43 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>5355</v>
+        <v>6457</v>
       </c>
       <c r="D33" t="n">
-        <v>568.2112138188609</v>
+        <v>524.5919518868411</v>
       </c>
       <c r="E33" t="n">
-        <v>163.2</v>
+        <v>153.3</v>
       </c>
       <c r="F33" t="n">
-        <v>9.470186896981016</v>
+        <v>8.74319919811402</v>
       </c>
       <c r="G33" t="n">
-        <v>2.72</v>
+        <v>2.555</v>
       </c>
       <c r="H33" t="n">
-        <v>795.264374173798</v>
+        <v>747.7614985970338</v>
       </c>
       <c r="I33" t="n">
-        <v>566.1833333333333</v>
+        <v>543.1333333333333</v>
       </c>
       <c r="J33" t="n">
-        <v>13.25440623622997</v>
+        <v>12.4626916432839</v>
       </c>
       <c r="K33" t="n">
-        <v>9.436388888888889</v>
+        <v>9.052222222222222</v>
       </c>
       <c r="L33" t="n">
-        <v>190.1371982188826</v>
+        <v>193.5098293534902</v>
       </c>
       <c r="M33" t="n">
-        <v>51.03333333333333</v>
+        <v>52.06666666666667</v>
       </c>
       <c r="N33" t="n">
-        <v>3.168953303648044</v>
+        <v>3.225163822558171</v>
       </c>
       <c r="O33" t="n">
-        <v>0.8505555555555555</v>
+        <v>0.8677777777777779</v>
       </c>
     </row>
     <row r="34">
@@ -6118,43 +6118,43 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2308</v>
+        <v>2831</v>
       </c>
       <c r="D34" t="n">
-        <v>1263.163272674754</v>
+        <v>1093.239703285058</v>
       </c>
       <c r="E34" t="n">
-        <v>906.5999999999999</v>
+        <v>764.05</v>
       </c>
       <c r="F34" t="n">
-        <v>21.05272121124591</v>
+        <v>18.22066172141764</v>
       </c>
       <c r="G34" t="n">
-        <v>15.11</v>
+        <v>12.73416666666667</v>
       </c>
       <c r="H34" t="n">
-        <v>1498.737374128583</v>
+        <v>1482.234134615385</v>
       </c>
       <c r="I34" t="n">
-        <v>1190.9</v>
+        <v>1171.775</v>
       </c>
       <c r="J34" t="n">
-        <v>24.97895623547637</v>
+        <v>24.70390224358974</v>
       </c>
       <c r="K34" t="n">
-        <v>19.84833333333334</v>
+        <v>19.52958333333333</v>
       </c>
       <c r="L34" t="n">
-        <v>363.4699457784663</v>
+        <v>377.2971997300945</v>
       </c>
       <c r="M34" t="n">
-        <v>437.1333333333333</v>
+        <v>359.4333333333333</v>
       </c>
       <c r="N34" t="n">
-        <v>6.057832429641104</v>
+        <v>6.288286662168241</v>
       </c>
       <c r="O34" t="n">
-        <v>7.285555555555556</v>
+        <v>5.990555555555556</v>
       </c>
     </row>
     <row r="35">
@@ -6169,43 +6169,43 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2321</v>
+        <v>2751</v>
       </c>
       <c r="D35" t="n">
-        <v>1506.567133419503</v>
+        <v>1356.237453047377</v>
       </c>
       <c r="E35" t="n">
-        <v>1013.666666666667</v>
+        <v>957.5833333333334</v>
       </c>
       <c r="F35" t="n">
-        <v>25.10945222365838</v>
+        <v>22.60395755078961</v>
       </c>
       <c r="G35" t="n">
-        <v>16.89444444444444</v>
+        <v>15.95972222222222</v>
       </c>
       <c r="H35" t="n">
-        <v>1748.829237947123</v>
+        <v>1711.791161223432</v>
       </c>
       <c r="I35" t="n">
-        <v>1370.8</v>
+        <v>1325.683333333333</v>
       </c>
       <c r="J35" t="n">
-        <v>29.14715396578539</v>
+        <v>28.5298526870572</v>
       </c>
       <c r="K35" t="n">
-        <v>22.84666666666667</v>
+        <v>22.09472222222222</v>
       </c>
       <c r="L35" t="n">
-        <v>363.0080093312597</v>
+        <v>360.0762484879903</v>
       </c>
       <c r="M35" t="n">
-        <v>399.925</v>
+        <v>357.2833333333334</v>
       </c>
       <c r="N35" t="n">
-        <v>6.050133488854329</v>
+        <v>6.001270808133172</v>
       </c>
       <c r="O35" t="n">
-        <v>6.665416666666666</v>
+        <v>5.954722222222222</v>
       </c>
     </row>
     <row r="36">
@@ -6220,43 +6220,43 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>488</v>
+        <v>587</v>
       </c>
       <c r="D36" t="n">
-        <v>6.110382513661201</v>
+        <v>5.31044860874503</v>
       </c>
       <c r="E36" t="n">
-        <v>1.716666666666667</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="F36" t="n">
-        <v>0.10183970856102</v>
+        <v>0.08850747681241719</v>
       </c>
       <c r="G36" t="n">
-        <v>0.02861111111111111</v>
+        <v>0.02777777777777778</v>
       </c>
       <c r="H36" t="n">
-        <v>1072.92518115942</v>
+        <v>1101.769933712121</v>
       </c>
       <c r="I36" t="n">
-        <v>1154.15</v>
+        <v>1177.408333333333</v>
       </c>
       <c r="J36" t="n">
-        <v>17.88208635265701</v>
+        <v>18.36283222853535</v>
       </c>
       <c r="K36" t="n">
-        <v>19.23583333333333</v>
+        <v>19.62347222222222</v>
       </c>
       <c r="L36" t="n">
-        <v>1062.995531400966</v>
+        <v>1093.621732954545</v>
       </c>
       <c r="M36" t="n">
-        <v>1150.308333333333</v>
+        <v>1174.908333333333</v>
       </c>
       <c r="N36" t="n">
-        <v>17.7165921900161</v>
+        <v>18.22702888257576</v>
       </c>
       <c r="O36" t="n">
-        <v>19.17180555555556</v>
+        <v>19.58180555555555</v>
       </c>
     </row>
     <row r="37">
@@ -6271,43 +6271,43 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>441</v>
+        <v>595</v>
       </c>
       <c r="D37" t="n">
-        <v>3563.801965230537</v>
+        <v>3214.939635854342</v>
       </c>
       <c r="E37" t="n">
-        <v>2929.883333333333</v>
+        <v>2568.433333333333</v>
       </c>
       <c r="F37" t="n">
-        <v>59.39669942050894</v>
+        <v>53.58232726423903</v>
       </c>
       <c r="G37" t="n">
-        <v>48.83138888888889</v>
+        <v>42.80722222222222</v>
       </c>
       <c r="H37" t="n">
-        <v>4119.318204488778</v>
+        <v>3713.384854014598</v>
       </c>
       <c r="I37" t="n">
-        <v>4314.4</v>
+        <v>3013.091666666667</v>
       </c>
       <c r="J37" t="n">
-        <v>68.6553034081463</v>
+        <v>61.88974756690997</v>
       </c>
       <c r="K37" t="n">
-        <v>71.90666666666667</v>
+        <v>50.21819444444444</v>
       </c>
       <c r="L37" t="n">
-        <v>237.6677888611804</v>
+        <v>265.4235705596108</v>
       </c>
       <c r="M37" t="n">
-        <v>235.75</v>
+        <v>284.0333333333333</v>
       </c>
       <c r="N37" t="n">
-        <v>3.961129814353006</v>
+        <v>4.423726175993511</v>
       </c>
       <c r="O37" t="n">
-        <v>3.929166666666667</v>
+        <v>4.733888888888888</v>
       </c>
     </row>
     <row r="38">
@@ -6322,43 +6322,43 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>728</v>
+        <v>896</v>
       </c>
       <c r="D38" t="n">
-        <v>2.844665750915751</v>
+        <v>2.543563988095238</v>
       </c>
       <c r="E38" t="n">
-        <v>1.716666666666667</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="F38" t="n">
-        <v>0.04741109584859585</v>
+        <v>0.04239273313492064</v>
       </c>
       <c r="G38" t="n">
-        <v>0.02861111111111111</v>
+        <v>0.02777777777777778</v>
       </c>
       <c r="H38" t="n">
-        <v>487.3917133956386</v>
+        <v>481.1858895705521</v>
       </c>
       <c r="I38" t="n">
-        <v>421.75</v>
+        <v>416.3583333333333</v>
       </c>
       <c r="J38" t="n">
-        <v>8.123195223260643</v>
+        <v>8.019764826175869</v>
       </c>
       <c r="K38" t="n">
-        <v>7.029166666666667</v>
+        <v>6.939305555555555</v>
       </c>
       <c r="L38" t="n">
-        <v>483.6088785046729</v>
+        <v>477.7957055214724</v>
       </c>
       <c r="M38" t="n">
-        <v>419.3833333333333</v>
+        <v>413.925</v>
       </c>
       <c r="N38" t="n">
-        <v>8.060147975077882</v>
+        <v>7.963261758691207</v>
       </c>
       <c r="O38" t="n">
-        <v>6.989722222222222</v>
+        <v>6.89875</v>
       </c>
     </row>
     <row r="39">
@@ -6373,43 +6373,43 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>796</v>
+        <v>976</v>
       </c>
       <c r="D39" t="n">
-        <v>203.6789572864322</v>
+        <v>213.0564378415301</v>
       </c>
       <c r="E39" t="n">
-        <v>75.40000000000001</v>
+        <v>82.19999999999999</v>
       </c>
       <c r="F39" t="n">
-        <v>3.394649288107203</v>
+        <v>3.550940630692168</v>
       </c>
       <c r="G39" t="n">
-        <v>1.256666666666667</v>
+        <v>1.37</v>
       </c>
       <c r="H39" t="n">
-        <v>674.4561985262245</v>
+        <v>680.8541622574957</v>
       </c>
       <c r="I39" t="n">
-        <v>639.6333333333333</v>
+        <v>670.5833333333334</v>
       </c>
       <c r="J39" t="n">
-        <v>11.24093664210374</v>
+        <v>11.34756937095826</v>
       </c>
       <c r="K39" t="n">
-        <v>10.66055555555556</v>
+        <v>11.17638888888889</v>
       </c>
       <c r="L39" t="n">
-        <v>469.6657563935847</v>
+        <v>466.2167372134039</v>
       </c>
       <c r="M39" t="n">
-        <v>302.5833333333333</v>
+        <v>290.4</v>
       </c>
       <c r="N39" t="n">
-        <v>7.827762606559746</v>
+        <v>7.770278953556732</v>
       </c>
       <c r="O39" t="n">
-        <v>5.043055555555555</v>
+        <v>4.84</v>
       </c>
     </row>
     <row r="40">
@@ -6424,40 +6424,40 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>27814</v>
+        <v>31189</v>
       </c>
       <c r="D40" t="n">
-        <v>50.04443026293713</v>
+        <v>47.07778543717335</v>
       </c>
       <c r="E40" t="n">
-        <v>1.833333333333333</v>
+        <v>1.783333333333333</v>
       </c>
       <c r="F40" t="n">
-        <v>0.8340738377156188</v>
+        <v>0.7846297572862226</v>
       </c>
       <c r="G40" t="n">
-        <v>0.03055555555555555</v>
+        <v>0.02972222222222222</v>
       </c>
       <c r="H40" t="n">
-        <v>76.69005151320026</v>
+        <v>72.65701603313241</v>
       </c>
       <c r="I40" t="n">
-        <v>2.216666666666667</v>
+        <v>2.183333333333333</v>
       </c>
       <c r="J40" t="n">
-        <v>1.278167525220004</v>
+        <v>1.210950267218873</v>
       </c>
       <c r="K40" t="n">
-        <v>0.03694444444444445</v>
+        <v>0.03638888888888889</v>
       </c>
       <c r="L40" t="n">
-        <v>14.25813172661209</v>
+        <v>13.97743879936031</v>
       </c>
       <c r="M40" t="n">
         <v>0.2333333333333333</v>
       </c>
       <c r="N40" t="n">
-        <v>0.2376355287768681</v>
+        <v>0.2329573133226719</v>
       </c>
       <c r="O40" t="n">
         <v>0.003888888888888889</v>
@@ -6475,43 +6475,43 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>6854</v>
+        <v>9682</v>
       </c>
       <c r="D41" t="n">
-        <v>865.0610373504522</v>
+        <v>899.1005749500791</v>
       </c>
       <c r="E41" t="n">
-        <v>791.2083333333334</v>
+        <v>792.0916666666667</v>
       </c>
       <c r="F41" t="n">
-        <v>14.41768395584087</v>
+        <v>14.98500958250132</v>
       </c>
       <c r="G41" t="n">
-        <v>13.18680555555556</v>
+        <v>13.20152777777778</v>
       </c>
       <c r="H41" t="n">
-        <v>922.7099593495934</v>
+        <v>966.1008261802574</v>
       </c>
       <c r="I41" t="n">
-        <v>839.9166666666666</v>
+        <v>841.2916666666666</v>
       </c>
       <c r="J41" t="n">
-        <v>15.37849932249322</v>
+        <v>16.10168043633763</v>
       </c>
       <c r="K41" t="n">
-        <v>13.99861111111111</v>
+        <v>14.02152777777778</v>
       </c>
       <c r="L41" t="n">
-        <v>50.42740138512496</v>
+        <v>61.45168633762518</v>
       </c>
       <c r="M41" t="n">
-        <v>42.05</v>
+        <v>42.85833333333333</v>
       </c>
       <c r="N41" t="n">
-        <v>0.8404566897520828</v>
+        <v>1.024194772293753</v>
       </c>
       <c r="O41" t="n">
-        <v>0.7008333333333333</v>
+        <v>0.7143055555555555</v>
       </c>
     </row>
     <row r="42">
@@ -6526,43 +6526,43 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>58084</v>
+        <v>68830</v>
       </c>
       <c r="D42" t="n">
-        <v>3.86301735417671</v>
+        <v>3.503384183253427</v>
       </c>
       <c r="E42" t="n">
-        <v>1.916666666666667</v>
+        <v>1.85</v>
       </c>
       <c r="F42" t="n">
-        <v>0.06438362256961183</v>
+        <v>0.0583897363875571</v>
       </c>
       <c r="G42" t="n">
-        <v>0.03194444444444445</v>
+        <v>0.03083333333333333</v>
       </c>
       <c r="H42" t="n">
-        <v>355.0888420809345</v>
+        <v>353.7265263997578</v>
       </c>
       <c r="I42" t="n">
-        <v>152.0166666666667</v>
+        <v>156.5583333333333</v>
       </c>
       <c r="J42" t="n">
-        <v>5.918147368015576</v>
+        <v>5.89544210666263</v>
       </c>
       <c r="K42" t="n">
-        <v>2.533611111111111</v>
+        <v>2.609305555555555</v>
       </c>
       <c r="L42" t="n">
-        <v>350.8898148926335</v>
+        <v>349.9612033025899</v>
       </c>
       <c r="M42" t="n">
-        <v>148.925</v>
+        <v>153.5166666666667</v>
       </c>
       <c r="N42" t="n">
-        <v>5.848163581543892</v>
+        <v>5.832686721709832</v>
       </c>
       <c r="O42" t="n">
-        <v>2.482083333333333</v>
+        <v>2.558611111111111</v>
       </c>
     </row>
     <row r="43">
@@ -6577,43 +6577,43 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>35054</v>
+        <v>42659</v>
       </c>
       <c r="D43" t="n">
-        <v>179.2518994503718</v>
+        <v>180.5679497097134</v>
       </c>
       <c r="E43" t="n">
-        <v>94.7</v>
+        <v>94.13333333333334</v>
       </c>
       <c r="F43" t="n">
-        <v>2.987531657506196</v>
+        <v>3.009465828495224</v>
       </c>
       <c r="G43" t="n">
-        <v>1.578333333333333</v>
+        <v>1.568888888888889</v>
       </c>
       <c r="H43" t="n">
-        <v>476.3966606230252</v>
+        <v>475.9913850684249</v>
       </c>
       <c r="I43" t="n">
-        <v>238.8416666666667</v>
+        <v>247.8583333333333</v>
       </c>
       <c r="J43" t="n">
-        <v>7.939944343717087</v>
+        <v>7.933189751140416</v>
       </c>
       <c r="K43" t="n">
-        <v>3.980694444444445</v>
+        <v>4.130972222222223</v>
       </c>
       <c r="L43" t="n">
-        <v>301.3248409568039</v>
+        <v>298.2019445732241</v>
       </c>
       <c r="M43" t="n">
-        <v>101.3416666666667</v>
+        <v>109.275</v>
       </c>
       <c r="N43" t="n">
-        <v>5.022080682613398</v>
+        <v>4.970032409553736</v>
       </c>
       <c r="O43" t="n">
-        <v>1.689027777777778</v>
+        <v>1.82125</v>
       </c>
     </row>
     <row r="44">
@@ -6628,43 +6628,43 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>6610</v>
+        <v>8960</v>
       </c>
       <c r="D44" t="n">
-        <v>4.45160363086233</v>
+        <v>3.66143043154762</v>
       </c>
       <c r="E44" t="n">
-        <v>1.983333333333333</v>
+        <v>1.816666666666667</v>
       </c>
       <c r="F44" t="n">
-        <v>0.0741933938477055</v>
+        <v>0.06102384052579365</v>
       </c>
       <c r="G44" t="n">
-        <v>0.03305555555555555</v>
+        <v>0.03027777777777778</v>
       </c>
       <c r="H44" t="n">
-        <v>799.7591884161602</v>
+        <v>861.6109548724656</v>
       </c>
       <c r="I44" t="n">
-        <v>816.8833333333333</v>
+        <v>878</v>
       </c>
       <c r="J44" t="n">
-        <v>13.329319806936</v>
+        <v>14.36018258120776</v>
       </c>
       <c r="K44" t="n">
-        <v>13.61472222222222</v>
+        <v>14.63333333333333</v>
       </c>
       <c r="L44" t="n">
-        <v>794.6534203313074</v>
+        <v>857.4419816873773</v>
       </c>
       <c r="M44" t="n">
-        <v>794.8</v>
+        <v>870.6833333333333</v>
       </c>
       <c r="N44" t="n">
-        <v>13.24422367218845</v>
+        <v>14.29069969478962</v>
       </c>
       <c r="O44" t="n">
-        <v>13.24666666666667</v>
+        <v>14.51138888888889</v>
       </c>
     </row>
     <row r="45">
@@ -6679,43 +6679,43 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>7706</v>
+        <v>10131</v>
       </c>
       <c r="D45" t="n">
-        <v>241.4909096807683</v>
+        <v>261.9331095976048</v>
       </c>
       <c r="E45" t="n">
-        <v>52.75</v>
+        <v>65.43333333333334</v>
       </c>
       <c r="F45" t="n">
-        <v>4.024848494679471</v>
+        <v>4.365551826626745</v>
       </c>
       <c r="G45" t="n">
-        <v>0.8791666666666667</v>
+        <v>1.090555555555556</v>
       </c>
       <c r="H45" t="n">
-        <v>933.6757616729764</v>
+        <v>964.0909429959626</v>
       </c>
       <c r="I45" t="n">
-        <v>939.8666666666667</v>
+        <v>968.4583333333333</v>
       </c>
       <c r="J45" t="n">
-        <v>15.5612626945496</v>
+        <v>16.06818238326604</v>
       </c>
       <c r="K45" t="n">
-        <v>15.66444444444445</v>
+        <v>16.14097222222222</v>
       </c>
       <c r="L45" t="n">
-        <v>693.1163714620516</v>
+        <v>701.8492592212414</v>
       </c>
       <c r="M45" t="n">
-        <v>511.9583333333333</v>
+        <v>525.6333333333333</v>
       </c>
       <c r="N45" t="n">
-        <v>11.55193952436753</v>
+        <v>11.69748765368736</v>
       </c>
       <c r="O45" t="n">
-        <v>8.53263888888889</v>
+        <v>8.760555555555555</v>
       </c>
     </row>
     <row r="46">
@@ -6730,43 +6730,43 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>454</v>
+        <v>508</v>
       </c>
       <c r="D46" t="n">
-        <v>1.718795888399413</v>
+        <v>1.612106299212599</v>
       </c>
       <c r="E46" t="n">
-        <v>1.716666666666667</v>
+        <v>1.608333333333333</v>
       </c>
       <c r="F46" t="n">
-        <v>0.02864659813999021</v>
+        <v>0.02686843832020997</v>
       </c>
       <c r="G46" t="n">
-        <v>0.02861111111111111</v>
+        <v>0.02680555555555555</v>
       </c>
       <c r="H46" t="n">
-        <v>1936.881588447653</v>
+        <v>1852.311521252797</v>
       </c>
       <c r="I46" t="n">
-        <v>2066.466666666667</v>
+        <v>1985.55</v>
       </c>
       <c r="J46" t="n">
-        <v>32.28135980746089</v>
+        <v>30.8718586875466</v>
       </c>
       <c r="K46" t="n">
-        <v>34.44111111111111</v>
+        <v>33.0925</v>
       </c>
       <c r="L46" t="n">
-        <v>1934.677858002407</v>
+        <v>1850.154138702461</v>
       </c>
       <c r="M46" t="n">
-        <v>2064.566666666667</v>
+        <v>1983.258333333333</v>
       </c>
       <c r="N46" t="n">
-        <v>32.24463096670678</v>
+        <v>30.83590231170768</v>
       </c>
       <c r="O46" t="n">
-        <v>34.40944444444445</v>
+        <v>33.05430555555556</v>
       </c>
     </row>
     <row r="47">
@@ -6781,43 +6781,43 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>346</v>
+        <v>357</v>
       </c>
       <c r="D47" t="n">
-        <v>333.0520231213873</v>
+        <v>332.5461251167133</v>
       </c>
       <c r="E47" t="n">
-        <v>152.4583333333333</v>
+        <v>148.3166666666667</v>
       </c>
       <c r="F47" t="n">
-        <v>5.550867052023122</v>
+        <v>5.542435418611888</v>
       </c>
       <c r="G47" t="n">
-        <v>2.540972222222222</v>
+        <v>2.471944444444444</v>
       </c>
       <c r="H47" t="n">
-        <v>1983.986612903226</v>
+        <v>1960.664755838641</v>
       </c>
       <c r="I47" t="n">
-        <v>2267.308333333333</v>
+        <v>2244.283333333333</v>
       </c>
       <c r="J47" t="n">
-        <v>33.0664435483871</v>
+        <v>32.67774593064402</v>
       </c>
       <c r="K47" t="n">
-        <v>37.78847222222223</v>
+        <v>37.40472222222222</v>
       </c>
       <c r="L47" t="n">
-        <v>1636.380967741936</v>
+        <v>1617.171496815286</v>
       </c>
       <c r="M47" t="n">
-        <v>1768.725</v>
+        <v>1766.816666666667</v>
       </c>
       <c r="N47" t="n">
-        <v>27.27301612903226</v>
+        <v>26.95285828025478</v>
       </c>
       <c r="O47" t="n">
-        <v>29.47875</v>
+        <v>29.44694444444444</v>
       </c>
     </row>
     <row r="48">
@@ -6832,43 +6832,43 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3089</v>
+        <v>3905</v>
       </c>
       <c r="D48" t="n">
-        <v>4.139003992662134</v>
+        <v>3.566376440460948</v>
       </c>
       <c r="E48" t="n">
-        <v>1.916666666666667</v>
+        <v>1.8</v>
       </c>
       <c r="F48" t="n">
-        <v>0.06898339987770225</v>
+        <v>0.0594396073410158</v>
       </c>
       <c r="G48" t="n">
-        <v>0.03194444444444445</v>
+        <v>0.03</v>
       </c>
       <c r="H48" t="n">
-        <v>460.4456556082148</v>
+        <v>438.0617387936877</v>
       </c>
       <c r="I48" t="n">
-        <v>388.8166666666667</v>
+        <v>368.9333333333333</v>
       </c>
       <c r="J48" t="n">
-        <v>7.674094260136914</v>
+        <v>7.301028979894795</v>
       </c>
       <c r="K48" t="n">
-        <v>6.480277777777777</v>
+        <v>6.148888888888889</v>
       </c>
       <c r="L48" t="n">
-        <v>455.8080325677482</v>
+        <v>434.0382708877916</v>
       </c>
       <c r="M48" t="n">
-        <v>382.5833333333333</v>
+        <v>364.5833333333333</v>
       </c>
       <c r="N48" t="n">
-        <v>7.596800542795805</v>
+        <v>7.233971181463194</v>
       </c>
       <c r="O48" t="n">
-        <v>6.376388888888888</v>
+        <v>6.076388888888888</v>
       </c>
     </row>
     <row r="49">
@@ -6883,43 +6883,43 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1287</v>
+        <v>1681</v>
       </c>
       <c r="D49" t="n">
-        <v>299.5193732193732</v>
+        <v>288.9701070791195</v>
       </c>
       <c r="E49" t="n">
-        <v>96.76666666666667</v>
+        <v>105.6333333333333</v>
       </c>
       <c r="F49" t="n">
-        <v>4.99198955365622</v>
+        <v>4.81616845131866</v>
       </c>
       <c r="G49" t="n">
-        <v>1.612777777777778</v>
+        <v>1.760555555555556</v>
       </c>
       <c r="H49" t="n">
-        <v>729.1852118305355</v>
+        <v>697.377431626568</v>
       </c>
       <c r="I49" t="n">
-        <v>591.75</v>
+        <v>586.35</v>
       </c>
       <c r="J49" t="n">
-        <v>12.15308686384226</v>
+        <v>11.62295719377613</v>
       </c>
       <c r="K49" t="n">
-        <v>9.862500000000001</v>
+        <v>9.772500000000001</v>
       </c>
       <c r="L49" t="n">
-        <v>429.4550093258727</v>
+        <v>406.8881554595928</v>
       </c>
       <c r="M49" t="n">
-        <v>265.9833333333333</v>
+        <v>259.2166666666666</v>
       </c>
       <c r="N49" t="n">
-        <v>7.157583488764544</v>
+        <v>6.781469257659881</v>
       </c>
       <c r="O49" t="n">
-        <v>4.433055555555556</v>
+        <v>4.320277777777777</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reemplazar marca Paniplay por Catraplay Honduras en dashboard y reportes
</commit_message>
<xml_diff>
--- a/Reporte_Efectividad_Automatizacion.xlsx
+++ b/Reporte_Efectividad_Automatizacion.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG16"/>
+  <dimension ref="A1:AG15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -724,19 +724,19 @@
         <v>68.64676231097324</v>
       </c>
       <c r="AC2" t="n">
-        <v>315</v>
+        <v>1516</v>
       </c>
       <c r="AD2" t="n">
-        <v>33.33333333333333</v>
+        <v>32.12401055408971</v>
       </c>
       <c r="AE2" t="n">
-        <v>68.57142857142857</v>
+        <v>67.94195250659631</v>
       </c>
       <c r="AF2" t="n">
-        <v>-2.680625565464652</v>
+        <v>-3.889948344708273</v>
       </c>
       <c r="AG2" t="n">
-        <v>-97.55719271035285</v>
+        <v>-88.24350523458705</v>
       </c>
     </row>
     <row r="3">
@@ -827,19 +827,19 @@
         <v>77.19869706840392</v>
       </c>
       <c r="AC3" t="n">
-        <v>31</v>
+        <v>164</v>
       </c>
       <c r="AD3" t="n">
-        <v>38.70967741935484</v>
+        <v>35.36585365853659</v>
       </c>
       <c r="AE3" t="n">
-        <v>83.87096774193549</v>
+        <v>78.04878048780488</v>
       </c>
       <c r="AF3" t="n">
-        <v>2.227592728801092</v>
+        <v>-1.116231032017161</v>
       </c>
       <c r="AG3" t="n">
-        <v>-96.63409337676438</v>
+        <v>-82.19326818675353</v>
       </c>
     </row>
     <row r="4">
@@ -849,67 +849,67 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>10991</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>72.30461286507143</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>86.31607679010099</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>12023</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>74.23272061881394</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>88.38060384263495</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>14042</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>76.31391539666714</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>88.14983620566871</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>13195</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>67.07843880257673</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>84.50928381962865</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>13769</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>74.71857070230227</v>
       </c>
       <c r="P4" t="n">
-        <v>0</v>
+        <v>84.62488198126226</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>16085</v>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
+        <v>70.71806030463165</v>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>81.03823437985702</v>
       </c>
       <c r="T4" t="n">
-        <v>0</v>
+        <v>16006</v>
       </c>
       <c r="U4" t="n">
-        <v>0</v>
+        <v>59.19655129326502</v>
       </c>
       <c r="V4" t="n">
-        <v>0</v>
+        <v>74.15969011620642</v>
       </c>
       <c r="W4" t="n">
         <v>16294</v>
@@ -930,19 +930,19 @@
         <v>73.31313006370215</v>
       </c>
       <c r="AC4" t="n">
-        <v>0</v>
+        <v>1154</v>
       </c>
       <c r="AD4" t="n">
-        <v>0</v>
+        <v>73.83015597920277</v>
       </c>
       <c r="AE4" t="n">
-        <v>0</v>
+        <v>77.55632582322357</v>
       </c>
       <c r="AF4" t="n">
-        <v>-66.31207866905807</v>
+        <v>7.518077310144704</v>
       </c>
       <c r="AG4" t="n">
-        <v>-100</v>
+        <v>-92.86288576906426</v>
       </c>
     </row>
     <row r="5">
@@ -1033,19 +1033,19 @@
         <v>64.44652908067542</v>
       </c>
       <c r="AC5" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="AD5" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="AE5" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="AF5" t="n">
-        <v>39.77485928705441</v>
+        <v>34.77485928705441</v>
       </c>
       <c r="AG5" t="n">
-        <v>-99.90619136960601</v>
+        <v>-98.12382739212008</v>
       </c>
     </row>
     <row r="6">
@@ -1136,19 +1136,19 @@
         <v>62.38116794929832</v>
       </c>
       <c r="AC6" t="n">
-        <v>16</v>
+        <v>145</v>
       </c>
       <c r="AD6" t="n">
-        <v>56.25</v>
+        <v>66.89655172413794</v>
       </c>
       <c r="AE6" t="n">
-        <v>62.5</v>
+        <v>69.6551724137931</v>
       </c>
       <c r="AF6" t="n">
-        <v>-1.377885921231325</v>
+        <v>9.268665802906611</v>
       </c>
       <c r="AG6" t="n">
-        <v>-99.27569035762789</v>
+        <v>-93.43594386600272</v>
       </c>
     </row>
     <row r="7">
@@ -1239,19 +1239,19 @@
         <v>75.22007042253522</v>
       </c>
       <c r="AC7" t="n">
-        <v>771</v>
+        <v>3365</v>
       </c>
       <c r="AD7" t="n">
-        <v>53.43709468223087</v>
+        <v>77.47399702823181</v>
       </c>
       <c r="AE7" t="n">
-        <v>58.75486381322958</v>
+        <v>80.44576523031203</v>
       </c>
       <c r="AF7" t="n">
-        <v>-17.42958265451689</v>
+        <v>6.607319691484051</v>
       </c>
       <c r="AG7" t="n">
-        <v>-96.91501280409732</v>
+        <v>-86.5356914212548</v>
       </c>
     </row>
     <row r="8">
@@ -1342,19 +1342,19 @@
         <v>63.54662436100828</v>
       </c>
       <c r="AC8" t="n">
-        <v>740</v>
+        <v>4232</v>
       </c>
       <c r="AD8" t="n">
-        <v>46.48648648648649</v>
+        <v>49.19659735349716</v>
       </c>
       <c r="AE8" t="n">
-        <v>63.37837837837837</v>
+        <v>64.22495274102079</v>
       </c>
       <c r="AF8" t="n">
-        <v>-4.6210991530928</v>
+        <v>-1.91098828608213</v>
       </c>
       <c r="AG8" t="n">
-        <v>-97.82595922204594</v>
+        <v>-87.56683706445737</v>
       </c>
     </row>
     <row r="9">
@@ -1445,19 +1445,19 @@
         <v>58.85237110242856</v>
       </c>
       <c r="AC9" t="n">
-        <v>641</v>
+        <v>3212</v>
       </c>
       <c r="AD9" t="n">
-        <v>46.02184087363494</v>
+        <v>50.21793275217933</v>
       </c>
       <c r="AE9" t="n">
-        <v>53.97815912636506</v>
+        <v>60.18057285180573</v>
       </c>
       <c r="AF9" t="n">
-        <v>-3.767479589093931</v>
+        <v>0.4286122894504558</v>
       </c>
       <c r="AG9" t="n">
-        <v>-95.08925151306214</v>
+        <v>-75.39263004673256</v>
       </c>
     </row>
     <row r="10">
@@ -1548,19 +1548,19 @@
         <v>70.28350515463917</v>
       </c>
       <c r="AC10" t="n">
-        <v>28</v>
+        <v>277</v>
       </c>
       <c r="AD10" t="n">
-        <v>78.57142857142857</v>
+        <v>61.73285198555957</v>
       </c>
       <c r="AE10" t="n">
-        <v>89.28571428571429</v>
+        <v>70.75812274368231</v>
       </c>
       <c r="AF10" t="n">
-        <v>13.80338733431516</v>
+        <v>-3.035189251553838</v>
       </c>
       <c r="AG10" t="n">
-        <v>-99.27835051546393</v>
+        <v>-92.86082474226805</v>
       </c>
     </row>
     <row r="11">
@@ -1651,19 +1651,19 @@
         <v>52.71958098307816</v>
       </c>
       <c r="AC11" t="n">
-        <v>130</v>
+        <v>685</v>
       </c>
       <c r="AD11" t="n">
-        <v>47.69230769230769</v>
+        <v>55.32846715328466</v>
       </c>
       <c r="AE11" t="n">
-        <v>52.30769230769231</v>
+        <v>59.70802919708029</v>
       </c>
       <c r="AF11" t="n">
-        <v>2.809148949358459</v>
+        <v>10.44530841033543</v>
       </c>
       <c r="AG11" t="n">
-        <v>-97.38114423851732</v>
+        <v>-86.20064464141821</v>
       </c>
     </row>
     <row r="12">
@@ -1754,19 +1754,19 @@
         <v>79.36049855181572</v>
       </c>
       <c r="AC12" t="n">
-        <v>2777</v>
+        <v>15307</v>
       </c>
       <c r="AD12" t="n">
-        <v>75.18905293482176</v>
+        <v>75.33808061671131</v>
       </c>
       <c r="AE12" t="n">
-        <v>81.63485776017285</v>
+        <v>80.52524988567322</v>
       </c>
       <c r="AF12" t="n">
-        <v>-0.35911356977374</v>
+        <v>-0.2100858878841905</v>
       </c>
       <c r="AG12" t="n">
-        <v>-97.09631209678263</v>
+        <v>-83.99468824827211</v>
       </c>
     </row>
     <row r="13">
@@ -1857,19 +1857,19 @@
         <v>77.12983384796354</v>
       </c>
       <c r="AC13" t="n">
-        <v>5803</v>
+        <v>39662</v>
       </c>
       <c r="AD13" t="n">
-        <v>61.9334826813717</v>
+        <v>59.5027986485805</v>
       </c>
       <c r="AE13" t="n">
-        <v>77.52886438049285</v>
+        <v>76.67540719076193</v>
       </c>
       <c r="AF13" t="n">
-        <v>0.05696125478410607</v>
+        <v>-2.373722778007092</v>
       </c>
       <c r="AG13" t="n">
-        <v>-98.10387361335752</v>
+        <v>-87.04046790504665</v>
       </c>
     </row>
     <row r="14">
@@ -1960,19 +1960,19 @@
         <v>65.35435553803705</v>
       </c>
       <c r="AC14" t="n">
-        <v>617</v>
+        <v>4594</v>
       </c>
       <c r="AD14" t="n">
-        <v>37.43922204213938</v>
+        <v>44.14453635176317</v>
       </c>
       <c r="AE14" t="n">
-        <v>56.56401944894651</v>
+        <v>63.16935132781889</v>
       </c>
       <c r="AF14" t="n">
-        <v>-8.719232825814892</v>
+        <v>-2.013918516191104</v>
       </c>
       <c r="AG14" t="n">
-        <v>-99.02719747733543</v>
+        <v>-92.75679936933386</v>
       </c>
     </row>
     <row r="15">
@@ -2063,122 +2063,19 @@
         <v>66.67719021310181</v>
       </c>
       <c r="AC15" t="n">
-        <v>25</v>
+        <v>137</v>
       </c>
       <c r="AD15" t="n">
-        <v>72</v>
+        <v>67.88321167883211</v>
       </c>
       <c r="AE15" t="n">
-        <v>84</v>
+        <v>80.29197080291971</v>
       </c>
       <c r="AF15" t="n">
-        <v>25.52801894238358</v>
+        <v>21.41123062121569</v>
       </c>
       <c r="AG15" t="n">
-        <v>-99.60536700868192</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Paniplay Honduras</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>10991</v>
-      </c>
-      <c r="C16" t="n">
-        <v>72.30461286507143</v>
-      </c>
-      <c r="D16" t="n">
-        <v>86.31607679010099</v>
-      </c>
-      <c r="E16" t="n">
-        <v>12023</v>
-      </c>
-      <c r="F16" t="n">
-        <v>74.23272061881394</v>
-      </c>
-      <c r="G16" t="n">
-        <v>88.38060384263495</v>
-      </c>
-      <c r="H16" t="n">
-        <v>14042</v>
-      </c>
-      <c r="I16" t="n">
-        <v>76.31391539666714</v>
-      </c>
-      <c r="J16" t="n">
-        <v>88.14983620566871</v>
-      </c>
-      <c r="K16" t="n">
-        <v>13195</v>
-      </c>
-      <c r="L16" t="n">
-        <v>67.07843880257673</v>
-      </c>
-      <c r="M16" t="n">
-        <v>84.50928381962865</v>
-      </c>
-      <c r="N16" t="n">
-        <v>13769</v>
-      </c>
-      <c r="O16" t="n">
-        <v>74.71857070230227</v>
-      </c>
-      <c r="P16" t="n">
-        <v>84.62488198126226</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>16085</v>
-      </c>
-      <c r="R16" t="n">
-        <v>70.71806030463165</v>
-      </c>
-      <c r="S16" t="n">
-        <v>81.03823437985702</v>
-      </c>
-      <c r="T16" t="n">
-        <v>16006</v>
-      </c>
-      <c r="U16" t="n">
-        <v>59.19655129326502</v>
-      </c>
-      <c r="V16" t="n">
-        <v>74.15969011620642</v>
-      </c>
-      <c r="W16" t="n">
-        <v>0</v>
-      </c>
-      <c r="X16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG16" t="n">
-        <v>0</v>
+        <v>-97.83741120757695</v>
       </c>
     </row>
   </sheetData>
@@ -2550,7 +2447,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -3912,7 +3809,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3963,7 +3860,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -4380,7 +4277,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -5754,7 +5651,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5805,7 +5702,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5929,19 +5826,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>206</v>
+        <v>1620</v>
       </c>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>211</v>
       </c>
       <c r="D4" t="n">
-        <v>5.825242718446602</v>
+        <v>13.02469135802469</v>
       </c>
       <c r="E4" t="n">
-        <v>71.23416666666667</v>
+        <v>1129.528578199052</v>
       </c>
       <c r="F4" t="n">
-        <v>2068.482989690722</v>
+        <v>1033.062838892832</v>
       </c>
     </row>
     <row r="5">
@@ -5951,19 +5848,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8296</v>
+        <v>52513</v>
       </c>
       <c r="C5" t="n">
-        <v>6739</v>
+        <v>42246</v>
       </c>
       <c r="D5" t="n">
-        <v>81.23191899710704</v>
+        <v>80.44865081027555</v>
       </c>
       <c r="E5" t="n">
-        <v>3401.143295739724</v>
+        <v>3422.031019977986</v>
       </c>
       <c r="F5" t="n">
-        <v>12017.92929993577</v>
+        <v>6395.370684718028</v>
       </c>
     </row>
     <row r="6">
@@ -5973,19 +5870,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2906</v>
+        <v>17238</v>
       </c>
       <c r="C6" t="n">
-        <v>275</v>
+        <v>2003</v>
       </c>
       <c r="D6" t="n">
-        <v>9.463179628355126</v>
+        <v>11.61967745678153</v>
       </c>
       <c r="E6" t="n">
-        <v>4147.505381818181</v>
+        <v>7713.67765351972</v>
       </c>
       <c r="F6" t="n">
-        <v>5952.025583428354</v>
+        <v>2771.867249097473</v>
       </c>
     </row>
     <row r="7">
@@ -5995,19 +5892,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>487</v>
+        <v>3099</v>
       </c>
       <c r="C7" t="n">
-        <v>167</v>
+        <v>1158</v>
       </c>
       <c r="D7" t="n">
-        <v>34.29158110882957</v>
+        <v>37.36689254598258</v>
       </c>
       <c r="E7" t="n">
-        <v>217.8389820359282</v>
+        <v>1101.094170984456</v>
       </c>
       <c r="F7" t="n">
-        <v>2443.36721875</v>
+        <v>3019.909654817105</v>
       </c>
     </row>
     <row r="8"/>
@@ -7245,7 +7142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O47"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7321,19 +7218,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>315</v>
+        <v>1516</v>
       </c>
       <c r="C4" t="n">
-        <v>105</v>
+        <v>487</v>
       </c>
       <c r="D4" t="n">
-        <v>33.33333333333333</v>
+        <v>32.12401055408971</v>
       </c>
       <c r="E4" t="n">
-        <v>216</v>
+        <v>1030</v>
       </c>
       <c r="F4" t="n">
-        <v>68.57142857142857</v>
+        <v>67.94195250659631</v>
       </c>
     </row>
     <row r="5">
@@ -7343,264 +7240,285 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>31</v>
+        <v>164</v>
       </c>
       <c r="C5" t="n">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="D5" t="n">
-        <v>38.70967741935484</v>
+        <v>35.36585365853659</v>
       </c>
       <c r="E5" t="n">
-        <v>26</v>
+        <v>128</v>
       </c>
       <c r="F5" t="n">
-        <v>83.87096774193549</v>
+        <v>78.04878048780488</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Doradobet Bolivia</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>1154</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>852</v>
       </c>
       <c r="D6" t="n">
-        <v>100</v>
+        <v>73.83015597920277</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>895</v>
       </c>
       <c r="F6" t="n">
-        <v>100</v>
+        <v>77.55632582322357</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Doradobet Chile</t>
+          <t>Doradobet Bolivia</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="D7" t="n">
-        <v>56.25</v>
+        <v>95</v>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F7" t="n">
-        <v>62.5</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Doradobet Costa Rica</t>
+          <t>Doradobet Chile</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>771</v>
+        <v>145</v>
       </c>
       <c r="C8" t="n">
-        <v>412</v>
+        <v>97</v>
       </c>
       <c r="D8" t="n">
-        <v>53.43709468223087</v>
+        <v>66.89655172413794</v>
       </c>
       <c r="E8" t="n">
-        <v>453</v>
+        <v>101</v>
       </c>
       <c r="F8" t="n">
-        <v>58.75486381322958</v>
+        <v>69.6551724137931</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Doradobet Ecuador</t>
+          <t>Doradobet Costa Rica</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>740</v>
+        <v>3365</v>
       </c>
       <c r="C9" t="n">
-        <v>344</v>
+        <v>2607</v>
       </c>
       <c r="D9" t="n">
-        <v>46.48648648648649</v>
+        <v>77.47399702823181</v>
       </c>
       <c r="E9" t="n">
-        <v>469</v>
+        <v>2707</v>
       </c>
       <c r="F9" t="n">
-        <v>63.37837837837837</v>
+        <v>80.44576523031203</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Doradobet El Salvador</t>
+          <t>Doradobet Ecuador</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>641</v>
+        <v>4232</v>
       </c>
       <c r="C10" t="n">
-        <v>295</v>
+        <v>2082</v>
       </c>
       <c r="D10" t="n">
-        <v>46.02184087363494</v>
+        <v>49.19659735349716</v>
       </c>
       <c r="E10" t="n">
-        <v>346</v>
+        <v>2718</v>
       </c>
       <c r="F10" t="n">
-        <v>53.97815912636506</v>
+        <v>64.22495274102079</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Doradobet Guatemala</t>
+          <t>Doradobet El Salvador</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>28</v>
+        <v>3212</v>
       </c>
       <c r="C11" t="n">
-        <v>22</v>
+        <v>1613</v>
       </c>
       <c r="D11" t="n">
-        <v>78.57142857142857</v>
+        <v>50.21793275217933</v>
       </c>
       <c r="E11" t="n">
-        <v>25</v>
+        <v>1933</v>
       </c>
       <c r="F11" t="n">
-        <v>89.28571428571429</v>
+        <v>60.18057285180573</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Doradobet Honduras</t>
+          <t>Doradobet Guatemala</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>130</v>
+        <v>277</v>
       </c>
       <c r="C12" t="n">
-        <v>62</v>
+        <v>171</v>
       </c>
       <c r="D12" t="n">
-        <v>47.69230769230769</v>
+        <v>61.73285198555957</v>
       </c>
       <c r="E12" t="n">
-        <v>68</v>
+        <v>196</v>
       </c>
       <c r="F12" t="n">
-        <v>52.30769230769231</v>
+        <v>70.75812274368231</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Doradobet Perú</t>
+          <t>Doradobet Honduras</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2777</v>
+        <v>685</v>
       </c>
       <c r="C13" t="n">
-        <v>2088</v>
+        <v>379</v>
       </c>
       <c r="D13" t="n">
-        <v>75.18905293482176</v>
+        <v>55.32846715328466</v>
       </c>
       <c r="E13" t="n">
-        <v>2267</v>
+        <v>409</v>
       </c>
       <c r="F13" t="n">
-        <v>81.63485776017285</v>
+        <v>59.70802919708029</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ecuabet Ecuador</t>
+          <t>Doradobet Perú</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5803</v>
+        <v>15307</v>
       </c>
       <c r="C14" t="n">
-        <v>3594</v>
+        <v>11532</v>
       </c>
       <c r="D14" t="n">
-        <v>61.9334826813717</v>
+        <v>75.33808061671131</v>
       </c>
       <c r="E14" t="n">
-        <v>4499</v>
+        <v>12326</v>
       </c>
       <c r="F14" t="n">
-        <v>77.52886438049285</v>
+        <v>80.52524988567322</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GanaPlay El Salvador</t>
+          <t>Ecuabet Ecuador</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>617</v>
+        <v>39662</v>
       </c>
       <c r="C15" t="n">
-        <v>231</v>
+        <v>23600</v>
       </c>
       <c r="D15" t="n">
-        <v>37.43922204213938</v>
+        <v>59.5027986485805</v>
       </c>
       <c r="E15" t="n">
-        <v>349</v>
+        <v>30411</v>
       </c>
       <c r="F15" t="n">
-        <v>56.56401944894651</v>
+        <v>76.67540719076193</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>GanaPlay El Salvador</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4594</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D16" t="n">
+        <v>44.14453635176317</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2902</v>
+      </c>
+      <c r="F16" t="n">
+        <v>63.16935132781889</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>GanaPlay Guatemala</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>25</v>
-      </c>
-      <c r="C16" t="n">
-        <v>18</v>
-      </c>
-      <c r="D16" t="n">
-        <v>72</v>
-      </c>
-      <c r="E16" t="n">
-        <v>21</v>
-      </c>
-      <c r="F16" t="n">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="17"/>
+      <c r="B17" t="n">
+        <v>137</v>
+      </c>
+      <c r="C17" t="n">
+        <v>93</v>
+      </c>
+      <c r="D17" t="n">
+        <v>67.88321167883211</v>
+      </c>
+      <c r="E17" t="n">
+        <v>110</v>
+      </c>
+      <c r="F17" t="n">
+        <v>80.29197080291971</v>
+      </c>
+    </row>
     <row r="18"/>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7699,43 +7617,43 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>105</v>
+        <v>487</v>
       </c>
       <c r="D22" t="n">
-        <v>1.375555555555556</v>
+        <v>1.563278576317591</v>
       </c>
       <c r="E22" t="n">
-        <v>1.583333333333333</v>
+        <v>1.566666666666667</v>
       </c>
       <c r="F22" t="n">
-        <v>0.02292592592592593</v>
+        <v>0.02605464293862651</v>
       </c>
       <c r="G22" t="n">
-        <v>0.02638888888888889</v>
+        <v>0.02611111111111111</v>
       </c>
       <c r="H22" t="n">
-        <v>190.4239215686275</v>
+        <v>198.1774324324324</v>
       </c>
       <c r="I22" t="n">
-        <v>110.0666666666667</v>
+        <v>107.6166666666667</v>
       </c>
       <c r="J22" t="n">
-        <v>3.17373202614379</v>
+        <v>3.302957207207208</v>
       </c>
       <c r="K22" t="n">
-        <v>1.834444444444444</v>
+        <v>1.793611111111111</v>
       </c>
       <c r="L22" t="n">
-        <v>188.724705882353</v>
+        <v>196.173963963964</v>
       </c>
       <c r="M22" t="n">
-        <v>108.1</v>
+        <v>106</v>
       </c>
       <c r="N22" t="n">
-        <v>3.145411764705882</v>
+        <v>3.269566066066066</v>
       </c>
       <c r="O22" t="n">
-        <v>1.801666666666667</v>
+        <v>1.766666666666667</v>
       </c>
     </row>
     <row r="23">
@@ -7750,43 +7668,43 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>210</v>
+        <v>1029</v>
       </c>
       <c r="D23" t="n">
-        <v>304.4066666666667</v>
+        <v>310.9427923550372</v>
       </c>
       <c r="E23" t="n">
-        <v>165.5833333333333</v>
+        <v>138.9666666666667</v>
       </c>
       <c r="F23" t="n">
-        <v>5.073444444444443</v>
+        <v>5.182379872583954</v>
       </c>
       <c r="G23" t="n">
-        <v>2.759722222222222</v>
+        <v>2.316111111111111</v>
       </c>
       <c r="H23" t="n">
-        <v>319.8262479871176</v>
+        <v>321.9956114398422</v>
       </c>
       <c r="I23" t="n">
-        <v>189.75</v>
+        <v>146.7166666666667</v>
       </c>
       <c r="J23" t="n">
-        <v>5.33043746645196</v>
+        <v>5.366593523997371</v>
       </c>
       <c r="K23" t="n">
-        <v>3.1625</v>
+        <v>2.445277777777778</v>
       </c>
       <c r="L23" t="n">
-        <v>11.81054750402576</v>
+        <v>9.674769888231427</v>
       </c>
       <c r="M23" t="n">
-        <v>4.966666666666667</v>
+        <v>5.033333333333333</v>
       </c>
       <c r="N23" t="n">
-        <v>0.1968424584004294</v>
+        <v>0.1612461648038571</v>
       </c>
       <c r="O23" t="n">
-        <v>0.08277777777777778</v>
+        <v>0.08388888888888889</v>
       </c>
     </row>
     <row r="24">
@@ -7801,43 +7719,43 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="D24" t="n">
-        <v>1.943055555555556</v>
+        <v>2.266379310344827</v>
       </c>
       <c r="E24" t="n">
-        <v>1.891666666666667</v>
+        <v>1.583333333333333</v>
       </c>
       <c r="F24" t="n">
-        <v>0.03238425925925926</v>
+        <v>0.03777298850574712</v>
       </c>
       <c r="G24" t="n">
-        <v>0.03152777777777778</v>
+        <v>0.02638888888888889</v>
       </c>
       <c r="H24" t="n">
-        <v>112.4875</v>
+        <v>91.6982905982906</v>
       </c>
       <c r="I24" t="n">
-        <v>68.83333333333333</v>
+        <v>17.5</v>
       </c>
       <c r="J24" t="n">
-        <v>1.874791666666667</v>
+        <v>1.528304843304843</v>
       </c>
       <c r="K24" t="n">
-        <v>1.147222222222222</v>
+        <v>0.2916666666666667</v>
       </c>
       <c r="L24" t="n">
-        <v>110.6645833333333</v>
+        <v>90.06324786324788</v>
       </c>
       <c r="M24" t="n">
-        <v>66.925</v>
+        <v>15.55</v>
       </c>
       <c r="N24" t="n">
-        <v>1.844409722222222</v>
+        <v>1.501054131054131</v>
       </c>
       <c r="O24" t="n">
-        <v>1.115416666666667</v>
+        <v>0.2591666666666667</v>
       </c>
     </row>
     <row r="25">
@@ -7852,49 +7770,49 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>19</v>
+        <v>106</v>
       </c>
       <c r="D25" t="n">
-        <v>187.6754385964912</v>
+        <v>271.6676100628931</v>
       </c>
       <c r="E25" t="n">
-        <v>34.45</v>
+        <v>21.96666666666667</v>
       </c>
       <c r="F25" t="n">
-        <v>3.127923976608187</v>
+        <v>4.527793501048219</v>
       </c>
       <c r="G25" t="n">
-        <v>0.5741666666666667</v>
+        <v>0.3661111111111111</v>
       </c>
       <c r="H25" t="n">
-        <v>196.2631578947368</v>
+        <v>294.1245283018868</v>
       </c>
       <c r="I25" t="n">
-        <v>44.78333333333333</v>
+        <v>37.89166666666667</v>
       </c>
       <c r="J25" t="n">
-        <v>3.271052631578947</v>
+        <v>4.902075471698114</v>
       </c>
       <c r="K25" t="n">
-        <v>0.7463888888888889</v>
+        <v>0.6315277777777777</v>
       </c>
       <c r="L25" t="n">
-        <v>8.587719298245615</v>
+        <v>22.45691823899371</v>
       </c>
       <c r="M25" t="n">
-        <v>3.35</v>
+        <v>2.975</v>
       </c>
       <c r="N25" t="n">
-        <v>0.1431286549707602</v>
+        <v>0.3742819706498952</v>
       </c>
       <c r="O25" t="n">
-        <v>0.05583333333333333</v>
+        <v>0.04958333333333333</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Doradobet Bolivia</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7903,25 +7821,49 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>852</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>2.5981220657277</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>1.675</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>0.04330203442879499</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>0.02791666666666667</v>
+      </c>
+      <c r="H26" t="n">
+        <v>669.6372267759563</v>
+      </c>
+      <c r="I26" t="n">
+        <v>662.0999999999999</v>
+      </c>
+      <c r="J26" t="n">
+        <v>11.16062044626594</v>
+      </c>
+      <c r="K26" t="n">
+        <v>11.035</v>
+      </c>
+      <c r="L26" t="n">
+        <v>666.835154826958</v>
+      </c>
+      <c r="M26" t="n">
+        <v>660.7083333333333</v>
+      </c>
+      <c r="N26" t="n">
+        <v>11.11391924711597</v>
+      </c>
+      <c r="O26" t="n">
+        <v>11.01180555555556</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Doradobet Bolivia</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7930,13 +7872,49 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>302</v>
+      </c>
+      <c r="D27" t="n">
+        <v>334.6443156732892</v>
+      </c>
+      <c r="E27" t="n">
+        <v>183</v>
+      </c>
+      <c r="F27" t="n">
+        <v>5.577405261221486</v>
+      </c>
+      <c r="G27" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="H27" t="n">
+        <v>954.086531986532</v>
+      </c>
+      <c r="I27" t="n">
+        <v>966.1333333333333</v>
+      </c>
+      <c r="J27" t="n">
+        <v>15.90144219977553</v>
+      </c>
+      <c r="K27" t="n">
+        <v>16.10222222222222</v>
+      </c>
+      <c r="L27" t="n">
+        <v>617.5066217732884</v>
+      </c>
+      <c r="M27" t="n">
+        <v>596.4833333333333</v>
+      </c>
+      <c r="N27" t="n">
+        <v>10.29177702955481</v>
+      </c>
+      <c r="O27" t="n">
+        <v>9.941388888888889</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Doradobet Chile</t>
+          <t>Doradobet Bolivia</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7945,49 +7923,49 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="D28" t="n">
-        <v>2.077777777777778</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="E28" t="n">
-        <v>1.85</v>
+        <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>0.03462962962962963</v>
+        <v>0.007777777777777778</v>
       </c>
       <c r="G28" t="n">
-        <v>0.03083333333333333</v>
+        <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>5.95625</v>
+        <v>1748.533333333333</v>
       </c>
       <c r="I28" t="n">
-        <v>5.166666666666666</v>
+        <v>1767.775</v>
       </c>
       <c r="J28" t="n">
-        <v>0.09927083333333334</v>
+        <v>29.14222222222223</v>
       </c>
       <c r="K28" t="n">
-        <v>0.08611111111111111</v>
+        <v>29.46291666666666</v>
       </c>
       <c r="L28" t="n">
-        <v>3.61875</v>
+        <v>1747.055555555556</v>
       </c>
       <c r="M28" t="n">
-        <v>3.416666666666667</v>
+        <v>1766.066666666667</v>
       </c>
       <c r="N28" t="n">
-        <v>0.0603125</v>
+        <v>29.11759259259259</v>
       </c>
       <c r="O28" t="n">
-        <v>0.05694444444444445</v>
+        <v>29.43444444444444</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Doradobet Chile</t>
+          <t>Doradobet Bolivia</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7996,49 +7974,49 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>46.07380952380952</v>
+        <v>58.55</v>
       </c>
       <c r="E29" t="n">
-        <v>40.45</v>
+        <v>58.55</v>
       </c>
       <c r="F29" t="n">
-        <v>0.7678968253968254</v>
+        <v>0.9758333333333333</v>
       </c>
       <c r="G29" t="n">
-        <v>0.6741666666666667</v>
+        <v>0.9758333333333333</v>
       </c>
       <c r="H29" t="n">
-        <v>49.15000000000001</v>
+        <v>1803.15</v>
       </c>
       <c r="I29" t="n">
-        <v>43.21666666666667</v>
+        <v>1803.15</v>
       </c>
       <c r="J29" t="n">
-        <v>0.8191666666666667</v>
+        <v>30.0525</v>
       </c>
       <c r="K29" t="n">
-        <v>0.7202777777777778</v>
+        <v>30.0525</v>
       </c>
       <c r="L29" t="n">
-        <v>3.076190476190476</v>
+        <v>1744.6</v>
       </c>
       <c r="M29" t="n">
-        <v>2.916666666666667</v>
+        <v>1744.6</v>
       </c>
       <c r="N29" t="n">
-        <v>0.05126984126984126</v>
+        <v>29.07666666666666</v>
       </c>
       <c r="O29" t="n">
-        <v>0.04861111111111111</v>
+        <v>29.07666666666666</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Doradobet Costa Rica</t>
+          <t>Doradobet Chile</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -8047,49 +8025,49 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>412</v>
+        <v>97</v>
       </c>
       <c r="D30" t="n">
-        <v>1.783940129449838</v>
+        <v>1.386254295532646</v>
       </c>
       <c r="E30" t="n">
-        <v>1.591666666666667</v>
+        <v>1.55</v>
       </c>
       <c r="F30" t="n">
-        <v>0.02973233549083064</v>
+        <v>0.02310423825887743</v>
       </c>
       <c r="G30" t="n">
-        <v>0.02652777777777778</v>
+        <v>0.02583333333333333</v>
       </c>
       <c r="H30" t="n">
-        <v>242.7850045167118</v>
+        <v>507.0838028169014</v>
       </c>
       <c r="I30" t="n">
-        <v>109.8833333333333</v>
+        <v>402.6333333333333</v>
       </c>
       <c r="J30" t="n">
-        <v>4.046416741945198</v>
+        <v>8.451396713615022</v>
       </c>
       <c r="K30" t="n">
-        <v>1.831388888888889</v>
+        <v>6.710555555555556</v>
       </c>
       <c r="L30" t="n">
-        <v>240.8019421860886</v>
+        <v>505.1899061032864</v>
       </c>
       <c r="M30" t="n">
-        <v>107.1666666666667</v>
+        <v>401.0166666666667</v>
       </c>
       <c r="N30" t="n">
-        <v>4.013365703101476</v>
+        <v>8.419831768388107</v>
       </c>
       <c r="O30" t="n">
-        <v>1.786111111111111</v>
+        <v>6.683611111111111</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Doradobet Costa Rica</t>
+          <t>Doradobet Chile</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -8098,49 +8076,49 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>359</v>
+        <v>48</v>
       </c>
       <c r="D31" t="n">
-        <v>1505.794011142061</v>
+        <v>163.6326388888889</v>
       </c>
       <c r="E31" t="n">
-        <v>1461.716666666667</v>
+        <v>82.88333333333333</v>
       </c>
       <c r="F31" t="n">
-        <v>25.09656685236769</v>
+        <v>2.727210648148148</v>
       </c>
       <c r="G31" t="n">
-        <v>24.36194444444444</v>
+        <v>1.381388888888889</v>
       </c>
       <c r="H31" t="n">
-        <v>1675.198611111111</v>
+        <v>536.78125</v>
       </c>
       <c r="I31" t="n">
-        <v>1635.558333333333</v>
+        <v>457</v>
       </c>
       <c r="J31" t="n">
-        <v>27.91997685185185</v>
+        <v>8.946354166666666</v>
       </c>
       <c r="K31" t="n">
-        <v>27.25930555555556</v>
+        <v>7.616666666666666</v>
       </c>
       <c r="L31" t="n">
-        <v>161.9007662835249</v>
+        <v>373.1486111111111</v>
       </c>
       <c r="M31" t="n">
-        <v>161.9</v>
+        <v>136.2333333333333</v>
       </c>
       <c r="N31" t="n">
-        <v>2.698346104725415</v>
+        <v>6.219143518518519</v>
       </c>
       <c r="O31" t="n">
-        <v>2.698333333333333</v>
+        <v>2.270555555555556</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Doradobet Ecuador</t>
+          <t>Doradobet Costa Rica</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -8149,49 +8127,49 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>344</v>
+        <v>2607</v>
       </c>
       <c r="D32" t="n">
-        <v>1.460949612403101</v>
+        <v>3.30393811533052</v>
       </c>
       <c r="E32" t="n">
-        <v>1.566666666666667</v>
+        <v>1.616666666666667</v>
       </c>
       <c r="F32" t="n">
-        <v>0.02434916020671835</v>
+        <v>0.05506563525550867</v>
       </c>
       <c r="G32" t="n">
-        <v>0.02611111111111111</v>
+        <v>0.02694444444444444</v>
       </c>
       <c r="H32" t="n">
-        <v>160.9389855072464</v>
+        <v>260.0381575123511</v>
       </c>
       <c r="I32" t="n">
-        <v>106.0583333333333</v>
+        <v>100.6833333333333</v>
       </c>
       <c r="J32" t="n">
-        <v>2.682316425120773</v>
+        <v>4.333969291872517</v>
       </c>
       <c r="K32" t="n">
-        <v>1.767638888888889</v>
+        <v>1.678055555555555</v>
       </c>
       <c r="L32" t="n">
-        <v>159.3046376811594</v>
+        <v>256.3003414705028</v>
       </c>
       <c r="M32" t="n">
-        <v>104.5166666666667</v>
+        <v>89.52500000000001</v>
       </c>
       <c r="N32" t="n">
-        <v>2.655077294685991</v>
+        <v>4.271672357841713</v>
       </c>
       <c r="O32" t="n">
-        <v>1.741944444444445</v>
+        <v>1.492083333333333</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Doradobet Ecuador</t>
+          <t>Doradobet Costa Rica</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -8200,49 +8178,49 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>396</v>
+        <v>758</v>
       </c>
       <c r="D33" t="n">
-        <v>208.6752104377104</v>
+        <v>1397.248153034301</v>
       </c>
       <c r="E33" t="n">
-        <v>66.59999999999999</v>
+        <v>1288.391666666667</v>
       </c>
       <c r="F33" t="n">
-        <v>3.477920173961841</v>
+        <v>23.28746921723835</v>
       </c>
       <c r="G33" t="n">
-        <v>1.11</v>
+        <v>21.47319444444445</v>
       </c>
       <c r="H33" t="n">
-        <v>323.4670694864049</v>
+        <v>1572.775191700496</v>
       </c>
       <c r="I33" t="n">
-        <v>195.9166666666667</v>
+        <v>1480.016666666667</v>
       </c>
       <c r="J33" t="n">
-        <v>5.391117824773414</v>
+        <v>26.21291986167493</v>
       </c>
       <c r="K33" t="n">
-        <v>3.265277777777778</v>
+        <v>24.66694444444444</v>
       </c>
       <c r="L33" t="n">
-        <v>94.86701913393756</v>
+        <v>169.6258457374831</v>
       </c>
       <c r="M33" t="n">
-        <v>56.68333333333333</v>
+        <v>161.9</v>
       </c>
       <c r="N33" t="n">
-        <v>1.581116985565626</v>
+        <v>2.827097428958052</v>
       </c>
       <c r="O33" t="n">
-        <v>0.9447222222222221</v>
+        <v>2.698333333333333</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Doradobet El Salvador</t>
+          <t>Doradobet Ecuador</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -8251,49 +8229,49 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>295</v>
+        <v>2082</v>
       </c>
       <c r="D34" t="n">
-        <v>505.4411864406779</v>
+        <v>65.49751841178355</v>
       </c>
       <c r="E34" t="n">
-        <v>558.5666666666667</v>
+        <v>1.683333333333333</v>
       </c>
       <c r="F34" t="n">
-        <v>8.424019774011301</v>
+        <v>1.091625306863059</v>
       </c>
       <c r="G34" t="n">
-        <v>9.309444444444445</v>
+        <v>0.02805555555555556</v>
       </c>
       <c r="H34" t="n">
-        <v>932.9759541984733</v>
+        <v>256.7667318557149</v>
       </c>
       <c r="I34" t="n">
-        <v>1005.816666666667</v>
+        <v>113.5083333333333</v>
       </c>
       <c r="J34" t="n">
-        <v>15.54959923664122</v>
+        <v>4.279445530928582</v>
       </c>
       <c r="K34" t="n">
-        <v>16.76361111111111</v>
+        <v>1.891805555555556</v>
       </c>
       <c r="L34" t="n">
-        <v>407.4479007633588</v>
+        <v>169.191416775315</v>
       </c>
       <c r="M34" t="n">
-        <v>430.4666666666666</v>
+        <v>68.64166666666667</v>
       </c>
       <c r="N34" t="n">
-        <v>6.790798346055979</v>
+        <v>2.819856946255252</v>
       </c>
       <c r="O34" t="n">
-        <v>7.174444444444444</v>
+        <v>1.144027777777778</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Doradobet El Salvador</t>
+          <t>Doradobet Ecuador</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -8302,49 +8280,49 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>346</v>
+        <v>2150</v>
       </c>
       <c r="D35" t="n">
-        <v>900.4449903660886</v>
+        <v>197.6119689922481</v>
       </c>
       <c r="E35" t="n">
-        <v>770.8583333333333</v>
+        <v>63.30833333333334</v>
       </c>
       <c r="F35" t="n">
-        <v>15.00741650610148</v>
+        <v>3.293532816537468</v>
       </c>
       <c r="G35" t="n">
-        <v>12.84763888888889</v>
+        <v>1.055138888888889</v>
       </c>
       <c r="H35" t="n">
-        <v>1337.81298026999</v>
+        <v>347.9481237415339</v>
       </c>
       <c r="I35" t="n">
-        <v>1201.866666666667</v>
+        <v>187</v>
       </c>
       <c r="J35" t="n">
-        <v>22.29688300449983</v>
+        <v>5.799135395692233</v>
       </c>
       <c r="K35" t="n">
-        <v>20.03111111111111</v>
+        <v>3.116666666666667</v>
       </c>
       <c r="L35" t="n">
-        <v>444.547507788162</v>
+        <v>132.2054182683507</v>
       </c>
       <c r="M35" t="n">
-        <v>430.8</v>
+        <v>53.91666666666666</v>
       </c>
       <c r="N35" t="n">
-        <v>7.409125129802699</v>
+        <v>2.203423637805845</v>
       </c>
       <c r="O35" t="n">
-        <v>7.180000000000001</v>
+        <v>0.898611111111111</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Doradobet Guatemala</t>
+          <t>Doradobet El Salvador</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -8353,49 +8331,49 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>22</v>
+        <v>1613</v>
       </c>
       <c r="D36" t="n">
-        <v>1.197727272727273</v>
+        <v>1420.111396982848</v>
       </c>
       <c r="E36" t="n">
-        <v>1.308333333333333</v>
+        <v>883.15</v>
       </c>
       <c r="F36" t="n">
-        <v>0.01996212121212121</v>
+        <v>23.66852328304746</v>
       </c>
       <c r="G36" t="n">
-        <v>0.02180555555555556</v>
+        <v>14.71916666666667</v>
       </c>
       <c r="H36" t="n">
-        <v>283</v>
+        <v>1619.586247198207</v>
       </c>
       <c r="I36" t="n">
-        <v>129.6916666666667</v>
+        <v>1143.85</v>
       </c>
       <c r="J36" t="n">
-        <v>4.716666666666667</v>
+        <v>26.99310411997011</v>
       </c>
       <c r="K36" t="n">
-        <v>2.161527777777778</v>
+        <v>19.06416666666667</v>
       </c>
       <c r="L36" t="n">
-        <v>281.3749999999999</v>
+        <v>351.7719660582773</v>
       </c>
       <c r="M36" t="n">
-        <v>127.9583333333333</v>
+        <v>397.0333333333334</v>
       </c>
       <c r="N36" t="n">
-        <v>4.689583333333333</v>
+        <v>5.862866100971289</v>
       </c>
       <c r="O36" t="n">
-        <v>2.132638888888889</v>
+        <v>6.617222222222223</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Doradobet Guatemala</t>
+          <t>Doradobet El Salvador</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -8404,49 +8382,49 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>6</v>
+        <v>1599</v>
       </c>
       <c r="D37" t="n">
-        <v>349.6166666666666</v>
+        <v>1569.035490931832</v>
       </c>
       <c r="E37" t="n">
-        <v>43.8</v>
+        <v>1046.816666666667</v>
       </c>
       <c r="F37" t="n">
-        <v>5.826944444444444</v>
+        <v>26.15059151553054</v>
       </c>
       <c r="G37" t="n">
-        <v>0.73</v>
+        <v>17.44694444444444</v>
       </c>
       <c r="H37" t="n">
-        <v>18.1</v>
+        <v>1686.301011122345</v>
       </c>
       <c r="I37" t="n">
-        <v>18.1</v>
+        <v>1231.733333333333</v>
       </c>
       <c r="J37" t="n">
-        <v>0.3016666666666667</v>
+        <v>28.1050168520391</v>
       </c>
       <c r="K37" t="n">
-        <v>0.3016666666666667</v>
+        <v>20.52888888888889</v>
       </c>
       <c r="L37" t="n">
-        <v>0.6333333333333333</v>
+        <v>364.367778901247</v>
       </c>
       <c r="M37" t="n">
-        <v>0.6333333333333333</v>
+        <v>398.0833333333333</v>
       </c>
       <c r="N37" t="n">
-        <v>0.01055555555555555</v>
+        <v>6.072796315020785</v>
       </c>
       <c r="O37" t="n">
-        <v>0.01055555555555555</v>
+        <v>6.634722222222222</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Doradobet Honduras</t>
+          <t>Doradobet Guatemala</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -8455,49 +8433,49 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>62</v>
+        <v>171</v>
       </c>
       <c r="D38" t="n">
-        <v>1.677150537634409</v>
+        <v>1.983040935672515</v>
       </c>
       <c r="E38" t="n">
-        <v>1.491666666666667</v>
+        <v>1.566666666666667</v>
       </c>
       <c r="F38" t="n">
-        <v>0.02795250896057347</v>
+        <v>0.03305068226120858</v>
       </c>
       <c r="G38" t="n">
-        <v>0.02486111111111111</v>
+        <v>0.02611111111111111</v>
       </c>
       <c r="H38" t="n">
-        <v>145.1900793650794</v>
+        <v>1114.46179245283</v>
       </c>
       <c r="I38" t="n">
-        <v>87.68333333333334</v>
+        <v>1338.55</v>
       </c>
       <c r="J38" t="n">
-        <v>2.419834656084656</v>
+        <v>18.57436320754717</v>
       </c>
       <c r="K38" t="n">
-        <v>1.461388888888889</v>
+        <v>22.30916666666667</v>
       </c>
       <c r="L38" t="n">
-        <v>143.0317460317461</v>
+        <v>1112.339622641509</v>
       </c>
       <c r="M38" t="n">
-        <v>79.16666666666666</v>
+        <v>1337.1</v>
       </c>
       <c r="N38" t="n">
-        <v>2.383862433862434</v>
+        <v>18.53899371069182</v>
       </c>
       <c r="O38" t="n">
-        <v>1.319444444444444</v>
+        <v>22.285</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Doradobet Honduras</t>
+          <t>Doradobet Guatemala</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -8506,49 +8484,49 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>68</v>
+        <v>106</v>
       </c>
       <c r="D39" t="n">
-        <v>178.2166666666667</v>
+        <v>2258.144182389938</v>
       </c>
       <c r="E39" t="n">
-        <v>85.91666666666666</v>
+        <v>2558.775</v>
       </c>
       <c r="F39" t="n">
-        <v>2.970277777777777</v>
+        <v>37.63573637316562</v>
       </c>
       <c r="G39" t="n">
-        <v>1.431944444444444</v>
+        <v>42.64624999999999</v>
       </c>
       <c r="H39" t="n">
-        <v>239.280376344086</v>
+        <v>2983.063257575758</v>
       </c>
       <c r="I39" t="n">
-        <v>146.7583333333333</v>
+        <v>3066.775</v>
       </c>
       <c r="J39" t="n">
-        <v>3.988006272401434</v>
+        <v>49.71772095959596</v>
       </c>
       <c r="K39" t="n">
-        <v>2.445972222222222</v>
+        <v>51.11291666666667</v>
       </c>
       <c r="L39" t="n">
-        <v>62.68655913978495</v>
+        <v>312.7573863636364</v>
       </c>
       <c r="M39" t="n">
-        <v>48.83333333333334</v>
+        <v>371.9666666666666</v>
       </c>
       <c r="N39" t="n">
-        <v>1.044775985663082</v>
+        <v>5.212623106060606</v>
       </c>
       <c r="O39" t="n">
-        <v>0.8138888888888889</v>
+        <v>6.199444444444444</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Doradobet Perú</t>
+          <t>Doradobet Honduras</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -8557,49 +8535,49 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2088</v>
+        <v>379</v>
       </c>
       <c r="D40" t="n">
-        <v>25.21633141762452</v>
+        <v>1.428320140721196</v>
       </c>
       <c r="E40" t="n">
-        <v>1.716666666666667</v>
+        <v>1.55</v>
       </c>
       <c r="F40" t="n">
-        <v>0.4202721902937421</v>
+        <v>0.0238053356786866</v>
       </c>
       <c r="G40" t="n">
-        <v>0.02861111111111111</v>
+        <v>0.02583333333333333</v>
       </c>
       <c r="H40" t="n">
-        <v>37.67813919867823</v>
+        <v>362.3328431372549</v>
       </c>
       <c r="I40" t="n">
-        <v>2.05</v>
+        <v>225.5166666666667</v>
       </c>
       <c r="J40" t="n">
-        <v>0.6279689866446372</v>
+        <v>6.038880718954249</v>
       </c>
       <c r="K40" t="n">
-        <v>0.03416666666666666</v>
+        <v>3.758611111111111</v>
       </c>
       <c r="L40" t="n">
-        <v>6.503159851301115</v>
+        <v>360.4293417366947</v>
       </c>
       <c r="M40" t="n">
-        <v>0.2333333333333333</v>
+        <v>224.025</v>
       </c>
       <c r="N40" t="n">
-        <v>0.1083859975216853</v>
+        <v>6.007155695611578</v>
       </c>
       <c r="O40" t="n">
-        <v>0.003888888888888889</v>
+        <v>3.73375</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Doradobet Perú</t>
+          <t>Doradobet Honduras</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8608,49 +8586,49 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>689</v>
+        <v>306</v>
       </c>
       <c r="D41" t="n">
-        <v>479.9092162554426</v>
+        <v>138.6327886710239</v>
       </c>
       <c r="E41" t="n">
-        <v>279.2666666666667</v>
+        <v>72.88333333333333</v>
       </c>
       <c r="F41" t="n">
-        <v>7.998486937590711</v>
+        <v>2.3105464778504</v>
       </c>
       <c r="G41" t="n">
-        <v>4.654444444444445</v>
+        <v>1.214722222222222</v>
       </c>
       <c r="H41" t="n">
-        <v>487.0816370490037</v>
+        <v>458.5338422391857</v>
       </c>
       <c r="I41" t="n">
-        <v>289.5</v>
+        <v>261.9833333333333</v>
       </c>
       <c r="J41" t="n">
-        <v>8.118027284150063</v>
+        <v>7.642230703986429</v>
       </c>
       <c r="K41" t="n">
-        <v>4.825</v>
+        <v>4.366388888888888</v>
       </c>
       <c r="L41" t="n">
-        <v>17.02501346257404</v>
+        <v>322.0881043256998</v>
       </c>
       <c r="M41" t="n">
-        <v>11.81666666666667</v>
+        <v>172.7</v>
       </c>
       <c r="N41" t="n">
-        <v>0.283750224376234</v>
+        <v>5.368135072094995</v>
       </c>
       <c r="O41" t="n">
-        <v>0.1969444444444444</v>
+        <v>2.878333333333333</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ecuabet Ecuador</t>
+          <t>Doradobet Perú</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8659,49 +8637,49 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3594</v>
+        <v>11532</v>
       </c>
       <c r="D42" t="n">
-        <v>2.267427193470599</v>
+        <v>51.89016938374379</v>
       </c>
       <c r="E42" t="n">
         <v>1.716666666666667</v>
       </c>
       <c r="F42" t="n">
-        <v>0.03779045322450999</v>
+        <v>0.8648361563957297</v>
       </c>
       <c r="G42" t="n">
         <v>0.02861111111111111</v>
       </c>
       <c r="H42" t="n">
-        <v>147.372594997595</v>
+        <v>76.40836901810533</v>
       </c>
       <c r="I42" t="n">
-        <v>100.2333333333333</v>
+        <v>2.066666666666667</v>
       </c>
       <c r="J42" t="n">
-        <v>2.456209916626583</v>
+        <v>1.273472816968422</v>
       </c>
       <c r="K42" t="n">
-        <v>1.670555555555556</v>
+        <v>0.03444444444444445</v>
       </c>
       <c r="L42" t="n">
-        <v>145.0155483405483</v>
+        <v>10.39482946435279</v>
       </c>
       <c r="M42" t="n">
-        <v>97.79166666666666</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="N42" t="n">
-        <v>2.416925805675806</v>
+        <v>0.1732471577392132</v>
       </c>
       <c r="O42" t="n">
-        <v>1.629861111111111</v>
+        <v>0.003888888888888889</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Ecuabet Ecuador</t>
+          <t>Doradobet Perú</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -8710,49 +8688,49 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2209</v>
+        <v>3775</v>
       </c>
       <c r="D43" t="n">
-        <v>184.1245133544591</v>
+        <v>854.7641368653422</v>
       </c>
       <c r="E43" t="n">
-        <v>101.7</v>
+        <v>759.3166666666667</v>
       </c>
       <c r="F43" t="n">
-        <v>3.068741889240984</v>
+        <v>14.2460689477557</v>
       </c>
       <c r="G43" t="n">
-        <v>1.695</v>
+        <v>12.65527777777778</v>
       </c>
       <c r="H43" t="n">
-        <v>300.9872888888889</v>
+        <v>833.0363063063062</v>
       </c>
       <c r="I43" t="n">
-        <v>184.65</v>
+        <v>752.525</v>
       </c>
       <c r="J43" t="n">
-        <v>5.016454814814815</v>
+        <v>13.88393843843844</v>
       </c>
       <c r="K43" t="n">
-        <v>3.0775</v>
+        <v>12.54208333333333</v>
       </c>
       <c r="L43" t="n">
-        <v>108.52304</v>
+        <v>16.59462962962963</v>
       </c>
       <c r="M43" t="n">
-        <v>68.81666666666666</v>
+        <v>10.93333333333333</v>
       </c>
       <c r="N43" t="n">
-        <v>1.808717333333333</v>
+        <v>0.2765771604938272</v>
       </c>
       <c r="O43" t="n">
-        <v>1.146944444444444</v>
+        <v>0.1822222222222222</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>GanaPlay El Salvador</t>
+          <t>Ecuabet Ecuador</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8761,49 +8739,49 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>231</v>
+        <v>23600</v>
       </c>
       <c r="D44" t="n">
-        <v>1.221356421356421</v>
+        <v>5.145854519774011</v>
       </c>
       <c r="E44" t="n">
-        <v>1.433333333333333</v>
+        <v>1.733333333333333</v>
       </c>
       <c r="F44" t="n">
-        <v>0.02035594035594035</v>
+        <v>0.08576424199623352</v>
       </c>
       <c r="G44" t="n">
-        <v>0.02388888888888889</v>
+        <v>0.02888888888888889</v>
       </c>
       <c r="H44" t="n">
-        <v>674.2703703703703</v>
+        <v>270.0224769181789</v>
       </c>
       <c r="I44" t="n">
-        <v>740.5083333333333</v>
+        <v>119.7</v>
       </c>
       <c r="J44" t="n">
-        <v>11.23783950617284</v>
+        <v>4.500374615302982</v>
       </c>
       <c r="K44" t="n">
-        <v>12.34180555555556</v>
+        <v>1.995</v>
       </c>
       <c r="L44" t="n">
-        <v>672.7029629629629</v>
+        <v>265.3009727970569</v>
       </c>
       <c r="M44" t="n">
-        <v>739</v>
+        <v>113.1</v>
       </c>
       <c r="N44" t="n">
-        <v>11.21171604938272</v>
+        <v>4.421682879950947</v>
       </c>
       <c r="O44" t="n">
-        <v>12.31666666666667</v>
+        <v>1.885</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>GanaPlay El Salvador</t>
+          <t>Ecuabet Ecuador</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8812,49 +8790,49 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>386</v>
+        <v>16062</v>
       </c>
       <c r="D45" t="n">
-        <v>428.3034974093264</v>
+        <v>141.0731083717262</v>
       </c>
       <c r="E45" t="n">
-        <v>493.7666666666667</v>
+        <v>85.44166666666666</v>
       </c>
       <c r="F45" t="n">
-        <v>7.138391623488774</v>
+        <v>2.351218472862104</v>
       </c>
       <c r="G45" t="n">
-        <v>8.229444444444443</v>
+        <v>1.424027777777778</v>
       </c>
       <c r="H45" t="n">
-        <v>775.8131140350876</v>
+        <v>366.8541334100333</v>
       </c>
       <c r="I45" t="n">
-        <v>855.6166666666667</v>
+        <v>170.85</v>
       </c>
       <c r="J45" t="n">
-        <v>12.93021856725146</v>
+        <v>6.114235556833888</v>
       </c>
       <c r="K45" t="n">
-        <v>14.26027777777778</v>
+        <v>2.8475</v>
       </c>
       <c r="L45" t="n">
-        <v>340.8565350877193</v>
+        <v>221.0794024591932</v>
       </c>
       <c r="M45" t="n">
-        <v>375.825</v>
+        <v>73.81666666666666</v>
       </c>
       <c r="N45" t="n">
-        <v>5.680942251461988</v>
+        <v>3.68465670765322</v>
       </c>
       <c r="O45" t="n">
-        <v>6.26375</v>
+        <v>1.230277777777778</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>GanaPlay Guatemala</t>
+          <t>GanaPlay El Salvador</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8863,94 +8841,196 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>18</v>
+        <v>2028</v>
       </c>
       <c r="D46" t="n">
-        <v>0.5527777777777777</v>
+        <v>1.541962524654833</v>
       </c>
       <c r="E46" t="n">
-        <v>0</v>
+        <v>1.583333333333333</v>
       </c>
       <c r="F46" t="n">
-        <v>0.009212962962962963</v>
+        <v>0.02569937541091387</v>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>0.02638888888888889</v>
       </c>
       <c r="H46" t="n">
-        <v>184.2966666666667</v>
+        <v>845.6316252587992</v>
       </c>
       <c r="I46" t="n">
-        <v>49.38333333333333</v>
+        <v>917.475</v>
       </c>
       <c r="J46" t="n">
-        <v>3.071611111111111</v>
+        <v>14.09386042097998</v>
       </c>
       <c r="K46" t="n">
-        <v>0.8230555555555555</v>
+        <v>15.29125</v>
       </c>
       <c r="L46" t="n">
-        <v>182.7</v>
+        <v>843.7354554865425</v>
       </c>
       <c r="M46" t="n">
-        <v>47.81666666666667</v>
+        <v>915.525</v>
       </c>
       <c r="N46" t="n">
-        <v>3.045</v>
+        <v>14.06225759144237</v>
       </c>
       <c r="O46" t="n">
-        <v>0.7969444444444445</v>
+        <v>15.25875</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>GanaPlay El Salvador</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2566</v>
+      </c>
+      <c r="D47" t="n">
+        <v>351.688847752663</v>
+      </c>
+      <c r="E47" t="n">
+        <v>387.55</v>
+      </c>
+      <c r="F47" t="n">
+        <v>5.861480795877717</v>
+      </c>
+      <c r="G47" t="n">
+        <v>6.459166666666667</v>
+      </c>
+      <c r="H47" t="n">
+        <v>1030.058451656525</v>
+      </c>
+      <c r="I47" t="n">
+        <v>1103.266666666667</v>
+      </c>
+      <c r="J47" t="n">
+        <v>17.16764086094208</v>
+      </c>
+      <c r="K47" t="n">
+        <v>18.38777777777778</v>
+      </c>
+      <c r="L47" t="n">
+        <v>674.2289249492901</v>
+      </c>
+      <c r="M47" t="n">
+        <v>468.3666666666667</v>
+      </c>
+      <c r="N47" t="n">
+        <v>11.23714874915483</v>
+      </c>
+      <c r="O47" t="n">
+        <v>7.806111111111111</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>GanaPlay Guatemala</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Automatico</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>93</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.4659498207885304</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.007765830346475508</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>334.776923076923</v>
+      </c>
+      <c r="I48" t="n">
+        <v>135.4166666666667</v>
+      </c>
+      <c r="J48" t="n">
+        <v>5.579615384615384</v>
+      </c>
+      <c r="K48" t="n">
+        <v>2.256944444444444</v>
+      </c>
+      <c r="L48" t="n">
+        <v>332.9871794871796</v>
+      </c>
+      <c r="M48" t="n">
+        <v>133.85</v>
+      </c>
+      <c r="N48" t="n">
+        <v>5.549786324786324</v>
+      </c>
+      <c r="O48" t="n">
+        <v>2.230833333333333</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>GanaPlay Guatemala</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
         <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="C47" t="n">
-        <v>7</v>
-      </c>
-      <c r="D47" t="n">
-        <v>289.5380952380953</v>
-      </c>
-      <c r="E47" t="n">
-        <v>385.8333333333333</v>
-      </c>
-      <c r="F47" t="n">
-        <v>4.82563492063492</v>
-      </c>
-      <c r="G47" t="n">
-        <v>6.430555555555555</v>
-      </c>
-      <c r="H47" t="n">
-        <v>465.9555555555556</v>
-      </c>
-      <c r="I47" t="n">
-        <v>372.5833333333334</v>
-      </c>
-      <c r="J47" t="n">
-        <v>7.765925925925927</v>
-      </c>
-      <c r="K47" t="n">
-        <v>6.209722222222222</v>
-      </c>
-      <c r="L47" t="n">
-        <v>231.6555555555556</v>
-      </c>
-      <c r="M47" t="n">
-        <v>155.3666666666667</v>
-      </c>
-      <c r="N47" t="n">
-        <v>3.860925925925926</v>
-      </c>
-      <c r="O47" t="n">
-        <v>2.589444444444444</v>
+      <c r="C49" t="n">
+        <v>44</v>
+      </c>
+      <c r="D49" t="n">
+        <v>185.917803030303</v>
+      </c>
+      <c r="E49" t="n">
+        <v>44.49166666666666</v>
+      </c>
+      <c r="F49" t="n">
+        <v>3.09863005050505</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.7415277777777778</v>
+      </c>
+      <c r="H49" t="n">
+        <v>272.4794444444444</v>
+      </c>
+      <c r="I49" t="n">
+        <v>62.99166666666667</v>
+      </c>
+      <c r="J49" t="n">
+        <v>4.541324074074073</v>
+      </c>
+      <c r="K49" t="n">
+        <v>1.049861111111111</v>
+      </c>
+      <c r="L49" t="n">
+        <v>161.6938888888889</v>
+      </c>
+      <c r="M49" t="n">
+        <v>14.525</v>
+      </c>
+      <c r="N49" t="n">
+        <v>2.694898148148148</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0.2420833333333333</v>
       </c>
     </row>
   </sheetData>
@@ -13090,7 +13170,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -14500,7 +14580,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -14551,7 +14631,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -14968,7 +15048,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -16378,7 +16458,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -16429,7 +16509,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -16846,7 +16926,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -18232,7 +18312,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -18283,7 +18363,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -18700,7 +18780,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -20074,7 +20154,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -20125,7 +20205,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -20542,7 +20622,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -21904,7 +21984,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -21955,7 +22035,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>Catraplay Honduras</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">

</xml_diff>